<commit_message>
Omit empty category sheets from the Excel client package
Leftover $0 catalog rows and untitled labor lanes no longer create blank
Crane Rental, OM Crane Subcontractor, or other optional tabs. Look samples
regenerated from the live vault payloads with the same real totals.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -892,7 +892,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.72429653935</v>
+        <v>46269.72952784722</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1165,7 +1165,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.724296458335</v>
+        <v>46269.72952774305</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -7053,7 +7053,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.72429648148</v>
+        <v>46269.72952778936</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -8753,7 +8753,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.724296493056</v>
+        <v>46269.72952778936</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -10453,7 +10453,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.724296493056</v>
+        <v>46269.72952778936</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -12077,7 +12077,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.7242965162</v>
+        <v>46269.729527812495</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -12267,7 +12267,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.72429652778</v>
+        <v>46269.72952783565</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -12377,7 +12377,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.72429652778</v>
+        <v>46269.72952783565</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -12521,7 +12521,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.72429637732</v>
+        <v>46269.729527662035</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Use COMP 6.5% commercial markup for P66 Excel and desk
P66 Summary, Subs, and third-party Total $ now use the RRFF 6.5% fee
instead of the old workbook 6% formula. B-2 exhibit Cost+6% rows stay.
Yates commercial fee stays 10%. Look samples regenerated.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -924,7 +924,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605528935</v>
+        <v>46269.749217847224</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1197,7 +1197,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605519676</v>
+        <v>46269.74921775463</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -7149,7 +7149,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605524306</v>
+        <v>46269.74921778935</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -8865,7 +8865,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605524306</v>
+        <v>46269.749217812496</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -10581,7 +10581,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.746055254625</v>
+        <v>46269.749217812496</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -12221,7 +12221,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605526621</v>
+        <v>46269.74921782408</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -12411,7 +12411,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605527778</v>
+        <v>46269.749217847224</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -12521,7 +12521,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.74605527778</v>
+        <v>46269.749217847224</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -12665,7 +12665,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.746055104166</v>
+        <v>46269.74921767361</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Refresh Look samples after COMP 6.5% desk card lock
Aromatics and CAT 2 still export at commercialMarkupRate 0.065. Money
unchanged; workbook timestamps refreshed from the live vault payloads.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -1225,7 +1225,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.75490638889</v>
+        <v>46269.756752256944</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1512,7 +1512,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.75490629629</v>
+        <v>46269.75675216435</v>
       </c>
       <c r="C5" s="20"/>
     </row>
@@ -8360,7 +8360,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.754906331014</v>
+        <v>46269.75675219907</v>
       </c>
       <c r="C5" s="20"/>
     </row>
@@ -10270,7 +10270,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.7549063426</v>
+        <v>46269.75675221065</v>
       </c>
       <c r="C5" s="20"/>
     </row>
@@ -12180,7 +12180,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.7549063426</v>
+        <v>46269.75675221065</v>
       </c>
       <c r="C5" s="20"/>
     </row>
@@ -14012,7 +14012,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.75490635417</v>
+        <v>46269.75675223379</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -14202,7 +14202,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.75490637732</v>
+        <v>46269.756752245376</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -14311,7 +14311,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.75490637732</v>
+        <v>46269.756752256944</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -14455,7 +14455,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="6">
-        <v>46269.7549062037</v>
+        <v>46269.75675208333</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Lock Excel ESTIMATE TOTAL to the desk rail and cache it
Robert’s Aromatics screenshot ($25,250,782.45) was weekday-clock labor.
The $73,889.52 gap is Staff+Foremen weekly-40 OT, not missing extras.
Summary now shares deskPackageBreakdown with the Estimate Total rail,
writes cached B21 so Excel opens on that number, and refuses a mismatch.
Compact header stays. Regenerated Look samples.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -1316,9 +1316,11 @@
       </c>
       <c r="B7" s="6">
         <f>Staff!K70</f>
+        <v>245898.48</v>
       </c>
       <c r="C7" s="7">
         <f>Staff!B70</f>
+        <v>2048</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1327,9 +1329,11 @@
       </c>
       <c r="B8" s="6">
         <f>Foremen!K22</f>
+        <v>121667.84</v>
       </c>
       <c r="C8" s="7">
         <f>Foremen!B22</f>
+        <v>976</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1338,9 +1342,11 @@
       </c>
       <c r="B9" s="6">
         <f>Direct!K22</f>
+        <v>806255.52</v>
       </c>
       <c r="C9" s="7">
         <f>Direct!B22</f>
+        <v>6608</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1349,9 +1355,11 @@
       </c>
       <c r="B10" s="6">
         <f>Support!K22</f>
+        <v>58500.31999999999</v>
       </c>
       <c r="C10" s="7">
         <f>Support!B22</f>
+        <v>448</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1360,9 +1368,11 @@
       </c>
       <c r="B11" s="9">
         <f>SUM(B7,B8,B9,B10)</f>
+        <v>1232322.1600000001</v>
       </c>
       <c r="C11" s="10">
         <f>SUM(C7,C8,C9,C10)</f>
+        <v>10080</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1371,6 +1381,7 @@
       </c>
       <c r="B12" s="6">
         <f>SUM(Staff!D70,Foremen!D22,Direct!D22,Support!D22)</f>
+        <v>71440</v>
       </c>
       <c r="C12" s="11"/>
     </row>
@@ -1381,6 +1392,7 @@
       <c r="B13" s="11"/>
       <c r="C13" s="13">
         <f>SUM(C7,C8,C9,C10)</f>
+        <v>10080</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1389,6 +1401,7 @@
       </c>
       <c r="B14" s="6">
         <f>'Staff Travel Cost'!E8</f>
+        <v>6840</v>
       </c>
       <c r="C14" s="11"/>
     </row>
@@ -1398,6 +1411,7 @@
       </c>
       <c r="B15" s="6">
         <f>'Misc Costs'!E10</f>
+        <v>10700</v>
       </c>
       <c r="C15" s="11"/>
     </row>
@@ -1407,6 +1421,7 @@
       </c>
       <c r="B16" s="6">
         <f>COE!G11</f>
+        <v>113368</v>
       </c>
       <c r="C16" s="11"/>
     </row>
@@ -1430,9 +1445,11 @@
       </c>
       <c r="B19" s="16">
         <f>SUM(B11,B12,B14,B15,B16,B17)</f>
+        <v>1435365.6600000001</v>
       </c>
       <c r="C19" s="13">
         <f>SUM(C7,C8,C9,C10)</f>
+        <v>10080</v>
       </c>
     </row>
   </sheetData>
@@ -1590,96 +1607,127 @@
       </c>
       <c r="M6" s="21">
         <f>L6+1</f>
+        <v>46287</v>
       </c>
       <c r="N6" s="21">
         <f>M6+1</f>
+        <v>46288</v>
       </c>
       <c r="O6" s="21">
         <f>N6+1</f>
+        <v>46289</v>
       </c>
       <c r="P6" s="21">
         <f>O6+1</f>
+        <v>46290</v>
       </c>
       <c r="Q6" s="22">
         <f>P6+1</f>
+        <v>46291</v>
       </c>
       <c r="R6" s="22">
         <f>Q6+1</f>
+        <v>46292</v>
       </c>
       <c r="S6" s="21">
         <f>R6+1</f>
+        <v>46293</v>
       </c>
       <c r="T6" s="21">
         <f>S6+1</f>
+        <v>46294</v>
       </c>
       <c r="U6" s="21">
         <f>T6+1</f>
+        <v>46295</v>
       </c>
       <c r="V6" s="21">
         <f>U6+1</f>
+        <v>46296</v>
       </c>
       <c r="W6" s="21">
         <f>V6+1</f>
+        <v>46297</v>
       </c>
       <c r="X6" s="22">
         <f>W6+1</f>
+        <v>46298</v>
       </c>
       <c r="Y6" s="22">
         <f>X6+1</f>
+        <v>46299</v>
       </c>
       <c r="Z6" s="21">
         <f>Y6+1</f>
+        <v>46300</v>
       </c>
       <c r="AA6" s="21">
         <f>Z6+1</f>
+        <v>46301</v>
       </c>
       <c r="AB6" s="21">
         <f>AA6+1</f>
+        <v>46302</v>
       </c>
       <c r="AC6" s="21">
         <f>AB6+1</f>
+        <v>46303</v>
       </c>
       <c r="AD6" s="21">
         <f>AC6+1</f>
+        <v>46304</v>
       </c>
       <c r="AE6" s="22">
         <f>AD6+1</f>
+        <v>46305</v>
       </c>
       <c r="AF6" s="22">
         <f>AE6+1</f>
+        <v>46306</v>
       </c>
       <c r="AG6" s="21">
         <f>AF6+1</f>
+        <v>46307</v>
       </c>
       <c r="AH6" s="21">
         <f>AG6+1</f>
+        <v>46308</v>
       </c>
       <c r="AI6" s="21">
         <f>AH6+1</f>
+        <v>46309</v>
       </c>
       <c r="AJ6" s="21">
         <f>AI6+1</f>
+        <v>46310</v>
       </c>
       <c r="AK6" s="21">
         <f>AJ6+1</f>
+        <v>46311</v>
       </c>
       <c r="AL6" s="22">
         <f>AK6+1</f>
+        <v>46312</v>
       </c>
       <c r="AM6" s="22">
         <f>AL6+1</f>
+        <v>46313</v>
       </c>
       <c r="AN6" s="21">
         <f>AM6+1</f>
+        <v>46314</v>
       </c>
       <c r="AO6" s="21">
         <f>AN6+1</f>
+        <v>46315</v>
       </c>
       <c r="AP6" s="21">
         <f>AO6+1</f>
+        <v>46316</v>
       </c>
       <c r="AQ6" s="21">
         <f>AP6+1</f>
+        <v>46317</v>
       </c>
     </row>
     <row r="7" spans="1:412" x14ac:dyDescent="0.25">
@@ -1688,12 +1736,14 @@
       </c>
       <c r="B7" s="24">
         <f>G7+H7+I7</f>
+        <v>280</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="26">
         <f>K7</f>
+        <v>35365.28</v>
       </c>
       <c r="E7" s="27"/>
       <c r="F7" s="27" t="s">
@@ -1701,18 +1751,23 @@
       </c>
       <c r="G7" s="24">
         <f>B10</f>
+        <v>212</v>
       </c>
       <c r="H7" s="24">
         <f>B11</f>
+        <v>44</v>
       </c>
       <c r="I7" s="24">
         <f>B12</f>
+        <v>24</v>
       </c>
       <c r="J7" s="24">
         <f>B13</f>
+        <v>22</v>
       </c>
       <c r="K7" s="28">
         <f>D10+D11+D12</f>
+        <v>35365.28</v>
       </c>
       <c r="L7" s="29"/>
       <c r="M7" s="30"/>
@@ -1984,13 +2039,16 @@
       <c r="A10" s="47"/>
       <c r="B10" s="48">
         <f>SUM(L10:AQ10)</f>
+        <v>212</v>
       </c>
       <c r="C10" s="49"/>
       <c r="D10" s="50">
         <f>B10*E10</f>
+        <v>23674.04</v>
       </c>
       <c r="E10" s="50">
         <f>'Rate Tables'!C7</f>
+        <v>111.67</v>
       </c>
       <c r="F10" s="51" t="s">
         <v>35</v>
@@ -2104,13 +2162,16 @@
       <c r="A11" s="47"/>
       <c r="B11" s="48">
         <f>SUM(L11:AQ11)</f>
+        <v>44</v>
       </c>
       <c r="C11" s="49"/>
       <c r="D11" s="50">
         <f>B11*E11</f>
+        <v>6873.240000000001</v>
       </c>
       <c r="E11" s="50">
         <f>'Rate Tables'!D7</f>
+        <v>156.21</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>36</v>
@@ -2224,13 +2285,16 @@
       <c r="A12" s="47"/>
       <c r="B12" s="48">
         <f>SUM(L12:AQ12)</f>
+        <v>24</v>
       </c>
       <c r="C12" s="49"/>
       <c r="D12" s="50">
         <f>B12*E12</f>
+        <v>4818</v>
       </c>
       <c r="E12" s="50">
         <f>'Rate Tables'!E7</f>
+        <v>200.75</v>
       </c>
       <c r="F12" s="51" t="s">
         <v>37</v>
@@ -2344,10 +2408,12 @@
       <c r="A13" s="57"/>
       <c r="B13" s="58">
         <f>SUM(L13:AQ13)</f>
+        <v>22</v>
       </c>
       <c r="C13" s="59"/>
       <c r="D13" s="60">
         <f>B13*E13</f>
+        <v>3080</v>
       </c>
       <c r="E13" s="60">
         <v>140</v>
@@ -2511,12 +2577,14 @@
       </c>
       <c r="B15" s="24">
         <f>G15+H15+I15</f>
+        <v>232</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>29</v>
       </c>
       <c r="D15" s="26">
         <f>K15</f>
+        <v>30005.120000000003</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="27" t="s">
@@ -2524,18 +2592,23 @@
       </c>
       <c r="G15" s="24">
         <f>B18</f>
+        <v>164</v>
       </c>
       <c r="H15" s="24">
         <f>B19</f>
+        <v>44</v>
       </c>
       <c r="I15" s="24">
         <f>B20</f>
+        <v>24</v>
       </c>
       <c r="J15" s="24">
         <f>B21</f>
+        <v>22</v>
       </c>
       <c r="K15" s="28">
         <f>D18+D19+D20</f>
+        <v>30005.120000000003</v>
       </c>
       <c r="L15" s="29"/>
       <c r="M15" s="30"/>
@@ -2807,13 +2880,16 @@
       <c r="A18" s="47"/>
       <c r="B18" s="48">
         <f>SUM(L18:AQ18)</f>
+        <v>164</v>
       </c>
       <c r="C18" s="49"/>
       <c r="D18" s="50">
         <f>B18*E18</f>
+        <v>18313.88</v>
       </c>
       <c r="E18" s="50">
         <f>'Rate Tables'!C7</f>
+        <v>111.67</v>
       </c>
       <c r="F18" s="51" t="s">
         <v>35</v>
@@ -2927,13 +3003,16 @@
       <c r="A19" s="47"/>
       <c r="B19" s="48">
         <f>SUM(L19:AQ19)</f>
+        <v>44</v>
       </c>
       <c r="C19" s="49"/>
       <c r="D19" s="50">
         <f>B19*E19</f>
+        <v>6873.240000000001</v>
       </c>
       <c r="E19" s="50">
         <f>'Rate Tables'!D7</f>
+        <v>156.21</v>
       </c>
       <c r="F19" s="51" t="s">
         <v>36</v>
@@ -3047,13 +3126,16 @@
       <c r="A20" s="47"/>
       <c r="B20" s="48">
         <f>SUM(L20:AQ20)</f>
+        <v>24</v>
       </c>
       <c r="C20" s="49"/>
       <c r="D20" s="50">
         <f>B20*E20</f>
+        <v>4818</v>
       </c>
       <c r="E20" s="50">
         <f>'Rate Tables'!E7</f>
+        <v>200.75</v>
       </c>
       <c r="F20" s="51" t="s">
         <v>37</v>
@@ -3167,10 +3249,12 @@
       <c r="A21" s="57"/>
       <c r="B21" s="58">
         <f>SUM(L21:AQ21)</f>
+        <v>22</v>
       </c>
       <c r="C21" s="59"/>
       <c r="D21" s="60">
         <f>B21*E21</f>
+        <v>3080</v>
       </c>
       <c r="E21" s="60">
         <v>140</v>
@@ -3334,12 +3418,14 @@
       </c>
       <c r="B23" s="24">
         <f>G23+H23+I23</f>
+        <v>280</v>
       </c>
       <c r="C23" s="25" t="s">
         <v>41</v>
       </c>
       <c r="D23" s="26">
         <f>K23</f>
+        <v>33109.96000000001</v>
       </c>
       <c r="E23" s="27"/>
       <c r="F23" s="27" t="s">
@@ -3347,18 +3433,23 @@
       </c>
       <c r="G23" s="24">
         <f>B26</f>
+        <v>212</v>
       </c>
       <c r="H23" s="24">
         <f>B27</f>
+        <v>44</v>
       </c>
       <c r="I23" s="24">
         <f>B28</f>
+        <v>24</v>
       </c>
       <c r="J23" s="24">
         <f>B29</f>
+        <v>22</v>
       </c>
       <c r="K23" s="28">
         <f>D26+D27+D28</f>
+        <v>33109.96000000001</v>
       </c>
       <c r="L23" s="29"/>
       <c r="M23" s="30"/>
@@ -3630,13 +3721,16 @@
       <c r="A26" s="47"/>
       <c r="B26" s="48">
         <f>SUM(L26:AQ26)</f>
+        <v>212</v>
       </c>
       <c r="C26" s="49"/>
       <c r="D26" s="50">
         <f>B26*E26</f>
+        <v>22421.120000000003</v>
       </c>
       <c r="E26" s="50">
         <f>'Rate Tables'!C8</f>
+        <v>105.76</v>
       </c>
       <c r="F26" s="51" t="s">
         <v>35</v>
@@ -3750,13 +3844,16 @@
       <c r="A27" s="47"/>
       <c r="B27" s="48">
         <f>SUM(L27:AQ27)</f>
+        <v>44</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="50">
         <f>B27*E27</f>
+        <v>6325.88</v>
       </c>
       <c r="E27" s="50">
         <f>'Rate Tables'!D8</f>
+        <v>143.77</v>
       </c>
       <c r="F27" s="51" t="s">
         <v>36</v>
@@ -3870,13 +3967,16 @@
       <c r="A28" s="47"/>
       <c r="B28" s="48">
         <f>SUM(L28:AQ28)</f>
+        <v>24</v>
       </c>
       <c r="C28" s="49"/>
       <c r="D28" s="50">
         <f>B28*E28</f>
+        <v>4362.96</v>
       </c>
       <c r="E28" s="50">
         <f>'Rate Tables'!E8</f>
+        <v>181.79</v>
       </c>
       <c r="F28" s="51" t="s">
         <v>37</v>
@@ -3990,10 +4090,12 @@
       <c r="A29" s="57"/>
       <c r="B29" s="58">
         <f>SUM(L29:AQ29)</f>
+        <v>22</v>
       </c>
       <c r="C29" s="59"/>
       <c r="D29" s="60">
         <f>B29*E29</f>
+        <v>3080</v>
       </c>
       <c r="E29" s="60">
         <v>140</v>
@@ -4157,12 +4259,14 @@
       </c>
       <c r="B31" s="24">
         <f>G31+H31+I31</f>
+        <v>232</v>
       </c>
       <c r="C31" s="25" t="s">
         <v>41</v>
       </c>
       <c r="D31" s="26">
         <f>K31</f>
+        <v>28033.48</v>
       </c>
       <c r="E31" s="27"/>
       <c r="F31" s="27" t="s">
@@ -4170,18 +4274,23 @@
       </c>
       <c r="G31" s="24">
         <f>B34</f>
+        <v>164</v>
       </c>
       <c r="H31" s="24">
         <f>B35</f>
+        <v>44</v>
       </c>
       <c r="I31" s="24">
         <f>B36</f>
+        <v>24</v>
       </c>
       <c r="J31" s="24">
         <f>B37</f>
+        <v>22</v>
       </c>
       <c r="K31" s="28">
         <f>D34+D35+D36</f>
+        <v>28033.48</v>
       </c>
       <c r="L31" s="29"/>
       <c r="M31" s="30"/>
@@ -4453,13 +4562,16 @@
       <c r="A34" s="47"/>
       <c r="B34" s="48">
         <f>SUM(L34:AQ34)</f>
+        <v>164</v>
       </c>
       <c r="C34" s="49"/>
       <c r="D34" s="50">
         <f>B34*E34</f>
+        <v>17344.64</v>
       </c>
       <c r="E34" s="50">
         <f>'Rate Tables'!C8</f>
+        <v>105.76</v>
       </c>
       <c r="F34" s="51" t="s">
         <v>35</v>
@@ -4573,13 +4685,16 @@
       <c r="A35" s="47"/>
       <c r="B35" s="48">
         <f>SUM(L35:AQ35)</f>
+        <v>44</v>
       </c>
       <c r="C35" s="49"/>
       <c r="D35" s="50">
         <f>B35*E35</f>
+        <v>6325.88</v>
       </c>
       <c r="E35" s="50">
         <f>'Rate Tables'!D8</f>
+        <v>143.77</v>
       </c>
       <c r="F35" s="51" t="s">
         <v>36</v>
@@ -4693,13 +4808,16 @@
       <c r="A36" s="47"/>
       <c r="B36" s="48">
         <f>SUM(L36:AQ36)</f>
+        <v>24</v>
       </c>
       <c r="C36" s="49"/>
       <c r="D36" s="50">
         <f>B36*E36</f>
+        <v>4362.96</v>
       </c>
       <c r="E36" s="50">
         <f>'Rate Tables'!E8</f>
+        <v>181.79</v>
       </c>
       <c r="F36" s="51" t="s">
         <v>37</v>
@@ -4813,10 +4931,12 @@
       <c r="A37" s="57"/>
       <c r="B37" s="58">
         <f>SUM(L37:AQ37)</f>
+        <v>22</v>
       </c>
       <c r="C37" s="59"/>
       <c r="D37" s="60">
         <f>B37*E37</f>
+        <v>3080</v>
       </c>
       <c r="E37" s="60">
         <v>140</v>
@@ -4980,12 +5100,14 @@
       </c>
       <c r="B39" s="24">
         <f>G39+H39+I39</f>
+        <v>280</v>
       </c>
       <c r="C39" s="25" t="s">
         <v>44</v>
       </c>
       <c r="D39" s="26">
         <f>K39</f>
+        <v>28354.399999999998</v>
       </c>
       <c r="E39" s="27"/>
       <c r="F39" s="27" t="s">
@@ -4993,18 +5115,23 @@
       </c>
       <c r="G39" s="24">
         <f>B42</f>
+        <v>212</v>
       </c>
       <c r="H39" s="24">
         <f>B43</f>
+        <v>44</v>
       </c>
       <c r="I39" s="24">
         <f>B44</f>
+        <v>24</v>
       </c>
       <c r="J39" s="24">
         <f>B45</f>
+        <v>22</v>
       </c>
       <c r="K39" s="28">
         <f>D42+D43+D44</f>
+        <v>28354.399999999998</v>
       </c>
       <c r="L39" s="29"/>
       <c r="M39" s="30"/>
@@ -5276,13 +5403,16 @@
       <c r="A42" s="47"/>
       <c r="B42" s="48">
         <f>SUM(L42:AQ42)</f>
+        <v>212</v>
       </c>
       <c r="C42" s="49"/>
       <c r="D42" s="50">
         <f>B42*E42</f>
+        <v>19296.239999999998</v>
       </c>
       <c r="E42" s="50">
         <f>'Rate Tables'!C9</f>
+        <v>91.02</v>
       </c>
       <c r="F42" s="51" t="s">
         <v>35</v>
@@ -5396,13 +5526,16 @@
       <c r="A43" s="47"/>
       <c r="B43" s="48">
         <f>SUM(L43:AQ43)</f>
+        <v>44</v>
       </c>
       <c r="C43" s="49"/>
       <c r="D43" s="50">
         <f>B43*E43</f>
+        <v>5376.8</v>
       </c>
       <c r="E43" s="50">
         <f>'Rate Tables'!D9</f>
+        <v>122.2</v>
       </c>
       <c r="F43" s="51" t="s">
         <v>36</v>
@@ -5516,13 +5649,16 @@
       <c r="A44" s="47"/>
       <c r="B44" s="48">
         <f>SUM(L44:AQ44)</f>
+        <v>24</v>
       </c>
       <c r="C44" s="49"/>
       <c r="D44" s="50">
         <f>B44*E44</f>
+        <v>3681.3599999999997</v>
       </c>
       <c r="E44" s="50">
         <f>'Rate Tables'!E9</f>
+        <v>153.39</v>
       </c>
       <c r="F44" s="51" t="s">
         <v>37</v>
@@ -5636,10 +5772,12 @@
       <c r="A45" s="57"/>
       <c r="B45" s="58">
         <f>SUM(L45:AQ45)</f>
+        <v>22</v>
       </c>
       <c r="C45" s="59"/>
       <c r="D45" s="60">
         <f>B45*E45</f>
+        <v>3080</v>
       </c>
       <c r="E45" s="60">
         <v>140</v>
@@ -5803,12 +5941,14 @@
       </c>
       <c r="B47" s="24">
         <f>G47+H47+I47</f>
+        <v>232</v>
       </c>
       <c r="C47" s="25" t="s">
         <v>44</v>
       </c>
       <c r="D47" s="26">
         <f>K47</f>
+        <v>23985.44</v>
       </c>
       <c r="E47" s="27"/>
       <c r="F47" s="27" t="s">
@@ -5816,18 +5956,23 @@
       </c>
       <c r="G47" s="24">
         <f>B50</f>
+        <v>164</v>
       </c>
       <c r="H47" s="24">
         <f>B51</f>
+        <v>44</v>
       </c>
       <c r="I47" s="24">
         <f>B52</f>
+        <v>24</v>
       </c>
       <c r="J47" s="24">
         <f>B53</f>
+        <v>22</v>
       </c>
       <c r="K47" s="28">
         <f>D50+D51+D52</f>
+        <v>23985.44</v>
       </c>
       <c r="L47" s="29"/>
       <c r="M47" s="30"/>
@@ -6099,13 +6244,16 @@
       <c r="A50" s="47"/>
       <c r="B50" s="48">
         <f>SUM(L50:AQ50)</f>
+        <v>164</v>
       </c>
       <c r="C50" s="49"/>
       <c r="D50" s="50">
         <f>B50*E50</f>
+        <v>14927.279999999999</v>
       </c>
       <c r="E50" s="50">
         <f>'Rate Tables'!C9</f>
+        <v>91.02</v>
       </c>
       <c r="F50" s="51" t="s">
         <v>35</v>
@@ -6219,13 +6367,16 @@
       <c r="A51" s="47"/>
       <c r="B51" s="48">
         <f>SUM(L51:AQ51)</f>
+        <v>44</v>
       </c>
       <c r="C51" s="49"/>
       <c r="D51" s="50">
         <f>B51*E51</f>
+        <v>5376.8</v>
       </c>
       <c r="E51" s="50">
         <f>'Rate Tables'!D9</f>
+        <v>122.2</v>
       </c>
       <c r="F51" s="51" t="s">
         <v>36</v>
@@ -6339,13 +6490,16 @@
       <c r="A52" s="47"/>
       <c r="B52" s="48">
         <f>SUM(L52:AQ52)</f>
+        <v>24</v>
       </c>
       <c r="C52" s="49"/>
       <c r="D52" s="50">
         <f>B52*E52</f>
+        <v>3681.3599999999997</v>
       </c>
       <c r="E52" s="50">
         <f>'Rate Tables'!E9</f>
+        <v>153.39</v>
       </c>
       <c r="F52" s="51" t="s">
         <v>37</v>
@@ -6459,10 +6613,12 @@
       <c r="A53" s="57"/>
       <c r="B53" s="58">
         <f>SUM(L53:AQ53)</f>
+        <v>22</v>
       </c>
       <c r="C53" s="59"/>
       <c r="D53" s="60">
         <f>B53*E53</f>
+        <v>3080</v>
       </c>
       <c r="E53" s="60">
         <v>140</v>
@@ -6626,12 +6782,14 @@
       </c>
       <c r="B55" s="24">
         <f>G55+H55+I55</f>
+        <v>280</v>
       </c>
       <c r="C55" s="25" t="s">
         <v>47</v>
       </c>
       <c r="D55" s="26">
         <f>K55</f>
+        <v>36191.68</v>
       </c>
       <c r="E55" s="27"/>
       <c r="F55" s="27" t="s">
@@ -6639,18 +6797,23 @@
       </c>
       <c r="G55" s="24">
         <f>B58</f>
+        <v>192</v>
       </c>
       <c r="H55" s="24">
         <f>B59</f>
+        <v>64</v>
       </c>
       <c r="I55" s="24">
         <f>B60</f>
+        <v>24</v>
       </c>
       <c r="J55" s="24">
         <f>B61</f>
+        <v>22</v>
       </c>
       <c r="K55" s="28">
         <f>D58+D59+D60</f>
+        <v>36191.68</v>
       </c>
       <c r="L55" s="29"/>
       <c r="M55" s="30"/>
@@ -6922,13 +7085,16 @@
       <c r="A58" s="47"/>
       <c r="B58" s="48">
         <f>SUM(L58:AQ58)</f>
+        <v>192</v>
       </c>
       <c r="C58" s="49"/>
       <c r="D58" s="50">
         <f>B58*E58</f>
+        <v>21354.239999999998</v>
       </c>
       <c r="E58" s="50">
         <f>'Rate Tables'!C10</f>
+        <v>111.22</v>
       </c>
       <c r="F58" s="51" t="s">
         <v>35</v>
@@ -7042,13 +7208,16 @@
       <c r="A59" s="47"/>
       <c r="B59" s="48">
         <f>SUM(L59:AQ59)</f>
+        <v>64</v>
       </c>
       <c r="C59" s="49"/>
       <c r="D59" s="50">
         <f>B59*E59</f>
+        <v>10003.84</v>
       </c>
       <c r="E59" s="50">
         <f>'Rate Tables'!D10</f>
+        <v>156.31</v>
       </c>
       <c r="F59" s="51" t="s">
         <v>36</v>
@@ -7162,13 +7331,16 @@
       <c r="A60" s="47"/>
       <c r="B60" s="48">
         <f>SUM(L60:AQ60)</f>
+        <v>24</v>
       </c>
       <c r="C60" s="49"/>
       <c r="D60" s="50">
         <f>B60*E60</f>
+        <v>4833.6</v>
       </c>
       <c r="E60" s="50">
         <f>'Rate Tables'!E10</f>
+        <v>201.4</v>
       </c>
       <c r="F60" s="51" t="s">
         <v>37</v>
@@ -7282,10 +7454,12 @@
       <c r="A61" s="57"/>
       <c r="B61" s="58">
         <f>SUM(L61:AQ61)</f>
+        <v>22</v>
       </c>
       <c r="C61" s="59"/>
       <c r="D61" s="60">
         <f>B61*E61</f>
+        <v>3080</v>
       </c>
       <c r="E61" s="60">
         <v>140</v>
@@ -7449,12 +7623,14 @@
       </c>
       <c r="B63" s="24">
         <f>G63+H63+I63</f>
+        <v>232</v>
       </c>
       <c r="C63" s="25" t="s">
         <v>47</v>
       </c>
       <c r="D63" s="26">
         <f>K63</f>
+        <v>30853.120000000003</v>
       </c>
       <c r="E63" s="27"/>
       <c r="F63" s="27" t="s">
@@ -7462,18 +7638,23 @@
       </c>
       <c r="G63" s="24">
         <f>B66</f>
+        <v>144</v>
       </c>
       <c r="H63" s="24">
         <f>B67</f>
+        <v>64</v>
       </c>
       <c r="I63" s="24">
         <f>B68</f>
+        <v>24</v>
       </c>
       <c r="J63" s="24">
         <f>B69</f>
+        <v>22</v>
       </c>
       <c r="K63" s="28">
         <f>D66+D67+D68</f>
+        <v>30853.120000000003</v>
       </c>
       <c r="L63" s="29"/>
       <c r="M63" s="30"/>
@@ -7745,13 +7926,16 @@
       <c r="A66" s="47"/>
       <c r="B66" s="48">
         <f>SUM(L66:AQ66)</f>
+        <v>144</v>
       </c>
       <c r="C66" s="49"/>
       <c r="D66" s="50">
         <f>B66*E66</f>
+        <v>16015.68</v>
       </c>
       <c r="E66" s="50">
         <f>'Rate Tables'!C10</f>
+        <v>111.22</v>
       </c>
       <c r="F66" s="51" t="s">
         <v>35</v>
@@ -7865,13 +8049,16 @@
       <c r="A67" s="47"/>
       <c r="B67" s="48">
         <f>SUM(L67:AQ67)</f>
+        <v>64</v>
       </c>
       <c r="C67" s="49"/>
       <c r="D67" s="50">
         <f>B67*E67</f>
+        <v>10003.84</v>
       </c>
       <c r="E67" s="50">
         <f>'Rate Tables'!D10</f>
+        <v>156.31</v>
       </c>
       <c r="F67" s="51" t="s">
         <v>36</v>
@@ -7985,13 +8172,16 @@
       <c r="A68" s="47"/>
       <c r="B68" s="48">
         <f>SUM(L68:AQ68)</f>
+        <v>24</v>
       </c>
       <c r="C68" s="49"/>
       <c r="D68" s="50">
         <f>B68*E68</f>
+        <v>4833.6</v>
       </c>
       <c r="E68" s="50">
         <f>'Rate Tables'!E10</f>
+        <v>201.4</v>
       </c>
       <c r="F68" s="51" t="s">
         <v>37</v>
@@ -8105,10 +8295,12 @@
       <c r="A69" s="57"/>
       <c r="B69" s="58">
         <f>SUM(L69:AQ69)</f>
+        <v>22</v>
       </c>
       <c r="C69" s="59"/>
       <c r="D69" s="60">
         <f>B69*E69</f>
+        <v>3080</v>
       </c>
       <c r="E69" s="60">
         <v>140</v>
@@ -8227,25 +8419,32 @@
       </c>
       <c r="B70" s="72">
         <f>SUM(B7,B15,B23,B31,B39,B47,B55,B63)</f>
+        <v>2048</v>
       </c>
       <c r="C70" s="17"/>
       <c r="D70" s="73">
         <f>SUM(D13,D21,D29,D37,D45,D53,D61,D69)</f>
+        <v>24640</v>
       </c>
       <c r="G70" s="72">
         <f>SUM(G7,G15,G23,G31,G39,G47,G55,G63)</f>
+        <v>1464</v>
       </c>
       <c r="H70" s="72">
         <f>SUM(H7,H15,H23,H31,H39,H47,H55,H63)</f>
+        <v>392</v>
       </c>
       <c r="I70" s="72">
         <f>SUM(I7,I15,I23,I31,I39,I47,I55,I63)</f>
+        <v>192</v>
       </c>
       <c r="J70" s="72">
         <f>SUM(J7,J15,J23,J31,J39,J47,J55,J63)</f>
+        <v>176</v>
       </c>
       <c r="K70" s="73">
         <f>SUM(K7,K15,K23,K31,K39,K47,K55,K63)</f>
+        <v>245898.48</v>
       </c>
     </row>
   </sheetData>
@@ -8448,96 +8647,127 @@
       </c>
       <c r="M6" s="21">
         <f>L6+1</f>
+        <v>46287</v>
       </c>
       <c r="N6" s="21">
         <f>M6+1</f>
+        <v>46288</v>
       </c>
       <c r="O6" s="21">
         <f>N6+1</f>
+        <v>46289</v>
       </c>
       <c r="P6" s="21">
         <f>O6+1</f>
+        <v>46290</v>
       </c>
       <c r="Q6" s="22">
         <f>P6+1</f>
+        <v>46291</v>
       </c>
       <c r="R6" s="22">
         <f>Q6+1</f>
+        <v>46292</v>
       </c>
       <c r="S6" s="21">
         <f>R6+1</f>
+        <v>46293</v>
       </c>
       <c r="T6" s="21">
         <f>S6+1</f>
+        <v>46294</v>
       </c>
       <c r="U6" s="21">
         <f>T6+1</f>
+        <v>46295</v>
       </c>
       <c r="V6" s="21">
         <f>U6+1</f>
+        <v>46296</v>
       </c>
       <c r="W6" s="21">
         <f>V6+1</f>
+        <v>46297</v>
       </c>
       <c r="X6" s="22">
         <f>W6+1</f>
+        <v>46298</v>
       </c>
       <c r="Y6" s="22">
         <f>X6+1</f>
+        <v>46299</v>
       </c>
       <c r="Z6" s="21">
         <f>Y6+1</f>
+        <v>46300</v>
       </c>
       <c r="AA6" s="21">
         <f>Z6+1</f>
+        <v>46301</v>
       </c>
       <c r="AB6" s="21">
         <f>AA6+1</f>
+        <v>46302</v>
       </c>
       <c r="AC6" s="21">
         <f>AB6+1</f>
+        <v>46303</v>
       </c>
       <c r="AD6" s="21">
         <f>AC6+1</f>
+        <v>46304</v>
       </c>
       <c r="AE6" s="22">
         <f>AD6+1</f>
+        <v>46305</v>
       </c>
       <c r="AF6" s="22">
         <f>AE6+1</f>
+        <v>46306</v>
       </c>
       <c r="AG6" s="21">
         <f>AF6+1</f>
+        <v>46307</v>
       </c>
       <c r="AH6" s="21">
         <f>AG6+1</f>
+        <v>46308</v>
       </c>
       <c r="AI6" s="21">
         <f>AH6+1</f>
+        <v>46309</v>
       </c>
       <c r="AJ6" s="21">
         <f>AI6+1</f>
+        <v>46310</v>
       </c>
       <c r="AK6" s="21">
         <f>AJ6+1</f>
+        <v>46311</v>
       </c>
       <c r="AL6" s="22">
         <f>AK6+1</f>
+        <v>46312</v>
       </c>
       <c r="AM6" s="22">
         <f>AL6+1</f>
+        <v>46313</v>
       </c>
       <c r="AN6" s="21">
         <f>AM6+1</f>
+        <v>46314</v>
       </c>
       <c r="AO6" s="21">
         <f>AN6+1</f>
+        <v>46315</v>
       </c>
       <c r="AP6" s="21">
         <f>AO6+1</f>
+        <v>46316</v>
       </c>
       <c r="AQ6" s="21">
         <f>AP6+1</f>
+        <v>46317</v>
       </c>
     </row>
     <row r="7" spans="1:412" x14ac:dyDescent="0.25">
@@ -8546,12 +8776,14 @@
       </c>
       <c r="B7" s="24">
         <f>G7+H7+I7</f>
+        <v>512</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>51</v>
       </c>
       <c r="D7" s="26">
         <f>K7</f>
+        <v>63360.64</v>
       </c>
       <c r="E7" s="27"/>
       <c r="F7" s="27" t="s">
@@ -8559,18 +8791,23 @@
       </c>
       <c r="G7" s="24">
         <f>B10</f>
+        <v>336</v>
       </c>
       <c r="H7" s="24">
         <f>B11</f>
+        <v>128</v>
       </c>
       <c r="I7" s="24">
         <f>B12</f>
+        <v>48</v>
       </c>
       <c r="J7" s="24">
         <f>B13</f>
+        <v>50</v>
       </c>
       <c r="K7" s="28">
         <f>D10+D11+D12</f>
+        <v>63360.64</v>
       </c>
       <c r="L7" s="29"/>
       <c r="M7" s="30"/>
@@ -8842,13 +9079,16 @@
       <c r="A10" s="47"/>
       <c r="B10" s="48">
         <f>SUM(L10:AQ10)</f>
+        <v>336</v>
       </c>
       <c r="C10" s="49"/>
       <c r="D10" s="50">
         <f>B10*E10</f>
+        <v>35374.08</v>
       </c>
       <c r="E10" s="50">
         <f>'Rate Tables'!C11</f>
+        <v>105.28</v>
       </c>
       <c r="F10" s="51" t="s">
         <v>35</v>
@@ -8962,13 +9202,16 @@
       <c r="A11" s="47"/>
       <c r="B11" s="48">
         <f>SUM(L11:AQ11)</f>
+        <v>128</v>
       </c>
       <c r="C11" s="49"/>
       <c r="D11" s="50">
         <f>B11*E11</f>
+        <v>18880</v>
       </c>
       <c r="E11" s="50">
         <f>'Rate Tables'!D11</f>
+        <v>147.5</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>36</v>
@@ -9082,13 +9325,16 @@
       <c r="A12" s="47"/>
       <c r="B12" s="48">
         <f>SUM(L12:AQ12)</f>
+        <v>48</v>
       </c>
       <c r="C12" s="49"/>
       <c r="D12" s="50">
         <f>B12*E12</f>
+        <v>9106.56</v>
       </c>
       <c r="E12" s="50">
         <f>'Rate Tables'!E11</f>
+        <v>189.72</v>
       </c>
       <c r="F12" s="51" t="s">
         <v>37</v>
@@ -9202,10 +9448,12 @@
       <c r="A13" s="57"/>
       <c r="B13" s="58">
         <f>SUM(L13:AQ13)</f>
+        <v>50</v>
       </c>
       <c r="C13" s="59"/>
       <c r="D13" s="60">
         <f>B13*E13</f>
+        <v>6500</v>
       </c>
       <c r="E13" s="60">
         <v>130</v>
@@ -9369,12 +9617,14 @@
       </c>
       <c r="B15" s="24">
         <f>G15+H15+I15</f>
+        <v>464</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>51</v>
       </c>
       <c r="D15" s="26">
         <f>K15</f>
+        <v>58307.2</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="27" t="s">
@@ -9382,18 +9632,23 @@
       </c>
       <c r="G15" s="24">
         <f>B18</f>
+        <v>288</v>
       </c>
       <c r="H15" s="24">
         <f>B19</f>
+        <v>128</v>
       </c>
       <c r="I15" s="24">
         <f>B20</f>
+        <v>48</v>
       </c>
       <c r="J15" s="24">
         <f>B21</f>
+        <v>44</v>
       </c>
       <c r="K15" s="28">
         <f>D18+D19+D20</f>
+        <v>58307.2</v>
       </c>
       <c r="L15" s="29"/>
       <c r="M15" s="30"/>
@@ -9665,13 +9920,16 @@
       <c r="A18" s="47"/>
       <c r="B18" s="48">
         <f>SUM(L18:AQ18)</f>
+        <v>288</v>
       </c>
       <c r="C18" s="49"/>
       <c r="D18" s="50">
         <f>B18*E18</f>
+        <v>30320.64</v>
       </c>
       <c r="E18" s="50">
         <f>'Rate Tables'!C11</f>
+        <v>105.28</v>
       </c>
       <c r="F18" s="51" t="s">
         <v>35</v>
@@ -9785,13 +10043,16 @@
       <c r="A19" s="47"/>
       <c r="B19" s="48">
         <f>SUM(L19:AQ19)</f>
+        <v>128</v>
       </c>
       <c r="C19" s="49"/>
       <c r="D19" s="50">
         <f>B19*E19</f>
+        <v>18880</v>
       </c>
       <c r="E19" s="50">
         <f>'Rate Tables'!D11</f>
+        <v>147.5</v>
       </c>
       <c r="F19" s="51" t="s">
         <v>36</v>
@@ -9905,13 +10166,16 @@
       <c r="A20" s="47"/>
       <c r="B20" s="48">
         <f>SUM(L20:AQ20)</f>
+        <v>48</v>
       </c>
       <c r="C20" s="49"/>
       <c r="D20" s="50">
         <f>B20*E20</f>
+        <v>9106.56</v>
       </c>
       <c r="E20" s="50">
         <f>'Rate Tables'!E11</f>
+        <v>189.72</v>
       </c>
       <c r="F20" s="51" t="s">
         <v>37</v>
@@ -10025,10 +10289,12 @@
       <c r="A21" s="57"/>
       <c r="B21" s="58">
         <f>SUM(L21:AQ21)</f>
+        <v>44</v>
       </c>
       <c r="C21" s="59"/>
       <c r="D21" s="60">
         <f>B21*E21</f>
+        <v>5720</v>
       </c>
       <c r="E21" s="60">
         <v>130</v>
@@ -10147,25 +10413,32 @@
       </c>
       <c r="B22" s="72">
         <f>SUM(B7,B15)</f>
+        <v>976</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="73">
         <f>SUM(D13,D21)</f>
+        <v>12220</v>
       </c>
       <c r="G22" s="72">
         <f>SUM(G7,G15)</f>
+        <v>624</v>
       </c>
       <c r="H22" s="72">
         <f>SUM(H7,H15)</f>
+        <v>256</v>
       </c>
       <c r="I22" s="72">
         <f>SUM(I7,I15)</f>
+        <v>96</v>
       </c>
       <c r="J22" s="72">
         <f>SUM(J7,J15)</f>
+        <v>94</v>
       </c>
       <c r="K22" s="73">
         <f>SUM(K7,K15)</f>
+        <v>121667.84</v>
       </c>
     </row>
   </sheetData>
@@ -10338,96 +10611,127 @@
       </c>
       <c r="M6" s="21">
         <f>L6+1</f>
+        <v>46287</v>
       </c>
       <c r="N6" s="21">
         <f>M6+1</f>
+        <v>46288</v>
       </c>
       <c r="O6" s="21">
         <f>N6+1</f>
+        <v>46289</v>
       </c>
       <c r="P6" s="21">
         <f>O6+1</f>
+        <v>46290</v>
       </c>
       <c r="Q6" s="22">
         <f>P6+1</f>
+        <v>46291</v>
       </c>
       <c r="R6" s="22">
         <f>Q6+1</f>
+        <v>46292</v>
       </c>
       <c r="S6" s="21">
         <f>R6+1</f>
+        <v>46293</v>
       </c>
       <c r="T6" s="21">
         <f>S6+1</f>
+        <v>46294</v>
       </c>
       <c r="U6" s="21">
         <f>T6+1</f>
+        <v>46295</v>
       </c>
       <c r="V6" s="21">
         <f>U6+1</f>
+        <v>46296</v>
       </c>
       <c r="W6" s="21">
         <f>V6+1</f>
+        <v>46297</v>
       </c>
       <c r="X6" s="22">
         <f>W6+1</f>
+        <v>46298</v>
       </c>
       <c r="Y6" s="22">
         <f>X6+1</f>
+        <v>46299</v>
       </c>
       <c r="Z6" s="21">
         <f>Y6+1</f>
+        <v>46300</v>
       </c>
       <c r="AA6" s="21">
         <f>Z6+1</f>
+        <v>46301</v>
       </c>
       <c r="AB6" s="21">
         <f>AA6+1</f>
+        <v>46302</v>
       </c>
       <c r="AC6" s="21">
         <f>AB6+1</f>
+        <v>46303</v>
       </c>
       <c r="AD6" s="21">
         <f>AC6+1</f>
+        <v>46304</v>
       </c>
       <c r="AE6" s="22">
         <f>AD6+1</f>
+        <v>46305</v>
       </c>
       <c r="AF6" s="22">
         <f>AE6+1</f>
+        <v>46306</v>
       </c>
       <c r="AG6" s="21">
         <f>AF6+1</f>
+        <v>46307</v>
       </c>
       <c r="AH6" s="21">
         <f>AG6+1</f>
+        <v>46308</v>
       </c>
       <c r="AI6" s="21">
         <f>AH6+1</f>
+        <v>46309</v>
       </c>
       <c r="AJ6" s="21">
         <f>AI6+1</f>
+        <v>46310</v>
       </c>
       <c r="AK6" s="21">
         <f>AJ6+1</f>
+        <v>46311</v>
       </c>
       <c r="AL6" s="22">
         <f>AK6+1</f>
+        <v>46312</v>
       </c>
       <c r="AM6" s="22">
         <f>AL6+1</f>
+        <v>46313</v>
       </c>
       <c r="AN6" s="21">
         <f>AM6+1</f>
+        <v>46314</v>
       </c>
       <c r="AO6" s="21">
         <f>AN6+1</f>
+        <v>46315</v>
       </c>
       <c r="AP6" s="21">
         <f>AO6+1</f>
+        <v>46316</v>
       </c>
       <c r="AQ6" s="21">
         <f>AP6+1</f>
+        <v>46317</v>
       </c>
     </row>
     <row r="7" spans="1:412" x14ac:dyDescent="0.25">
@@ -10436,12 +10740,14 @@
       </c>
       <c r="B7" s="24">
         <f>G7+H7+I7</f>
+        <v>3920</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>54</v>
       </c>
       <c r="D7" s="26">
         <f>K7</f>
+        <v>468723.36</v>
       </c>
       <c r="E7" s="27"/>
       <c r="F7" s="27" t="s">
@@ -10449,18 +10755,23 @@
       </c>
       <c r="G7" s="24">
         <f>B10</f>
+        <v>2336</v>
       </c>
       <c r="H7" s="24">
         <f>B11</f>
+        <v>1152</v>
       </c>
       <c r="I7" s="24">
         <f>B12</f>
+        <v>432</v>
       </c>
       <c r="J7" s="24">
         <f>B13</f>
+        <v>210</v>
       </c>
       <c r="K7" s="28">
         <f>D10+D11+D12</f>
+        <v>468723.36</v>
       </c>
       <c r="L7" s="29"/>
       <c r="M7" s="30"/>
@@ -10732,13 +11043,16 @@
       <c r="A10" s="47"/>
       <c r="B10" s="48">
         <f>SUM(L10:AQ10)</f>
+        <v>2336</v>
       </c>
       <c r="C10" s="49"/>
       <c r="D10" s="50">
         <f>B10*E10</f>
+        <v>232034.88</v>
       </c>
       <c r="E10" s="50">
         <f>'Rate Tables'!C12</f>
+        <v>99.33</v>
       </c>
       <c r="F10" s="51" t="s">
         <v>35</v>
@@ -10852,13 +11166,16 @@
       <c r="A11" s="47"/>
       <c r="B11" s="48">
         <f>SUM(L11:AQ11)</f>
+        <v>1152</v>
       </c>
       <c r="C11" s="49"/>
       <c r="D11" s="50">
         <f>B11*E11</f>
+        <v>159770.88</v>
       </c>
       <c r="E11" s="50">
         <f>'Rate Tables'!D12</f>
+        <v>138.69</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>36</v>
@@ -10972,13 +11289,16 @@
       <c r="A12" s="47"/>
       <c r="B12" s="48">
         <f>SUM(L12:AQ12)</f>
+        <v>432</v>
       </c>
       <c r="C12" s="49"/>
       <c r="D12" s="50">
         <f>B12*E12</f>
+        <v>76917.6</v>
       </c>
       <c r="E12" s="50">
         <f>'Rate Tables'!E12</f>
+        <v>178.05</v>
       </c>
       <c r="F12" s="51" t="s">
         <v>37</v>
@@ -11092,10 +11412,12 @@
       <c r="A13" s="57"/>
       <c r="B13" s="58">
         <f>SUM(L13:AQ13)</f>
+        <v>210</v>
       </c>
       <c r="C13" s="59"/>
       <c r="D13" s="60">
         <f>B13*E13</f>
+        <v>27300</v>
       </c>
       <c r="E13" s="60">
         <v>130</v>
@@ -11259,12 +11581,14 @@
       </c>
       <c r="B15" s="24">
         <f>G15+H15+I15</f>
+        <v>2688</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>54</v>
       </c>
       <c r="D15" s="26">
         <f>K15</f>
+        <v>337532.16</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="27" t="s">
@@ -11272,18 +11596,23 @@
       </c>
       <c r="G15" s="24">
         <f>B18</f>
+        <v>1280</v>
       </c>
       <c r="H15" s="24">
         <f>B19</f>
+        <v>1024</v>
       </c>
       <c r="I15" s="24">
         <f>B20</f>
+        <v>384</v>
       </c>
       <c r="J15" s="24">
         <f>B21</f>
+        <v>14</v>
       </c>
       <c r="K15" s="28">
         <f>D18+D19+D20</f>
+        <v>337532.16</v>
       </c>
       <c r="L15" s="29"/>
       <c r="M15" s="30"/>
@@ -11555,13 +11884,16 @@
       <c r="A18" s="47"/>
       <c r="B18" s="48">
         <f>SUM(L18:AQ18)</f>
+        <v>1280</v>
       </c>
       <c r="C18" s="49"/>
       <c r="D18" s="50">
         <f>B18*E18</f>
+        <v>127142.4</v>
       </c>
       <c r="E18" s="50">
         <f>'Rate Tables'!C12</f>
+        <v>99.33</v>
       </c>
       <c r="F18" s="51" t="s">
         <v>35</v>
@@ -11675,13 +12007,16 @@
       <c r="A19" s="47"/>
       <c r="B19" s="48">
         <f>SUM(L19:AQ19)</f>
+        <v>1024</v>
       </c>
       <c r="C19" s="49"/>
       <c r="D19" s="50">
         <f>B19*E19</f>
+        <v>142018.56</v>
       </c>
       <c r="E19" s="50">
         <f>'Rate Tables'!D12</f>
+        <v>138.69</v>
       </c>
       <c r="F19" s="51" t="s">
         <v>36</v>
@@ -11795,13 +12130,16 @@
       <c r="A20" s="47"/>
       <c r="B20" s="48">
         <f>SUM(L20:AQ20)</f>
+        <v>384</v>
       </c>
       <c r="C20" s="49"/>
       <c r="D20" s="50">
         <f>B20*E20</f>
+        <v>68371.20000000001</v>
       </c>
       <c r="E20" s="50">
         <f>'Rate Tables'!E12</f>
+        <v>178.05</v>
       </c>
       <c r="F20" s="51" t="s">
         <v>37</v>
@@ -11915,10 +12253,12 @@
       <c r="A21" s="57"/>
       <c r="B21" s="58">
         <f>SUM(L21:AQ21)</f>
+        <v>14</v>
       </c>
       <c r="C21" s="59"/>
       <c r="D21" s="60">
         <f>B21*E21</f>
+        <v>1820</v>
       </c>
       <c r="E21" s="60">
         <v>130</v>
@@ -12037,25 +12377,32 @@
       </c>
       <c r="B22" s="72">
         <f>SUM(B7,B15)</f>
+        <v>6608</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="73">
         <f>SUM(D13,D21)</f>
+        <v>29120</v>
       </c>
       <c r="G22" s="72">
         <f>SUM(G7,G15)</f>
+        <v>3616</v>
       </c>
       <c r="H22" s="72">
         <f>SUM(H7,H15)</f>
+        <v>2176</v>
       </c>
       <c r="I22" s="72">
         <f>SUM(I7,I15)</f>
+        <v>816</v>
       </c>
       <c r="J22" s="72">
         <f>SUM(J7,J15)</f>
+        <v>224</v>
       </c>
       <c r="K22" s="73">
         <f>SUM(K7,K15)</f>
+        <v>806255.52</v>
       </c>
     </row>
   </sheetData>
@@ -12228,96 +12575,127 @@
       </c>
       <c r="M6" s="21">
         <f>L6+1</f>
+        <v>46287</v>
       </c>
       <c r="N6" s="21">
         <f>M6+1</f>
+        <v>46288</v>
       </c>
       <c r="O6" s="21">
         <f>N6+1</f>
+        <v>46289</v>
       </c>
       <c r="P6" s="21">
         <f>O6+1</f>
+        <v>46290</v>
       </c>
       <c r="Q6" s="22">
         <f>P6+1</f>
+        <v>46291</v>
       </c>
       <c r="R6" s="22">
         <f>Q6+1</f>
+        <v>46292</v>
       </c>
       <c r="S6" s="21">
         <f>R6+1</f>
+        <v>46293</v>
       </c>
       <c r="T6" s="21">
         <f>S6+1</f>
+        <v>46294</v>
       </c>
       <c r="U6" s="21">
         <f>T6+1</f>
+        <v>46295</v>
       </c>
       <c r="V6" s="21">
         <f>U6+1</f>
+        <v>46296</v>
       </c>
       <c r="W6" s="21">
         <f>V6+1</f>
+        <v>46297</v>
       </c>
       <c r="X6" s="22">
         <f>W6+1</f>
+        <v>46298</v>
       </c>
       <c r="Y6" s="22">
         <f>X6+1</f>
+        <v>46299</v>
       </c>
       <c r="Z6" s="21">
         <f>Y6+1</f>
+        <v>46300</v>
       </c>
       <c r="AA6" s="21">
         <f>Z6+1</f>
+        <v>46301</v>
       </c>
       <c r="AB6" s="21">
         <f>AA6+1</f>
+        <v>46302</v>
       </c>
       <c r="AC6" s="21">
         <f>AB6+1</f>
+        <v>46303</v>
       </c>
       <c r="AD6" s="21">
         <f>AC6+1</f>
+        <v>46304</v>
       </c>
       <c r="AE6" s="22">
         <f>AD6+1</f>
+        <v>46305</v>
       </c>
       <c r="AF6" s="22">
         <f>AE6+1</f>
+        <v>46306</v>
       </c>
       <c r="AG6" s="21">
         <f>AF6+1</f>
+        <v>46307</v>
       </c>
       <c r="AH6" s="21">
         <f>AG6+1</f>
+        <v>46308</v>
       </c>
       <c r="AI6" s="21">
         <f>AH6+1</f>
+        <v>46309</v>
       </c>
       <c r="AJ6" s="21">
         <f>AI6+1</f>
+        <v>46310</v>
       </c>
       <c r="AK6" s="21">
         <f>AJ6+1</f>
+        <v>46311</v>
       </c>
       <c r="AL6" s="22">
         <f>AK6+1</f>
+        <v>46312</v>
       </c>
       <c r="AM6" s="22">
         <f>AL6+1</f>
+        <v>46313</v>
       </c>
       <c r="AN6" s="21">
         <f>AM6+1</f>
+        <v>46314</v>
       </c>
       <c r="AO6" s="21">
         <f>AN6+1</f>
+        <v>46315</v>
       </c>
       <c r="AP6" s="21">
         <f>AO6+1</f>
+        <v>46316</v>
       </c>
       <c r="AQ6" s="21">
         <f>AP6+1</f>
+        <v>46317</v>
       </c>
     </row>
     <row r="7" spans="1:412" x14ac:dyDescent="0.25">
@@ -12326,12 +12704,14 @@
       </c>
       <c r="B7" s="24">
         <f>G7+H7+I7</f>
+        <v>280</v>
       </c>
       <c r="C7" s="25" t="s">
         <v>57</v>
       </c>
       <c r="D7" s="26">
         <f>K7</f>
+        <v>35319.439999999995</v>
       </c>
       <c r="E7" s="27"/>
       <c r="F7" s="27" t="s">
@@ -12339,18 +12719,23 @@
       </c>
       <c r="G7" s="24">
         <f>B10</f>
+        <v>192</v>
       </c>
       <c r="H7" s="24">
         <f>B11</f>
+        <v>64</v>
       </c>
       <c r="I7" s="24">
         <f>B12</f>
+        <v>24</v>
       </c>
       <c r="J7" s="24">
         <f>B13</f>
+        <v>28</v>
       </c>
       <c r="K7" s="28">
         <f>D10+D11+D12</f>
+        <v>35319.439999999995</v>
       </c>
       <c r="L7" s="29"/>
       <c r="M7" s="30"/>
@@ -12622,13 +13007,16 @@
       <c r="A10" s="47"/>
       <c r="B10" s="48">
         <f>SUM(L10:AQ10)</f>
+        <v>192</v>
       </c>
       <c r="C10" s="49"/>
       <c r="D10" s="50">
         <f>B10*E10</f>
+        <v>20808.96</v>
       </c>
       <c r="E10" s="50">
         <f>'Rate Tables'!C13</f>
+        <v>108.38</v>
       </c>
       <c r="F10" s="51" t="s">
         <v>35</v>
@@ -12742,13 +13130,16 @@
       <c r="A11" s="47"/>
       <c r="B11" s="48">
         <f>SUM(L11:AQ11)</f>
+        <v>64</v>
       </c>
       <c r="C11" s="49"/>
       <c r="D11" s="50">
         <f>B11*E11</f>
+        <v>9777.92</v>
       </c>
       <c r="E11" s="50">
         <f>'Rate Tables'!D13</f>
+        <v>152.78</v>
       </c>
       <c r="F11" s="51" t="s">
         <v>36</v>
@@ -12862,13 +13253,16 @@
       <c r="A12" s="47"/>
       <c r="B12" s="48">
         <f>SUM(L12:AQ12)</f>
+        <v>24</v>
       </c>
       <c r="C12" s="49"/>
       <c r="D12" s="50">
         <f>B12*E12</f>
+        <v>4732.5599999999995</v>
       </c>
       <c r="E12" s="50">
         <f>'Rate Tables'!E13</f>
+        <v>197.19</v>
       </c>
       <c r="F12" s="51" t="s">
         <v>37</v>
@@ -12982,10 +13376,12 @@
       <c r="A13" s="57"/>
       <c r="B13" s="58">
         <f>SUM(L13:AQ13)</f>
+        <v>28</v>
       </c>
       <c r="C13" s="59"/>
       <c r="D13" s="60">
         <f>B13*E13</f>
+        <v>3640</v>
       </c>
       <c r="E13" s="60">
         <v>130</v>
@@ -13149,12 +13545,14 @@
       </c>
       <c r="B15" s="24">
         <f>G15+H15+I15</f>
+        <v>168</v>
       </c>
       <c r="C15" s="25" t="s">
         <v>57</v>
       </c>
       <c r="D15" s="26">
         <f>K15</f>
+        <v>23180.879999999997</v>
       </c>
       <c r="E15" s="27"/>
       <c r="F15" s="27" t="s">
@@ -13162,18 +13560,23 @@
       </c>
       <c r="G15" s="24">
         <f>B18</f>
+        <v>80</v>
       </c>
       <c r="H15" s="24">
         <f>B19</f>
+        <v>64</v>
       </c>
       <c r="I15" s="24">
         <f>B20</f>
+        <v>24</v>
       </c>
       <c r="J15" s="24">
         <f>B21</f>
+        <v>14</v>
       </c>
       <c r="K15" s="28">
         <f>D18+D19+D20</f>
+        <v>23180.879999999997</v>
       </c>
       <c r="L15" s="29"/>
       <c r="M15" s="30"/>
@@ -13445,13 +13848,16 @@
       <c r="A18" s="47"/>
       <c r="B18" s="48">
         <f>SUM(L18:AQ18)</f>
+        <v>80</v>
       </c>
       <c r="C18" s="49"/>
       <c r="D18" s="50">
         <f>B18*E18</f>
+        <v>8670.4</v>
       </c>
       <c r="E18" s="50">
         <f>'Rate Tables'!C13</f>
+        <v>108.38</v>
       </c>
       <c r="F18" s="51" t="s">
         <v>35</v>
@@ -13565,13 +13971,16 @@
       <c r="A19" s="47"/>
       <c r="B19" s="48">
         <f>SUM(L19:AQ19)</f>
+        <v>64</v>
       </c>
       <c r="C19" s="49"/>
       <c r="D19" s="50">
         <f>B19*E19</f>
+        <v>9777.92</v>
       </c>
       <c r="E19" s="50">
         <f>'Rate Tables'!D13</f>
+        <v>152.78</v>
       </c>
       <c r="F19" s="51" t="s">
         <v>36</v>
@@ -13685,13 +14094,16 @@
       <c r="A20" s="47"/>
       <c r="B20" s="48">
         <f>SUM(L20:AQ20)</f>
+        <v>24</v>
       </c>
       <c r="C20" s="49"/>
       <c r="D20" s="50">
         <f>B20*E20</f>
+        <v>4732.5599999999995</v>
       </c>
       <c r="E20" s="50">
         <f>'Rate Tables'!E13</f>
+        <v>197.19</v>
       </c>
       <c r="F20" s="51" t="s">
         <v>37</v>
@@ -13805,10 +14217,12 @@
       <c r="A21" s="57"/>
       <c r="B21" s="58">
         <f>SUM(L21:AQ21)</f>
+        <v>14</v>
       </c>
       <c r="C21" s="59"/>
       <c r="D21" s="60">
         <f>B21*E21</f>
+        <v>1820</v>
       </c>
       <c r="E21" s="60">
         <v>130</v>
@@ -13927,25 +14341,32 @@
       </c>
       <c r="B22" s="72">
         <f>SUM(B7,B15)</f>
+        <v>448</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="73">
         <f>SUM(D13,D21)</f>
+        <v>5460</v>
       </c>
       <c r="G22" s="72">
         <f>SUM(G7,G15)</f>
+        <v>272</v>
       </c>
       <c r="H22" s="72">
         <f>SUM(H7,H15)</f>
+        <v>128</v>
       </c>
       <c r="I22" s="72">
         <f>SUM(I7,I15)</f>
+        <v>48</v>
       </c>
       <c r="J22" s="72">
         <f>SUM(J7,J15)</f>
+        <v>42</v>
       </c>
       <c r="K22" s="73">
         <f>SUM(K7,K15)</f>
+        <v>58500.31999999999</v>
       </c>
     </row>
   </sheetData>
@@ -14063,6 +14484,7 @@
       </c>
       <c r="G7" s="75">
         <f>C7*D7*E7+F7</f>
+        <v>66960</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -14086,6 +14508,7 @@
       </c>
       <c r="G8" s="75">
         <f>C8*D8*E8+F8</f>
+        <v>3672</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -14109,6 +14532,7 @@
       </c>
       <c r="G9" s="75">
         <f>C9*D9*E9+F9</f>
+        <v>5616</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -14132,6 +14556,7 @@
       </c>
       <c r="G10" s="75">
         <f>C10*D10*E10+F10</f>
+        <v>37120</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -14140,6 +14565,7 @@
       </c>
       <c r="G11" s="73">
         <f>SUM(G7:G10)</f>
+        <v>113368</v>
       </c>
     </row>
   </sheetData>
@@ -14225,6 +14651,7 @@
       </c>
       <c r="E7" s="75">
         <f>B7*C7*D7</f>
+        <v>6840</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -14233,6 +14660,7 @@
       </c>
       <c r="E8" s="73">
         <f>SUM(E7:E7)</f>
+        <v>6840</v>
       </c>
     </row>
   </sheetData>
@@ -14318,6 +14746,7 @@
       </c>
       <c r="E7" s="75">
         <f>C7*D7</f>
+        <v>3500</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -14335,6 +14764,7 @@
       </c>
       <c r="E8" s="75">
         <f>C8*D8</f>
+        <v>1200</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -14352,6 +14782,7 @@
       </c>
       <c r="E9" s="75">
         <f>C9*D9</f>
+        <v>6000</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -14360,6 +14791,7 @@
       </c>
       <c r="E10" s="73">
         <f>SUM(E7:E9)</f>
+        <v>10700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clear yellow voids on HC/HPS B–K; yellow stays on day cells
Paint empty metric columns white on Enter Hours rows so they are not
fake input holes. Day-grid HC/HPS cells stay yellow. Craft cages,
formula lock, and desk totals unchanged. Regenerated Look samples.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -399,7 +399,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -429,6 +429,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDBDBDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -743,41 +748,41 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="3" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="3" fontId="5" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="5" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="5" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="5" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
@@ -786,7 +791,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -815,11 +820,11 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>

</xml_diff>

<commit_message>
Regenerate Aromatics and CAT 2 Look samples after TOTAL-bar and BW fill
v151_real_aromatics.xlsx and v151_real_cat2.xlsx rebuilt from the live vault
packs so Rate Tables COMP BW and continuous amber TOTAL bars are in the
client files. Desk ESTIMATE TOTAL $ unchanged.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -332,7 +332,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="D-MMM"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -402,6 +402,17 @@
       <b/>
       <color rgb="FF083943"/>
       <sz val="9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF3D4F54"/>
+      <sz val="9"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF083943"/>
+      <sz val="10"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -527,6 +538,21 @@
       </top>
       <bottom style="hair">
         <color rgb="FF8AA3A1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="hair">
+        <color rgb="FF8AA3A1"/>
+      </left>
+      <right style="hair">
+        <color rgb="FF8AA3A1"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -691,26 +717,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="hair">
-        <color rgb="FF8AA3A1"/>
-      </left>
-      <right style="hair">
-        <color rgb="FF8AA3A1"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -742,13 +753,13 @@
     <xf numFmtId="164" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="165" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="164" fontId="8" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -767,30 +778,30 @@
     <xf numFmtId="166" fontId="9" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="5" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="5" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -799,16 +810,16 @@
     <xf numFmtId="3" fontId="5" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="3" fontId="5" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
@@ -817,10 +828,10 @@
     <xf numFmtId="165" fontId="5" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="165" fontId="5" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -830,54 +841,59 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="165" fontId="5" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="165" fontId="5" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="165" fontId="5" fillId="13" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="9" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="165" fontId="5" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="5" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="14" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="5" fillId="14" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="5" fillId="13" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="13" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="9" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="13" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="9" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="13" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="15" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="165" fontId="7" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="3" fontId="5" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="3" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8495,35 +8511,37 @@
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A70" s="86" t="s">
+      <c r="A70" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B70" s="87">
+      <c r="B70" s="17">
         <f>SUM(B7,B15,B23,B31,B39,B47,B55,B63)</f>
         <v>2048</v>
       </c>
-      <c r="C70" s="22"/>
-      <c r="D70" s="88">
+      <c r="C70" s="86"/>
+      <c r="D70" s="21">
         <f>SUM(D13,D21,D29,D37,D45,D53,D61,D69)</f>
         <v>24640</v>
       </c>
-      <c r="G70" s="87">
+      <c r="E70" s="16"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="17">
         <f>SUM(G7,G15,G23,G31,G39,G47,G55,G63)</f>
         <v>1464</v>
       </c>
-      <c r="H70" s="87">
+      <c r="H70" s="17">
         <f>SUM(H7,H15,H23,H31,H39,H47,H55,H63)</f>
         <v>392</v>
       </c>
-      <c r="I70" s="87">
+      <c r="I70" s="17">
         <f>SUM(I7,I15,I23,I31,I39,I47,I55,I63)</f>
         <v>192</v>
       </c>
-      <c r="J70" s="87">
+      <c r="J70" s="17">
         <f>SUM(J7,J15,J23,J31,J39,J47,J55,J63)</f>
         <v>176</v>
       </c>
-      <c r="K70" s="88">
+      <c r="K70" s="21">
         <f>SUM(K7,K15,K23,K31,K39,K47,K55,K63)</f>
         <v>245898.48</v>
       </c>
@@ -10490,35 +10508,37 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="86" t="s">
+      <c r="A22" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="87">
+      <c r="B22" s="17">
         <f>SUM(B7,B15)</f>
         <v>976</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="88">
+      <c r="C22" s="86"/>
+      <c r="D22" s="21">
         <f>SUM(D13,D21)</f>
         <v>12220</v>
       </c>
-      <c r="G22" s="87">
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17">
         <f>SUM(G7,G15)</f>
         <v>624</v>
       </c>
-      <c r="H22" s="87">
+      <c r="H22" s="17">
         <f>SUM(H7,H15)</f>
         <v>256</v>
       </c>
-      <c r="I22" s="87">
+      <c r="I22" s="17">
         <f>SUM(I7,I15)</f>
         <v>96</v>
       </c>
-      <c r="J22" s="87">
+      <c r="J22" s="17">
         <f>SUM(J7,J15)</f>
         <v>94</v>
       </c>
-      <c r="K22" s="88">
+      <c r="K22" s="21">
         <f>SUM(K7,K15)</f>
         <v>121667.84</v>
       </c>
@@ -12455,35 +12475,37 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="86" t="s">
+      <c r="A22" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="87">
+      <c r="B22" s="17">
         <f>SUM(B7,B15)</f>
         <v>6608</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="88">
+      <c r="C22" s="86"/>
+      <c r="D22" s="21">
         <f>SUM(D13,D21)</f>
         <v>29120</v>
       </c>
-      <c r="G22" s="87">
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17">
         <f>SUM(G7,G15)</f>
         <v>3616</v>
       </c>
-      <c r="H22" s="87">
+      <c r="H22" s="17">
         <f>SUM(H7,H15)</f>
         <v>2176</v>
       </c>
-      <c r="I22" s="87">
+      <c r="I22" s="17">
         <f>SUM(I7,I15)</f>
         <v>816</v>
       </c>
-      <c r="J22" s="87">
+      <c r="J22" s="17">
         <f>SUM(J7,J15)</f>
         <v>224</v>
       </c>
-      <c r="K22" s="88">
+      <c r="K22" s="21">
         <f>SUM(K7,K15)</f>
         <v>806255.52</v>
       </c>
@@ -14420,35 +14442,37 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="86" t="s">
+      <c r="A22" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="B22" s="87">
+      <c r="B22" s="17">
         <f>SUM(B7,B15)</f>
         <v>448</v>
       </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="88">
+      <c r="C22" s="86"/>
+      <c r="D22" s="21">
         <f>SUM(D13,D21)</f>
         <v>5460</v>
       </c>
-      <c r="G22" s="87">
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="17">
         <f>SUM(G7,G15)</f>
         <v>272</v>
       </c>
-      <c r="H22" s="87">
+      <c r="H22" s="17">
         <f>SUM(H7,H15)</f>
         <v>128</v>
       </c>
-      <c r="I22" s="87">
+      <c r="I22" s="17">
         <f>SUM(I7,I15)</f>
         <v>48</v>
       </c>
-      <c r="J22" s="87">
+      <c r="J22" s="17">
         <f>SUM(J7,J15)</f>
         <v>42</v>
       </c>
-      <c r="K22" s="88">
+      <c r="K22" s="21">
         <f>SUM(K7,K15)</f>
         <v>58500.31999999999</v>
       </c>
@@ -14513,150 +14537,185 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="87"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+      <c r="G4" s="87"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="87"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+      <c r="G5" s="87"/>
+    </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="G6" s="24" t="s">
+      <c r="G6" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="88" t="s">
         <v>67</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="89" t="s">
         <v>68</v>
       </c>
-      <c r="C7" s="89">
+      <c r="C7" s="90">
         <v>5</v>
       </c>
-      <c r="D7" s="89">
+      <c r="D7" s="90">
         <v>3</v>
       </c>
-      <c r="E7" s="90">
+      <c r="E7" s="69">
         <v>4464</v>
       </c>
-      <c r="F7" s="90">
-        <v>0</v>
-      </c>
-      <c r="G7" s="90">
+      <c r="F7" s="69">
+        <v>0</v>
+      </c>
+      <c r="G7" s="69">
         <f>C7*D7*E7+F7</f>
         <v>66960</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="91" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="92" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="89">
+      <c r="C8" s="93">
         <v>3</v>
       </c>
-      <c r="D8" s="89">
-        <v>2</v>
-      </c>
-      <c r="E8" s="90">
+      <c r="D8" s="93">
+        <v>2</v>
+      </c>
+      <c r="E8" s="58">
         <v>612</v>
       </c>
-      <c r="F8" s="90">
-        <v>0</v>
-      </c>
-      <c r="G8" s="90">
+      <c r="F8" s="58">
+        <v>0</v>
+      </c>
+      <c r="G8" s="58">
         <f>C8*D8*E8+F8</f>
         <v>3672</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="88" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="89" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="89">
+      <c r="C9" s="90">
         <v>3</v>
       </c>
-      <c r="D9" s="89">
-        <v>2</v>
-      </c>
-      <c r="E9" s="90">
+      <c r="D9" s="90">
+        <v>2</v>
+      </c>
+      <c r="E9" s="69">
         <v>936</v>
       </c>
-      <c r="F9" s="90">
-        <v>0</v>
-      </c>
-      <c r="G9" s="90">
+      <c r="F9" s="69">
+        <v>0</v>
+      </c>
+      <c r="G9" s="69">
         <f>C9*D9*E9+F9</f>
         <v>5616</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="91" t="s">
         <v>71</v>
       </c>
-      <c r="B10" s="39" t="s">
+      <c r="B10" s="92" t="s">
         <v>72</v>
       </c>
-      <c r="C10" s="89">
-        <v>1</v>
-      </c>
-      <c r="D10" s="89">
+      <c r="C10" s="93">
+        <v>1</v>
+      </c>
+      <c r="D10" s="93">
         <v>32</v>
       </c>
-      <c r="E10" s="90">
+      <c r="E10" s="58">
         <v>1160</v>
       </c>
-      <c r="F10" s="90">
-        <v>0</v>
-      </c>
-      <c r="G10" s="90">
+      <c r="F10" s="58">
+        <v>0</v>
+      </c>
+      <c r="G10" s="58">
         <f>C10*D10*E10+F10</f>
         <v>37120</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="86" t="s">
+      <c r="A11" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="88">
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="21">
         <f>SUM(G7:G10)</f>
         <v>113368</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
@@ -14693,66 +14752,91 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="87"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="87"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+    </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="88" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="89">
+      <c r="B7" s="90">
         <v>6</v>
       </c>
-      <c r="C7" s="89">
+      <c r="C7" s="90">
         <v>1500</v>
       </c>
-      <c r="D7" s="90">
+      <c r="D7" s="69">
         <v>0.76</v>
       </c>
-      <c r="E7" s="90">
+      <c r="E7" s="69">
         <f>B7*C7*D7</f>
         <v>6840</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="86" t="s">
+      <c r="A8" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="88">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="21">
         <f>SUM(E7:E7)</f>
         <v>6840</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
@@ -14789,102 +14873,127 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="87"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="87"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+    </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="88" t="s">
         <v>80</v>
       </c>
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="89" t="s">
         <v>81</v>
       </c>
-      <c r="C7" s="89">
+      <c r="C7" s="90">
         <v>3.5</v>
       </c>
-      <c r="D7" s="90">
+      <c r="D7" s="69">
         <v>1000</v>
       </c>
-      <c r="E7" s="90">
+      <c r="E7" s="69">
         <f>C7*D7</f>
         <v>3500</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="91" t="s">
         <v>82</v>
       </c>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="92" t="s">
         <v>83</v>
       </c>
-      <c r="C8" s="89">
-        <v>1</v>
-      </c>
-      <c r="D8" s="90">
+      <c r="C8" s="93">
+        <v>1</v>
+      </c>
+      <c r="D8" s="58">
         <v>1200</v>
       </c>
-      <c r="E8" s="90">
+      <c r="E8" s="58">
         <f>C8*D8</f>
         <v>1200</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="88" t="s">
         <v>84</v>
       </c>
-      <c r="B9" s="39" t="s">
+      <c r="B9" s="89" t="s">
         <v>85</v>
       </c>
-      <c r="C9" s="89">
-        <v>1</v>
-      </c>
-      <c r="D9" s="90">
+      <c r="C9" s="90">
+        <v>1</v>
+      </c>
+      <c r="D9" s="69">
         <v>6000</v>
       </c>
-      <c r="E9" s="90">
+      <c r="E9" s="69">
         <f>C9*D9</f>
         <v>6000</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="86" t="s">
+      <c r="A10" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="88">
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="21">
         <f>SUM(E7:E9)</f>
         <v>10700</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
@@ -14921,176 +15030,208 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="87"/>
+      <c r="B4" s="87"/>
+      <c r="C4" s="87"/>
+      <c r="D4" s="87"/>
+      <c r="E4" s="87"/>
+      <c r="F4" s="87"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="87"/>
+      <c r="B5" s="87"/>
+      <c r="C5" s="87"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+    </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="4" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="88" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="90">
+      <c r="B7" s="69">
+        <v>57.9</v>
+      </c>
+      <c r="C7" s="69">
         <v>111.67</v>
       </c>
-      <c r="D7" s="90">
+      <c r="D7" s="69">
         <v>156.21</v>
       </c>
-      <c r="E7" s="90">
+      <c r="E7" s="69">
         <v>200.75</v>
       </c>
-      <c r="F7" s="90">
+      <c r="F7" s="69">
         <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="91" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="90">
+      <c r="B8" s="58">
         <v>64</v>
       </c>
-      <c r="C8" s="90">
+      <c r="C8" s="58">
         <v>105.76</v>
       </c>
-      <c r="D8" s="90">
+      <c r="D8" s="58">
         <v>143.77</v>
       </c>
-      <c r="E8" s="90">
+      <c r="E8" s="58">
         <v>181.79</v>
       </c>
-      <c r="F8" s="90">
+      <c r="F8" s="58">
         <v>140</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="39" t="s">
+      <c r="A9" s="88" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="90">
+      <c r="B9" s="69">
         <v>52.5</v>
       </c>
-      <c r="C9" s="90">
+      <c r="C9" s="69">
         <v>91.02</v>
       </c>
-      <c r="D9" s="90">
+      <c r="D9" s="69">
         <v>122.2</v>
       </c>
-      <c r="E9" s="90">
+      <c r="E9" s="69">
         <v>153.39</v>
       </c>
-      <c r="F9" s="90">
+      <c r="F9" s="69">
         <v>140</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="39" t="s">
+      <c r="A10" s="91" t="s">
         <v>47</v>
       </c>
-      <c r="B10" s="90">
+      <c r="B10" s="58">
         <v>58.84</v>
       </c>
-      <c r="C10" s="90">
+      <c r="C10" s="58">
         <v>111.22</v>
       </c>
-      <c r="D10" s="90">
+      <c r="D10" s="58">
         <v>156.31</v>
       </c>
-      <c r="E10" s="90">
+      <c r="E10" s="58">
         <v>201.4</v>
       </c>
-      <c r="F10" s="90">
+      <c r="F10" s="58">
         <v>140</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="39" t="s">
+      <c r="A11" s="88" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="90">
+      <c r="B11" s="69">
+        <v>53.93</v>
+      </c>
+      <c r="C11" s="69">
         <v>105.28</v>
       </c>
-      <c r="D11" s="90">
+      <c r="D11" s="69">
         <v>147.5</v>
       </c>
-      <c r="E11" s="90">
+      <c r="E11" s="69">
         <v>189.72</v>
       </c>
-      <c r="F11" s="90">
+      <c r="F11" s="69">
         <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="91" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="90">
+      <c r="B12" s="58">
         <v>49.03</v>
       </c>
-      <c r="C12" s="90">
+      <c r="C12" s="58">
         <v>99.33</v>
       </c>
-      <c r="D12" s="90">
+      <c r="D12" s="58">
         <v>138.69</v>
       </c>
-      <c r="E12" s="90">
+      <c r="E12" s="58">
         <v>178.05</v>
       </c>
-      <c r="F12" s="90">
+      <c r="F12" s="58">
         <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="39" t="s">
+      <c r="A13" s="88" t="s">
         <v>92</v>
       </c>
-      <c r="B13" s="90">
+      <c r="B13" s="69">
         <v>45.6</v>
       </c>
-      <c r="C13" s="90">
+      <c r="C13" s="69">
         <v>108.38</v>
       </c>
-      <c r="D13" s="90">
+      <c r="D13" s="69">
         <v>152.78</v>
       </c>
-      <c r="E13" s="90">
+      <c r="E13" s="69">
         <v>197.19</v>
       </c>
-      <c r="F13" s="90">
+      <c r="F13" s="69">
         <v>130</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>

</xml_diff>

<commit_message>
Regenerate Look samples with Large tools and rental Rate Tables
Aromatics and CAT 2 exports now include live COE dry/wet rates and
third-party rental catalogs on Rate Tables. Desk totals unchanged.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -34,7 +34,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Staff Travel Cost'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'Misc Costs'!$A1:$E10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Misc Costs'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'Rate Tables'!$A1:$F13</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'Rate Tables'!$A1:$F20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Rate Tables'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="100">
   <si>
     <t>HIT SQUAD / PROJECT CONTROLS</t>
   </si>
@@ -318,6 +318,30 @@
   </si>
   <si>
     <t>Boilermaker Journeyman</t>
+  </si>
+  <si>
+    <t>Large tools (COE / dry rates)</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Daily $</t>
+  </si>
+  <si>
+    <t>Weekly $</t>
+  </si>
+  <si>
+    <t>Monthly $</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Dry</t>
+  </si>
+  <si>
+    <t>Wet</t>
   </si>
 </sst>
 </file>
@@ -718,7 +742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -878,6 +902,9 @@
     <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
     <xf numFmtId="3" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14534,25 +14561,25 @@
       <c r="G5" s="82"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="24" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="24" t="s">
         <v>65</v>
       </c>
     </row>
@@ -14741,19 +14768,19 @@
       <c r="E5" s="82"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="24" t="s">
         <v>65</v>
       </c>
     </row>
@@ -14862,19 +14889,19 @@
       <c r="E5" s="82"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="24" t="s">
         <v>65</v>
       </c>
     </row>
@@ -14969,7 +14996,7 @@
     <tabColor rgb="FF083943"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -15023,22 +15050,22 @@
       <c r="F5" s="82"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F6" s="24" t="s">
         <v>90</v>
       </c>
     </row>
@@ -15182,12 +15209,123 @@
         <v>130</v>
       </c>
     </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="89"/>
+      <c r="B14" s="90"/>
+      <c r="C14" s="90"/>
+      <c r="D14" s="90"/>
+      <c r="E14" s="90"/>
+      <c r="F14" s="90"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="11"/>
+      <c r="C15" s="11"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="F16" s="24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="83" t="s">
+        <v>66</v>
+      </c>
+      <c r="B17" s="84" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" s="64">
+        <v>496</v>
+      </c>
+      <c r="D17" s="64">
+        <v>1488</v>
+      </c>
+      <c r="E17" s="64">
+        <v>4464</v>
+      </c>
+      <c r="F17" s="91"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="86" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18" s="87" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" s="53">
+        <v>68</v>
+      </c>
+      <c r="D18" s="53">
+        <v>204</v>
+      </c>
+      <c r="E18" s="53">
+        <v>612</v>
+      </c>
+      <c r="F18" s="90"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="83" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" s="84" t="s">
+        <v>98</v>
+      </c>
+      <c r="C19" s="64">
+        <v>104</v>
+      </c>
+      <c r="D19" s="64">
+        <v>312</v>
+      </c>
+      <c r="E19" s="64">
+        <v>936</v>
+      </c>
+      <c r="F19" s="91"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="86" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="87" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="53">
+        <v>1160</v>
+      </c>
+      <c r="D20" s="53">
+        <v>3480</v>
+      </c>
+      <c r="E20" s="53">
+        <v>10440</v>
+      </c>
+      <c r="F20" s="90"/>
+    </row>
   </sheetData>
   <sheetProtection sheet="1"/>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>

</xml_diff>

<commit_message>
Regenerate Look samples with wrapped Summary header rows
Aromatics and CAT 2 Summary subtitles now wrap so East Coast COMP
and the produced line stay fully readable. Desk totals unchanged.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -748,10 +748,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1390,14 +1390,14 @@
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" ht="28" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -14520,7 +14520,7 @@
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -14531,7 +14531,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -14735,7 +14735,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -14744,7 +14744,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -14856,7 +14856,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -14865,7 +14865,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -15013,7 +15013,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -15023,7 +15023,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
Regenerate Look samples with even Hours/shift row height
HPS no longer wraps or doubles row height. Desk totals unchanged.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -140,7 +140,7 @@
     <t>HC</t>
   </si>
   <si>
-    <t>Enter Hours Per shift Here</t>
+    <t>Hours/shift</t>
   </si>
   <si>
     <t>HPS</t>
@@ -839,7 +839,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -872,7 +874,7 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1671,7 +1673,7 @@
   <dimension ref="A1:OV70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" style="22" customWidth="1"/>
     <col min="3" max="3" width="24" style="23" customWidth="1"/>
     <col min="4" max="4" width="14" style="22" customWidth="1"/>
@@ -2174,7 +2176,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
         <v>32</v>
       </c>
@@ -3013,7 +3015,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
         <v>32</v>
       </c>
@@ -3852,7 +3854,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="25" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A25" s="52" t="s">
         <v>32</v>
       </c>
@@ -4691,7 +4693,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A33" s="52" t="s">
         <v>32</v>
       </c>
@@ -5530,7 +5532,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A41" s="52" t="s">
         <v>32</v>
       </c>
@@ -6369,7 +6371,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="49" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A49" s="52" t="s">
         <v>32</v>
       </c>
@@ -7208,7 +7210,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="57" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A57" s="52" t="s">
         <v>32</v>
       </c>
@@ -8047,7 +8049,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="65" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A65" s="52" t="s">
         <v>32</v>
       </c>
@@ -8794,7 +8796,7 @@
   <dimension ref="A1:OV22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" style="22" customWidth="1"/>
     <col min="3" max="3" width="24" style="23" customWidth="1"/>
     <col min="4" max="4" width="14" style="22" customWidth="1"/>
@@ -9297,7 +9299,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
         <v>32</v>
       </c>
@@ -10136,7 +10138,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
         <v>32</v>
       </c>
@@ -10853,7 +10855,7 @@
   <dimension ref="A1:OV22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" style="22" customWidth="1"/>
     <col min="3" max="3" width="24" style="23" customWidth="1"/>
     <col min="4" max="4" width="14" style="22" customWidth="1"/>
@@ -11356,7 +11358,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
         <v>32</v>
       </c>
@@ -12195,7 +12197,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
         <v>32</v>
       </c>
@@ -12912,7 +12914,7 @@
   <dimension ref="A1:OV22"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="13" style="22" customWidth="1"/>
     <col min="3" max="3" width="24" style="23" customWidth="1"/>
     <col min="4" max="4" width="14" style="22" customWidth="1"/>
@@ -13415,7 +13417,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
         <v>32</v>
       </c>
@@ -14254,7 +14256,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" ht="28" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A17" s="52" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
Regenerate Look samples with full-width labor subtitle bands
Staff / Foremen / Direct / Support now merge and plate-wash rows 2–3 through the last day column. Desk and Excel ESTIMATE TOTAL $ stay $25,324,671.97 (Aromatics) and $1,435,365.66 (CAT 2).

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -1742,38 +1742,38 @@
       <c r="I2" s="25"/>
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
-      <c r="Z2" s="22"/>
-      <c r="AA2" s="22"/>
-      <c r="AB2" s="22"/>
-      <c r="AC2" s="22"/>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
-      <c r="AJ2" s="22"/>
-      <c r="AK2" s="22"/>
-      <c r="AL2" s="22"/>
-      <c r="AM2" s="22"/>
-      <c r="AN2" s="22"/>
-      <c r="AO2" s="22"/>
-      <c r="AP2" s="22"/>
-      <c r="AQ2" s="22"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="25"/>
+      <c r="T2" s="25"/>
+      <c r="U2" s="25"/>
+      <c r="V2" s="25"/>
+      <c r="W2" s="25"/>
+      <c r="X2" s="25"/>
+      <c r="Y2" s="25"/>
+      <c r="Z2" s="25"/>
+      <c r="AA2" s="25"/>
+      <c r="AB2" s="25"/>
+      <c r="AC2" s="25"/>
+      <c r="AD2" s="25"/>
+      <c r="AE2" s="25"/>
+      <c r="AF2" s="25"/>
+      <c r="AG2" s="25"/>
+      <c r="AH2" s="25"/>
+      <c r="AI2" s="25"/>
+      <c r="AJ2" s="25"/>
+      <c r="AK2" s="25"/>
+      <c r="AL2" s="25"/>
+      <c r="AM2" s="25"/>
+      <c r="AN2" s="25"/>
+      <c r="AO2" s="25"/>
+      <c r="AP2" s="25"/>
+      <c r="AQ2" s="25"/>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
@@ -1789,38 +1789,38 @@
       <c r="I3" s="26"/>
       <c r="J3" s="26"/>
       <c r="K3" s="26"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="22"/>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="22"/>
-      <c r="AC3" s="22"/>
-      <c r="AD3" s="22"/>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="22"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
-      <c r="AJ3" s="22"/>
-      <c r="AK3" s="22"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="22"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26"/>
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="26"/>
+      <c r="AC3" s="26"/>
+      <c r="AD3" s="26"/>
+      <c r="AE3" s="26"/>
+      <c r="AF3" s="26"/>
+      <c r="AG3" s="26"/>
+      <c r="AH3" s="26"/>
+      <c r="AI3" s="26"/>
+      <c r="AJ3" s="26"/>
+      <c r="AK3" s="26"/>
+      <c r="AL3" s="26"/>
+      <c r="AM3" s="26"/>
+      <c r="AN3" s="26"/>
+      <c r="AO3" s="26"/>
+      <c r="AP3" s="26"/>
+      <c r="AQ3" s="26"/>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -8725,8 +8725,8 @@
   <sheetProtection sheet="1"/>
   <mergeCells count="3">
     <mergeCell ref="A1:AQ1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A2:AQ2"/>
+    <mergeCell ref="A3:AQ3"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:AQ6">
     <cfRule type="expression" dxfId="8" priority="1">
@@ -8865,38 +8865,38 @@
       <c r="I2" s="25"/>
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
-      <c r="Z2" s="22"/>
-      <c r="AA2" s="22"/>
-      <c r="AB2" s="22"/>
-      <c r="AC2" s="22"/>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
-      <c r="AJ2" s="22"/>
-      <c r="AK2" s="22"/>
-      <c r="AL2" s="22"/>
-      <c r="AM2" s="22"/>
-      <c r="AN2" s="22"/>
-      <c r="AO2" s="22"/>
-      <c r="AP2" s="22"/>
-      <c r="AQ2" s="22"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="25"/>
+      <c r="T2" s="25"/>
+      <c r="U2" s="25"/>
+      <c r="V2" s="25"/>
+      <c r="W2" s="25"/>
+      <c r="X2" s="25"/>
+      <c r="Y2" s="25"/>
+      <c r="Z2" s="25"/>
+      <c r="AA2" s="25"/>
+      <c r="AB2" s="25"/>
+      <c r="AC2" s="25"/>
+      <c r="AD2" s="25"/>
+      <c r="AE2" s="25"/>
+      <c r="AF2" s="25"/>
+      <c r="AG2" s="25"/>
+      <c r="AH2" s="25"/>
+      <c r="AI2" s="25"/>
+      <c r="AJ2" s="25"/>
+      <c r="AK2" s="25"/>
+      <c r="AL2" s="25"/>
+      <c r="AM2" s="25"/>
+      <c r="AN2" s="25"/>
+      <c r="AO2" s="25"/>
+      <c r="AP2" s="25"/>
+      <c r="AQ2" s="25"/>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
@@ -8912,38 +8912,38 @@
       <c r="I3" s="26"/>
       <c r="J3" s="26"/>
       <c r="K3" s="26"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="22"/>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="22"/>
-      <c r="AC3" s="22"/>
-      <c r="AD3" s="22"/>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="22"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
-      <c r="AJ3" s="22"/>
-      <c r="AK3" s="22"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="22"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26"/>
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="26"/>
+      <c r="AC3" s="26"/>
+      <c r="AD3" s="26"/>
+      <c r="AE3" s="26"/>
+      <c r="AF3" s="26"/>
+      <c r="AG3" s="26"/>
+      <c r="AH3" s="26"/>
+      <c r="AI3" s="26"/>
+      <c r="AJ3" s="26"/>
+      <c r="AK3" s="26"/>
+      <c r="AL3" s="26"/>
+      <c r="AM3" s="26"/>
+      <c r="AN3" s="26"/>
+      <c r="AO3" s="26"/>
+      <c r="AP3" s="26"/>
+      <c r="AQ3" s="26"/>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -10814,8 +10814,8 @@
   <sheetProtection sheet="1"/>
   <mergeCells count="3">
     <mergeCell ref="A1:AQ1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A2:AQ2"/>
+    <mergeCell ref="A3:AQ3"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:AQ6">
     <cfRule type="expression" dxfId="11" priority="1">
@@ -10924,38 +10924,38 @@
       <c r="I2" s="25"/>
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
-      <c r="Z2" s="22"/>
-      <c r="AA2" s="22"/>
-      <c r="AB2" s="22"/>
-      <c r="AC2" s="22"/>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
-      <c r="AJ2" s="22"/>
-      <c r="AK2" s="22"/>
-      <c r="AL2" s="22"/>
-      <c r="AM2" s="22"/>
-      <c r="AN2" s="22"/>
-      <c r="AO2" s="22"/>
-      <c r="AP2" s="22"/>
-      <c r="AQ2" s="22"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="25"/>
+      <c r="T2" s="25"/>
+      <c r="U2" s="25"/>
+      <c r="V2" s="25"/>
+      <c r="W2" s="25"/>
+      <c r="X2" s="25"/>
+      <c r="Y2" s="25"/>
+      <c r="Z2" s="25"/>
+      <c r="AA2" s="25"/>
+      <c r="AB2" s="25"/>
+      <c r="AC2" s="25"/>
+      <c r="AD2" s="25"/>
+      <c r="AE2" s="25"/>
+      <c r="AF2" s="25"/>
+      <c r="AG2" s="25"/>
+      <c r="AH2" s="25"/>
+      <c r="AI2" s="25"/>
+      <c r="AJ2" s="25"/>
+      <c r="AK2" s="25"/>
+      <c r="AL2" s="25"/>
+      <c r="AM2" s="25"/>
+      <c r="AN2" s="25"/>
+      <c r="AO2" s="25"/>
+      <c r="AP2" s="25"/>
+      <c r="AQ2" s="25"/>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
@@ -10971,38 +10971,38 @@
       <c r="I3" s="26"/>
       <c r="J3" s="26"/>
       <c r="K3" s="26"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="22"/>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="22"/>
-      <c r="AC3" s="22"/>
-      <c r="AD3" s="22"/>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="22"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
-      <c r="AJ3" s="22"/>
-      <c r="AK3" s="22"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="22"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26"/>
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="26"/>
+      <c r="AC3" s="26"/>
+      <c r="AD3" s="26"/>
+      <c r="AE3" s="26"/>
+      <c r="AF3" s="26"/>
+      <c r="AG3" s="26"/>
+      <c r="AH3" s="26"/>
+      <c r="AI3" s="26"/>
+      <c r="AJ3" s="26"/>
+      <c r="AK3" s="26"/>
+      <c r="AL3" s="26"/>
+      <c r="AM3" s="26"/>
+      <c r="AN3" s="26"/>
+      <c r="AO3" s="26"/>
+      <c r="AP3" s="26"/>
+      <c r="AQ3" s="26"/>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12873,8 +12873,8 @@
   <sheetProtection sheet="1"/>
   <mergeCells count="3">
     <mergeCell ref="A1:AQ1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A2:AQ2"/>
+    <mergeCell ref="A3:AQ3"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:AQ6">
     <cfRule type="expression" dxfId="14" priority="1">
@@ -12983,38 +12983,38 @@
       <c r="I2" s="25"/>
       <c r="J2" s="25"/>
       <c r="K2" s="25"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="22"/>
-      <c r="P2" s="22"/>
-      <c r="Q2" s="22"/>
-      <c r="R2" s="22"/>
-      <c r="S2" s="22"/>
-      <c r="T2" s="22"/>
-      <c r="U2" s="22"/>
-      <c r="V2" s="22"/>
-      <c r="W2" s="22"/>
-      <c r="X2" s="22"/>
-      <c r="Y2" s="22"/>
-      <c r="Z2" s="22"/>
-      <c r="AA2" s="22"/>
-      <c r="AB2" s="22"/>
-      <c r="AC2" s="22"/>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
-      <c r="AJ2" s="22"/>
-      <c r="AK2" s="22"/>
-      <c r="AL2" s="22"/>
-      <c r="AM2" s="22"/>
-      <c r="AN2" s="22"/>
-      <c r="AO2" s="22"/>
-      <c r="AP2" s="22"/>
-      <c r="AQ2" s="22"/>
+      <c r="L2" s="25"/>
+      <c r="M2" s="25"/>
+      <c r="N2" s="25"/>
+      <c r="O2" s="25"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="25"/>
+      <c r="R2" s="25"/>
+      <c r="S2" s="25"/>
+      <c r="T2" s="25"/>
+      <c r="U2" s="25"/>
+      <c r="V2" s="25"/>
+      <c r="W2" s="25"/>
+      <c r="X2" s="25"/>
+      <c r="Y2" s="25"/>
+      <c r="Z2" s="25"/>
+      <c r="AA2" s="25"/>
+      <c r="AB2" s="25"/>
+      <c r="AC2" s="25"/>
+      <c r="AD2" s="25"/>
+      <c r="AE2" s="25"/>
+      <c r="AF2" s="25"/>
+      <c r="AG2" s="25"/>
+      <c r="AH2" s="25"/>
+      <c r="AI2" s="25"/>
+      <c r="AJ2" s="25"/>
+      <c r="AK2" s="25"/>
+      <c r="AL2" s="25"/>
+      <c r="AM2" s="25"/>
+      <c r="AN2" s="25"/>
+      <c r="AO2" s="25"/>
+      <c r="AP2" s="25"/>
+      <c r="AQ2" s="25"/>
     </row>
     <row r="3" ht="16" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
@@ -13030,38 +13030,38 @@
       <c r="I3" s="26"/>
       <c r="J3" s="26"/>
       <c r="K3" s="26"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="22"/>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="22"/>
-      <c r="R3" s="22"/>
-      <c r="S3" s="22"/>
-      <c r="T3" s="22"/>
-      <c r="U3" s="22"/>
-      <c r="V3" s="22"/>
-      <c r="W3" s="22"/>
-      <c r="X3" s="22"/>
-      <c r="Y3" s="22"/>
-      <c r="Z3" s="22"/>
-      <c r="AA3" s="22"/>
-      <c r="AB3" s="22"/>
-      <c r="AC3" s="22"/>
-      <c r="AD3" s="22"/>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="22"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
-      <c r="AJ3" s="22"/>
-      <c r="AK3" s="22"/>
-      <c r="AL3" s="22"/>
-      <c r="AM3" s="22"/>
-      <c r="AN3" s="22"/>
-      <c r="AO3" s="22"/>
-      <c r="AP3" s="22"/>
-      <c r="AQ3" s="22"/>
+      <c r="L3" s="26"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="26"/>
+      <c r="O3" s="26"/>
+      <c r="P3" s="26"/>
+      <c r="Q3" s="26"/>
+      <c r="R3" s="26"/>
+      <c r="S3" s="26"/>
+      <c r="T3" s="26"/>
+      <c r="U3" s="26"/>
+      <c r="V3" s="26"/>
+      <c r="W3" s="26"/>
+      <c r="X3" s="26"/>
+      <c r="Y3" s="26"/>
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="26"/>
+      <c r="AB3" s="26"/>
+      <c r="AC3" s="26"/>
+      <c r="AD3" s="26"/>
+      <c r="AE3" s="26"/>
+      <c r="AF3" s="26"/>
+      <c r="AG3" s="26"/>
+      <c r="AH3" s="26"/>
+      <c r="AI3" s="26"/>
+      <c r="AJ3" s="26"/>
+      <c r="AK3" s="26"/>
+      <c r="AL3" s="26"/>
+      <c r="AM3" s="26"/>
+      <c r="AN3" s="26"/>
+      <c r="AO3" s="26"/>
+      <c r="AP3" s="26"/>
+      <c r="AQ3" s="26"/>
     </row>
     <row r="4" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" ht="6" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -14932,8 +14932,8 @@
   <sheetProtection sheet="1"/>
   <mergeCells count="3">
     <mergeCell ref="A1:AQ1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A2:AQ2"/>
+    <mergeCell ref="A3:AQ3"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:AQ6">
     <cfRule type="expression" dxfId="17" priority="1">

</xml_diff>

<commit_message>
Regenerate Look samples with native A–K column outline.
Staff / Foremen / Direct / Support now ship the Excel +/− group.
Desk totals unchanged: Aromatics $25,324,671.97, CAT 2 $1,435,365.66.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -1715,21 +1715,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF0F5F6D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:OV70"/>
-  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="1" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9.01" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="2" max="2" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="32" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="16" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="14" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="9.01" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="16" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="3.2" customWidth="1"/>
     <col min="13" max="13" width="3.2" customWidth="1"/>
     <col min="14" max="14" width="3.2" customWidth="1"/>
@@ -8902,7 +8903,7 @@
       <c r="AQ70" s="84"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
+  <sheetProtection sheet="1" formatColumns="1"/>
   <mergeCells count="7">
     <mergeCell ref="A1:AQ1"/>
     <mergeCell ref="A2:AQ2"/>
@@ -8973,21 +8974,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF0F5F6D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:OV22"/>
-  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="1" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9.01" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="2" max="2" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="32" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="16" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="14" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="9.01" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="16" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="3.2" customWidth="1"/>
     <col min="13" max="13" width="3.2" customWidth="1"/>
     <col min="14" max="14" width="3.2" customWidth="1"/>
@@ -11126,7 +11128,7 @@
       <c r="AQ22" s="84"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
+  <sheetProtection sheet="1" formatColumns="1"/>
   <mergeCells count="7">
     <mergeCell ref="A1:AQ1"/>
     <mergeCell ref="A2:AQ2"/>
@@ -11167,21 +11169,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF0F5F6D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:OV22"/>
-  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="1" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9.01" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="2" max="2" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="32" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="16" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="14" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="9.01" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="16" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="3.2" customWidth="1"/>
     <col min="13" max="13" width="3.2" customWidth="1"/>
     <col min="14" max="14" width="3.2" customWidth="1"/>
@@ -13320,7 +13323,7 @@
       <c r="AQ22" s="84"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
+  <sheetProtection sheet="1" formatColumns="1"/>
   <mergeCells count="7">
     <mergeCell ref="A1:AQ1"/>
     <mergeCell ref="A2:AQ2"/>
@@ -13361,21 +13364,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF0F5F6D"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
   <dimension ref="A1:OV22"/>
-  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
+  <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="1" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="9.01" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
-    <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="10" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="2" max="2" width="11" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="32" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="16" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="14" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="9.01" customWidth="1" outlineLevel="1"/>
+    <col min="7" max="7" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="16" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="3.2" customWidth="1"/>
     <col min="13" max="13" width="3.2" customWidth="1"/>
     <col min="14" max="14" width="3.2" customWidth="1"/>
@@ -15514,7 +15518,7 @@
       <c r="AQ22" s="84"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1"/>
+  <sheetProtection sheet="1" formatColumns="1"/>
   <mergeCells count="7">
     <mergeCell ref="A1:AQ1"/>
     <mergeCell ref="A2:AQ2"/>

</xml_diff>

<commit_message>
Rebuild Look samples with Support Bill as on the position block.
Aromatics and CAT 2 Support rows show the live-pack billedAs craft next to Position. Desk and Excel totals stay $25,324,671.97 and $1,435,365.66.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="111">
   <si>
     <t>HIT SQUAD / PROJECT CONTROLS</t>
   </si>
@@ -248,6 +248,12 @@
     <t>sup-1787768630004-lgj97|day</t>
   </si>
   <si>
+    <t>Bill as</t>
+  </si>
+  <si>
+    <t>Boilermaker Journeyman</t>
+  </si>
+  <si>
     <t>sup-1787768630004-lgj97|night</t>
   </si>
   <si>
@@ -345,9 +351,6 @@
   </si>
   <si>
     <t>PD Rate</t>
-  </si>
-  <si>
-    <t>Boilermaker Journeyman</t>
   </si>
   <si>
     <t>Large tools (COE / dry rates)</t>
@@ -739,7 +742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -958,6 +961,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1"/>
@@ -14089,7 +14102,7 @@
         <f>G7+H7+I7</f>
         <v>280</v>
       </c>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="75" t="s">
         <v>66</v>
       </c>
       <c r="D7" s="37">
@@ -14157,7 +14170,7 @@
     <row r="8" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A8" s="46"/>
       <c r="B8" s="47"/>
-      <c r="C8" s="36"/>
+      <c r="C8" s="75"/>
       <c r="D8" s="47"/>
       <c r="E8" s="47"/>
       <c r="F8" s="48" t="s">
@@ -14273,7 +14286,7 @@
         <v>43</v>
       </c>
       <c r="B9" s="47"/>
-      <c r="C9" s="36"/>
+      <c r="C9" s="75"/>
       <c r="D9" s="47"/>
       <c r="E9" s="47"/>
       <c r="F9" s="48" t="s">
@@ -14390,7 +14403,9 @@
         <f>SUM(L10:AQ10)</f>
         <v>192</v>
       </c>
-      <c r="C10" s="36"/>
+      <c r="C10" s="76" t="s">
+        <v>68</v>
+      </c>
       <c r="D10" s="56">
         <f>B10*E10</f>
         <v>20808.96</v>
@@ -14513,7 +14528,9 @@
         <f>SUM(L11:AQ11)</f>
         <v>64</v>
       </c>
-      <c r="C11" s="36"/>
+      <c r="C11" s="77" t="s">
+        <v>69</v>
+      </c>
       <c r="D11" s="62">
         <f>B11*E11</f>
         <v>9777.92</v>
@@ -14636,7 +14653,7 @@
         <f>SUM(L12:AQ12)</f>
         <v>24</v>
       </c>
-      <c r="C12" s="36"/>
+      <c r="C12" s="77"/>
       <c r="D12" s="56">
         <f>B12*E12</f>
         <v>4732.5599999999995</v>
@@ -14759,7 +14776,7 @@
         <f>SUM(L13:AQ13)</f>
         <v>28</v>
       </c>
-      <c r="C13" s="36"/>
+      <c r="C13" s="77"/>
       <c r="D13" s="65">
         <f>B13*E13</f>
         <v>3640</v>
@@ -14928,7 +14945,7 @@
         <f>G15+H15+I15</f>
         <v>168</v>
       </c>
-      <c r="C15" s="36" t="s">
+      <c r="C15" s="75" t="s">
         <v>66</v>
       </c>
       <c r="D15" s="37">
@@ -14990,13 +15007,13 @@
       <c r="AP15" s="42"/>
       <c r="AQ15" s="44"/>
       <c r="OV15" s="45" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
       <c r="A16" s="46"/>
       <c r="B16" s="47"/>
-      <c r="C16" s="36"/>
+      <c r="C16" s="75"/>
       <c r="D16" s="47"/>
       <c r="E16" s="47"/>
       <c r="F16" s="48" t="s">
@@ -15104,7 +15121,7 @@
         <v>0</v>
       </c>
       <c r="OV16" s="53" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
@@ -15112,7 +15129,7 @@
         <v>43</v>
       </c>
       <c r="B17" s="47"/>
-      <c r="C17" s="36"/>
+      <c r="C17" s="75"/>
       <c r="D17" s="47"/>
       <c r="E17" s="47"/>
       <c r="F17" s="48" t="s">
@@ -15220,7 +15237,7 @@
         <v>0</v>
       </c>
       <c r="OV17" s="53" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
@@ -15229,7 +15246,9 @@
         <f>SUM(L18:AQ18)</f>
         <v>80</v>
       </c>
-      <c r="C18" s="36"/>
+      <c r="C18" s="76" t="s">
+        <v>68</v>
+      </c>
       <c r="D18" s="56">
         <f>B18*E18</f>
         <v>8670.4</v>
@@ -15343,7 +15362,7 @@
         <v>0</v>
       </c>
       <c r="OV18" s="45" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
@@ -15352,7 +15371,9 @@
         <f>SUM(L19:AQ19)</f>
         <v>64</v>
       </c>
-      <c r="C19" s="36"/>
+      <c r="C19" s="77" t="s">
+        <v>69</v>
+      </c>
       <c r="D19" s="62">
         <f>B19*E19</f>
         <v>9777.92</v>
@@ -15466,7 +15487,7 @@
         <v>0</v>
       </c>
       <c r="OV19" s="45" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
@@ -15475,7 +15496,7 @@
         <f>SUM(L20:AQ20)</f>
         <v>24</v>
       </c>
-      <c r="C20" s="36"/>
+      <c r="C20" s="77"/>
       <c r="D20" s="56">
         <f>B20*E20</f>
         <v>4732.5599999999995</v>
@@ -15589,7 +15610,7 @@
         <v>0</v>
       </c>
       <c r="OV20" s="45" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:412" x14ac:dyDescent="0.25">
@@ -15598,7 +15619,7 @@
         <f>SUM(L21:AQ21)</f>
         <v>14</v>
       </c>
-      <c r="C21" s="36"/>
+      <c r="C21" s="77"/>
       <c r="D21" s="65">
         <f>B21*E21</f>
         <v>1820</v>
@@ -15711,7 +15732,7 @@
         <v>0</v>
       </c>
       <c r="OV21" s="53" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:43" x14ac:dyDescent="0.25">
@@ -15784,7 +15805,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" formatColumns="1"/>
-  <mergeCells count="19">
+  <mergeCells count="21">
     <mergeCell ref="A1:AQ1"/>
     <mergeCell ref="A2:AQ2"/>
     <mergeCell ref="A3:AQ3"/>
@@ -15792,18 +15813,20 @@
     <mergeCell ref="L4:U4"/>
     <mergeCell ref="V4:AI4"/>
     <mergeCell ref="AJ4:AQ4"/>
-    <mergeCell ref="C7:C13"/>
+    <mergeCell ref="C7:C9"/>
     <mergeCell ref="G7:G13"/>
     <mergeCell ref="H7:H13"/>
     <mergeCell ref="I7:I13"/>
     <mergeCell ref="J7:J13"/>
     <mergeCell ref="K7:K13"/>
-    <mergeCell ref="C15:C21"/>
+    <mergeCell ref="C11:C13"/>
+    <mergeCell ref="C15:C17"/>
     <mergeCell ref="G15:G21"/>
     <mergeCell ref="H15:H21"/>
     <mergeCell ref="I15:I21"/>
     <mergeCell ref="J15:J21"/>
     <mergeCell ref="K15:K21"/>
+    <mergeCell ref="C19:C21"/>
   </mergeCells>
   <conditionalFormatting sqref="L6:AQ6">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -15882,52 +15905,52 @@
       <c r="G3" s="3"/>
     </row>
     <row r="4" ht="6" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
+      <c r="G4" s="78"/>
     </row>
     <row r="5" ht="6" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="75"/>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
+      <c r="A5" s="78"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="78"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="78"/>
+      <c r="F5" s="78"/>
+      <c r="G5" s="78"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C7" s="8">
         <v>5</v>
@@ -15947,11 +15970,11 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="76" t="s">
-        <v>78</v>
+      <c r="A8" s="79" t="s">
+        <v>80</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C8" s="11">
         <v>3</v>
@@ -15972,10 +15995,10 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="C9" s="8">
         <v>3</v>
@@ -15995,11 +16018,11 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="76" t="s">
-        <v>80</v>
+      <c r="A10" s="79" t="s">
+        <v>82</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C10" s="11">
         <v>1</v>
@@ -16094,39 +16117,39 @@
       <c r="E3" s="3"/>
     </row>
     <row r="4" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
     </row>
     <row r="5" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="75"/>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
+      <c r="A5" s="78"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="78"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="78"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B7" s="8">
         <v>6</v>
@@ -16216,42 +16239,42 @@
       <c r="E3" s="3"/>
     </row>
     <row r="4" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
     </row>
     <row r="5" ht="6" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="75"/>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
+      <c r="A5" s="78"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="78"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="78"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C7" s="8">
         <v>3.5</v>
@@ -16265,11 +16288,11 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="76" t="s">
-        <v>91</v>
+      <c r="A8" s="79" t="s">
+        <v>93</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C8" s="11">
         <v>1</v>
@@ -16284,10 +16307,10 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C9" s="8">
         <v>1</v>
@@ -16376,39 +16399,39 @@
       <c r="F3" s="3"/>
     </row>
     <row r="4" ht="6" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="75"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
+      <c r="A4" s="78"/>
+      <c r="B4" s="78"/>
+      <c r="C4" s="78"/>
+      <c r="D4" s="78"/>
+      <c r="E4" s="78"/>
+      <c r="F4" s="78"/>
     </row>
     <row r="5" ht="6" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="75"/>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
+      <c r="A5" s="78"/>
+      <c r="B5" s="78"/>
+      <c r="C5" s="78"/>
+      <c r="D5" s="78"/>
+      <c r="E5" s="78"/>
+      <c r="F5" s="78"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B6" s="31" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E6" s="31" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F6" s="31" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -16432,7 +16455,7 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="76" t="s">
+      <c r="A8" s="79" t="s">
         <v>50</v>
       </c>
       <c r="B8" s="56">
@@ -16472,7 +16495,7 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="76" t="s">
+      <c r="A10" s="79" t="s">
         <v>56</v>
       </c>
       <c r="B10" s="56">
@@ -16512,7 +16535,7 @@
       </c>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="76" t="s">
+      <c r="A12" s="79" t="s">
         <v>63</v>
       </c>
       <c r="B12" s="56">
@@ -16533,7 +16556,7 @@
     </row>
     <row r="13" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="B13" s="62">
         <v>45.6</v>
@@ -16552,7 +16575,7 @@
       </c>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="77"/>
+      <c r="A14" s="80"/>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -16560,41 +16583,41 @@
       <c r="F14" s="15"/>
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="78" t="s">
-        <v>102</v>
-      </c>
-      <c r="B15" s="78"/>
-      <c r="C15" s="78"/>
-      <c r="D15" s="78"/>
-      <c r="E15" s="78"/>
-      <c r="F15" s="78"/>
+      <c r="A15" s="81" t="s">
+        <v>103</v>
+      </c>
+      <c r="B15" s="81"/>
+      <c r="C15" s="81"/>
+      <c r="D15" s="81"/>
+      <c r="E15" s="81"/>
+      <c r="F15" s="81"/>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="31" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B16" s="31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" s="31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D16" s="31" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E16" s="31" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F16" s="31" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" s="62">
         <v>496</v>
@@ -16605,14 +16628,14 @@
       <c r="E17" s="62">
         <v>4464</v>
       </c>
-      <c r="F17" s="79"/>
+      <c r="F17" s="82"/>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="76" t="s">
-        <v>78</v>
+      <c r="A18" s="79" t="s">
+        <v>80</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C18" s="56">
         <v>68</v>
@@ -16627,10 +16650,10 @@
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C19" s="62">
         <v>104</v>
@@ -16641,14 +16664,14 @@
       <c r="E19" s="62">
         <v>936</v>
       </c>
-      <c r="F19" s="79"/>
+      <c r="F19" s="82"/>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="76" t="s">
-        <v>80</v>
+      <c r="A20" s="79" t="s">
+        <v>82</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C20" s="56">
         <v>1160</v>

</xml_diff>

<commit_message>
Unlock Misc, Travel, and Equipment input cells for offline edits.
Estimator text, qty, and rate cells stay editable on a protected sheet; formula totals stay locked. Re-apply unlocks after chrome so Excel does not treat those inputs as locked.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -1295,7 +1295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
@@ -1525,8 +1525,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -5397,7 +5403,7 @@
       </c>
     </row>
     <row r="162" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A162" s="80"/>
+      <c r="A162" s="82"/>
       <c r="B162" s="15"/>
       <c r="C162" s="15"/>
       <c r="D162" s="15"/>
@@ -5405,14 +5411,14 @@
       <c r="F162" s="15"/>
     </row>
     <row r="163" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A163" s="81" t="s">
+      <c r="A163" s="83" t="s">
         <v>266</v>
       </c>
-      <c r="B163" s="81"/>
-      <c r="C163" s="81"/>
-      <c r="D163" s="81"/>
-      <c r="E163" s="81"/>
-      <c r="F163" s="81"/>
+      <c r="B163" s="83"/>
+      <c r="C163" s="83"/>
+      <c r="D163" s="83"/>
+      <c r="E163" s="83"/>
+      <c r="F163" s="83"/>
     </row>
     <row r="164" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A164" s="24" t="s">
@@ -5450,7 +5456,7 @@
       <c r="E165" s="64">
         <v>4464</v>
       </c>
-      <c r="F165" s="82"/>
+      <c r="F165" s="84"/>
     </row>
     <row r="166" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A166" s="29" t="s">
@@ -5486,7 +5492,7 @@
       <c r="E167" s="64">
         <v>936</v>
       </c>
-      <c r="F167" s="82"/>
+      <c r="F167" s="84"/>
     </row>
     <row r="168" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A168" s="29" t="s">
@@ -5600,50 +5606,50 @@
       <c r="H3" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="I3" s="83"/>
+      <c r="I3" s="85"/>
     </row>
     <row r="4" ht="6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4" s="84" t="s">
+      <c r="A4" s="86" t="s">
         <v>121</v>
       </c>
-      <c r="B4" s="84" t="s">
+      <c r="B4" s="86" t="s">
         <v>212</v>
       </c>
-      <c r="C4" s="84" t="s">
+      <c r="C4" s="86" t="s">
         <v>219</v>
       </c>
       <c r="D4" s="23"/>
-      <c r="E4" s="84" t="s">
+      <c r="E4" s="86" t="s">
         <v>212</v>
       </c>
-      <c r="F4" s="84" t="s">
+      <c r="F4" s="86" t="s">
         <v>283</v>
       </c>
-      <c r="G4" s="84" t="s">
+      <c r="G4" s="86" t="s">
         <v>284</v>
       </c>
-      <c r="H4" s="84" t="s">
+      <c r="H4" s="86" t="s">
         <v>285</v>
       </c>
       <c r="I4" s="23"/>
     </row>
     <row r="5" ht="6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" s="84" t="s">
+      <c r="A5" s="86" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="84" t="s">
+      <c r="B5" s="86" t="s">
         <v>213</v>
       </c>
-      <c r="C5" s="84" t="s">
+      <c r="C5" s="86" t="s">
         <v>220</v>
       </c>
       <c r="D5" s="23"/>
-      <c r="E5" s="84" t="s">
+      <c r="E5" s="86" t="s">
         <v>213</v>
       </c>
       <c r="F5" s="23"/>
       <c r="G5" s="23"/>
-      <c r="H5" s="84" t="s">
+      <c r="H5" s="86" t="s">
         <v>286</v>
       </c>
       <c r="I5" s="23"/>
@@ -5658,14 +5664,14 @@
       <c r="C6" s="24" t="s">
         <v>221</v>
       </c>
-      <c r="D6" s="85"/>
+      <c r="D6" s="87"/>
       <c r="E6" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="F6" s="85"/>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="85"/>
+      <c r="F6" s="87"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="87"/>
+      <c r="I6" s="87"/>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
@@ -5677,14 +5683,14 @@
       <c r="C7" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="D7" s="82"/>
+      <c r="D7" s="84"/>
       <c r="E7" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="F7" s="82"/>
-      <c r="G7" s="82"/>
-      <c r="H7" s="82"/>
-      <c r="I7" s="82"/>
+      <c r="F7" s="84"/>
+      <c r="G7" s="84"/>
+      <c r="H7" s="84"/>
+      <c r="I7" s="84"/>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="29" t="s">
@@ -5707,18 +5713,18 @@
       <c r="A9" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="B9" s="82"/>
+      <c r="B9" s="84"/>
       <c r="C9" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D9" s="82"/>
+      <c r="D9" s="84"/>
       <c r="E9" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
-      <c r="H9" s="82"/>
-      <c r="I9" s="82"/>
+      <c r="F9" s="84"/>
+      <c r="G9" s="84"/>
+      <c r="H9" s="84"/>
+      <c r="I9" s="84"/>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
@@ -5741,18 +5747,18 @@
       <c r="A11" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="B11" s="82"/>
+      <c r="B11" s="84"/>
       <c r="C11" s="6" t="s">
         <v>225</v>
       </c>
-      <c r="D11" s="82"/>
+      <c r="D11" s="84"/>
       <c r="E11" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="F11" s="82"/>
-      <c r="G11" s="82"/>
-      <c r="H11" s="82"/>
-      <c r="I11" s="82"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="84"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="84"/>
     </row>
     <row r="12" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
@@ -5775,18 +5781,18 @@
       <c r="A13" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="B13" s="82"/>
+      <c r="B13" s="84"/>
       <c r="C13" s="6" t="s">
         <v>227</v>
       </c>
-      <c r="D13" s="82"/>
+      <c r="D13" s="84"/>
       <c r="E13" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="F13" s="82"/>
-      <c r="G13" s="82"/>
-      <c r="H13" s="82"/>
-      <c r="I13" s="82"/>
+      <c r="F13" s="84"/>
+      <c r="G13" s="84"/>
+      <c r="H13" s="84"/>
+      <c r="I13" s="84"/>
     </row>
     <row r="14" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
@@ -5809,18 +5815,18 @@
       <c r="A15" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="82"/>
+      <c r="B15" s="84"/>
       <c r="C15" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="D15" s="82"/>
+      <c r="D15" s="84"/>
       <c r="E15" s="6" t="s">
         <v>223</v>
       </c>
-      <c r="F15" s="82"/>
-      <c r="G15" s="82"/>
-      <c r="H15" s="82"/>
-      <c r="I15" s="82"/>
+      <c r="F15" s="84"/>
+      <c r="G15" s="84"/>
+      <c r="H15" s="84"/>
+      <c r="I15" s="84"/>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
@@ -5843,18 +5849,18 @@
       <c r="A17" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="B17" s="82"/>
+      <c r="B17" s="84"/>
       <c r="C17" s="6" t="s">
         <v>231</v>
       </c>
-      <c r="D17" s="82"/>
+      <c r="D17" s="84"/>
       <c r="E17" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="F17" s="82"/>
-      <c r="G17" s="82"/>
-      <c r="H17" s="82"/>
-      <c r="I17" s="82"/>
+      <c r="F17" s="84"/>
+      <c r="G17" s="84"/>
+      <c r="H17" s="84"/>
+      <c r="I17" s="84"/>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
@@ -5877,18 +5883,18 @@
       <c r="A19" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="82"/>
+      <c r="B19" s="84"/>
       <c r="C19" s="6" t="s">
         <v>233</v>
       </c>
-      <c r="D19" s="82"/>
+      <c r="D19" s="84"/>
       <c r="E19" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="F19" s="82"/>
-      <c r="G19" s="82"/>
-      <c r="H19" s="82"/>
-      <c r="I19" s="82"/>
+      <c r="F19" s="84"/>
+      <c r="G19" s="84"/>
+      <c r="H19" s="84"/>
+      <c r="I19" s="84"/>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
@@ -5911,18 +5917,18 @@
       <c r="A21" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="82"/>
+      <c r="B21" s="84"/>
       <c r="C21" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="D21" s="82"/>
+      <c r="D21" s="84"/>
       <c r="E21" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="F21" s="82"/>
-      <c r="G21" s="82"/>
-      <c r="H21" s="82"/>
-      <c r="I21" s="82"/>
+      <c r="F21" s="84"/>
+      <c r="G21" s="84"/>
+      <c r="H21" s="84"/>
+      <c r="I21" s="84"/>
     </row>
     <row r="22" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
@@ -5945,18 +5951,18 @@
       <c r="A23" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="B23" s="82"/>
+      <c r="B23" s="84"/>
       <c r="C23" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="D23" s="82"/>
+      <c r="D23" s="84"/>
       <c r="E23" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="F23" s="82"/>
-      <c r="G23" s="82"/>
-      <c r="H23" s="82"/>
-      <c r="I23" s="82"/>
+      <c r="F23" s="84"/>
+      <c r="G23" s="84"/>
+      <c r="H23" s="84"/>
+      <c r="I23" s="84"/>
     </row>
     <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
@@ -5979,18 +5985,18 @@
       <c r="A25" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="82"/>
+      <c r="B25" s="84"/>
       <c r="C25" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="D25" s="82"/>
+      <c r="D25" s="84"/>
       <c r="E25" s="6" t="s">
         <v>232</v>
       </c>
-      <c r="F25" s="82"/>
-      <c r="G25" s="82"/>
-      <c r="H25" s="82"/>
-      <c r="I25" s="82"/>
+      <c r="F25" s="84"/>
+      <c r="G25" s="84"/>
+      <c r="H25" s="84"/>
+      <c r="I25" s="84"/>
     </row>
     <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="29" t="s">
@@ -6013,18 +6019,18 @@
       <c r="A27" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="B27" s="82"/>
+      <c r="B27" s="84"/>
       <c r="C27" s="6" t="s">
         <v>241</v>
       </c>
-      <c r="D27" s="82"/>
+      <c r="D27" s="84"/>
       <c r="E27" s="6" t="s">
         <v>234</v>
       </c>
-      <c r="F27" s="82"/>
-      <c r="G27" s="82"/>
-      <c r="H27" s="82"/>
-      <c r="I27" s="82"/>
+      <c r="F27" s="84"/>
+      <c r="G27" s="84"/>
+      <c r="H27" s="84"/>
+      <c r="I27" s="84"/>
     </row>
     <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
@@ -6047,18 +6053,18 @@
       <c r="A29" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="82"/>
+      <c r="B29" s="84"/>
       <c r="C29" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="D29" s="82"/>
+      <c r="D29" s="84"/>
       <c r="E29" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="F29" s="82"/>
-      <c r="G29" s="82"/>
-      <c r="H29" s="82"/>
-      <c r="I29" s="82"/>
+      <c r="F29" s="84"/>
+      <c r="G29" s="84"/>
+      <c r="H29" s="84"/>
+      <c r="I29" s="84"/>
     </row>
     <row r="30" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
@@ -6081,18 +6087,18 @@
       <c r="A31" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B31" s="82"/>
+      <c r="B31" s="84"/>
       <c r="C31" s="6" t="s">
         <v>245</v>
       </c>
-      <c r="D31" s="82"/>
+      <c r="D31" s="84"/>
       <c r="E31" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="F31" s="82"/>
-      <c r="G31" s="82"/>
-      <c r="H31" s="82"/>
-      <c r="I31" s="82"/>
+      <c r="F31" s="84"/>
+      <c r="G31" s="84"/>
+      <c r="H31" s="84"/>
+      <c r="I31" s="84"/>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="29" t="s">
@@ -6115,18 +6121,18 @@
       <c r="A33" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="B33" s="82"/>
+      <c r="B33" s="84"/>
       <c r="C33" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="D33" s="82"/>
+      <c r="D33" s="84"/>
       <c r="E33" s="6" t="s">
         <v>240</v>
       </c>
-      <c r="F33" s="82"/>
-      <c r="G33" s="82"/>
-      <c r="H33" s="82"/>
-      <c r="I33" s="82"/>
+      <c r="F33" s="84"/>
+      <c r="G33" s="84"/>
+      <c r="H33" s="84"/>
+      <c r="I33" s="84"/>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="29" t="s">
@@ -6149,18 +6155,18 @@
       <c r="A35" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="B35" s="82"/>
+      <c r="B35" s="84"/>
       <c r="C35" s="6" t="s">
         <v>249</v>
       </c>
-      <c r="D35" s="82"/>
+      <c r="D35" s="84"/>
       <c r="E35" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="F35" s="82"/>
-      <c r="G35" s="82"/>
-      <c r="H35" s="82"/>
-      <c r="I35" s="82"/>
+      <c r="F35" s="84"/>
+      <c r="G35" s="84"/>
+      <c r="H35" s="84"/>
+      <c r="I35" s="84"/>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="29" t="s">
@@ -6183,18 +6189,18 @@
       <c r="A37" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="B37" s="82"/>
+      <c r="B37" s="84"/>
       <c r="C37" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="D37" s="82"/>
+      <c r="D37" s="84"/>
       <c r="E37" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="F37" s="82"/>
-      <c r="G37" s="82"/>
-      <c r="H37" s="82"/>
-      <c r="I37" s="82"/>
+      <c r="F37" s="84"/>
+      <c r="G37" s="84"/>
+      <c r="H37" s="84"/>
+      <c r="I37" s="84"/>
     </row>
     <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="29" t="s">
@@ -6217,18 +6223,18 @@
       <c r="A39" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="82"/>
+      <c r="B39" s="84"/>
       <c r="C39" s="6" t="s">
         <v>253</v>
       </c>
-      <c r="D39" s="82"/>
+      <c r="D39" s="84"/>
       <c r="E39" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="F39" s="82"/>
-      <c r="G39" s="82"/>
-      <c r="H39" s="82"/>
-      <c r="I39" s="82"/>
+      <c r="F39" s="84"/>
+      <c r="G39" s="84"/>
+      <c r="H39" s="84"/>
+      <c r="I39" s="84"/>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
@@ -6251,18 +6257,18 @@
       <c r="A41" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="B41" s="82"/>
+      <c r="B41" s="84"/>
       <c r="C41" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="D41" s="82"/>
+      <c r="D41" s="84"/>
       <c r="E41" s="6" t="s">
         <v>248</v>
       </c>
-      <c r="F41" s="82"/>
-      <c r="G41" s="82"/>
-      <c r="H41" s="82"/>
-      <c r="I41" s="82"/>
+      <c r="F41" s="84"/>
+      <c r="G41" s="84"/>
+      <c r="H41" s="84"/>
+      <c r="I41" s="84"/>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="29" t="s">
@@ -6285,18 +6291,18 @@
       <c r="A43" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="B43" s="82"/>
+      <c r="B43" s="84"/>
       <c r="C43" s="6" t="s">
         <v>257</v>
       </c>
-      <c r="D43" s="82"/>
+      <c r="D43" s="84"/>
       <c r="E43" s="6" t="s">
         <v>250</v>
       </c>
-      <c r="F43" s="82"/>
-      <c r="G43" s="82"/>
-      <c r="H43" s="82"/>
-      <c r="I43" s="82"/>
+      <c r="F43" s="84"/>
+      <c r="G43" s="84"/>
+      <c r="H43" s="84"/>
+      <c r="I43" s="84"/>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="29" t="s">
@@ -6319,18 +6325,18 @@
       <c r="A45" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="B45" s="82"/>
+      <c r="B45" s="84"/>
       <c r="C45" s="6" t="s">
         <v>259</v>
       </c>
-      <c r="D45" s="82"/>
+      <c r="D45" s="84"/>
       <c r="E45" s="6" t="s">
         <v>252</v>
       </c>
-      <c r="F45" s="82"/>
-      <c r="G45" s="82"/>
-      <c r="H45" s="82"/>
-      <c r="I45" s="82"/>
+      <c r="F45" s="84"/>
+      <c r="G45" s="84"/>
+      <c r="H45" s="84"/>
+      <c r="I45" s="84"/>
     </row>
     <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="29" t="s">
@@ -6353,18 +6359,18 @@
       <c r="A47" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="B47" s="82"/>
+      <c r="B47" s="84"/>
       <c r="C47" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="D47" s="82"/>
+      <c r="D47" s="84"/>
       <c r="E47" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="F47" s="82"/>
-      <c r="G47" s="82"/>
-      <c r="H47" s="82"/>
-      <c r="I47" s="82"/>
+      <c r="F47" s="84"/>
+      <c r="G47" s="84"/>
+      <c r="H47" s="84"/>
+      <c r="I47" s="84"/>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="29" t="s">
@@ -6387,18 +6393,18 @@
       <c r="A49" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="B49" s="82"/>
+      <c r="B49" s="84"/>
       <c r="C49" s="6" t="s">
         <v>263</v>
       </c>
-      <c r="D49" s="82"/>
+      <c r="D49" s="84"/>
       <c r="E49" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="F49" s="82"/>
-      <c r="G49" s="82"/>
-      <c r="H49" s="82"/>
-      <c r="I49" s="82"/>
+      <c r="F49" s="84"/>
+      <c r="G49" s="84"/>
+      <c r="H49" s="84"/>
+      <c r="I49" s="84"/>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="29" t="s">
@@ -6421,18 +6427,18 @@
       <c r="A51" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="B51" s="82"/>
+      <c r="B51" s="84"/>
       <c r="C51" s="6" t="s">
         <v>265</v>
       </c>
-      <c r="D51" s="82"/>
+      <c r="D51" s="84"/>
       <c r="E51" s="6" t="s">
         <v>258</v>
       </c>
-      <c r="F51" s="82"/>
-      <c r="G51" s="82"/>
-      <c r="H51" s="82"/>
-      <c r="I51" s="82"/>
+      <c r="F51" s="84"/>
+      <c r="G51" s="84"/>
+      <c r="H51" s="84"/>
+      <c r="I51" s="84"/>
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="29" t="s">
@@ -6453,16 +6459,16 @@
       <c r="A53" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="B53" s="82"/>
-      <c r="C53" s="82"/>
-      <c r="D53" s="82"/>
+      <c r="B53" s="84"/>
+      <c r="C53" s="84"/>
+      <c r="D53" s="84"/>
       <c r="E53" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="F53" s="82"/>
-      <c r="G53" s="82"/>
-      <c r="H53" s="82"/>
-      <c r="I53" s="82"/>
+      <c r="F53" s="84"/>
+      <c r="G53" s="84"/>
+      <c r="H53" s="84"/>
+      <c r="I53" s="84"/>
     </row>
     <row r="54" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="29" t="s">
@@ -6483,16 +6489,16 @@
       <c r="A55" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="B55" s="82"/>
-      <c r="C55" s="82"/>
-      <c r="D55" s="82"/>
+      <c r="B55" s="84"/>
+      <c r="C55" s="84"/>
+      <c r="D55" s="84"/>
       <c r="E55" s="6" t="s">
         <v>262</v>
       </c>
-      <c r="F55" s="82"/>
-      <c r="G55" s="82"/>
-      <c r="H55" s="82"/>
-      <c r="I55" s="82"/>
+      <c r="F55" s="84"/>
+      <c r="G55" s="84"/>
+      <c r="H55" s="84"/>
+      <c r="I55" s="84"/>
     </row>
     <row r="56" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="29" t="s">
@@ -6513,16 +6519,16 @@
       <c r="A57" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="B57" s="82"/>
-      <c r="C57" s="82"/>
-      <c r="D57" s="82"/>
+      <c r="B57" s="84"/>
+      <c r="C57" s="84"/>
+      <c r="D57" s="84"/>
       <c r="E57" s="6" t="s">
         <v>264</v>
       </c>
-      <c r="F57" s="82"/>
-      <c r="G57" s="82"/>
-      <c r="H57" s="82"/>
-      <c r="I57" s="82"/>
+      <c r="F57" s="84"/>
+      <c r="G57" s="84"/>
+      <c r="H57" s="84"/>
+      <c r="I57" s="84"/>
     </row>
     <row r="58" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="29" t="s">
@@ -6543,14 +6549,14 @@
       <c r="A59" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="B59" s="82"/>
-      <c r="C59" s="82"/>
-      <c r="D59" s="82"/>
-      <c r="E59" s="82"/>
-      <c r="F59" s="82"/>
-      <c r="G59" s="82"/>
-      <c r="H59" s="82"/>
-      <c r="I59" s="82"/>
+      <c r="B59" s="84"/>
+      <c r="C59" s="84"/>
+      <c r="D59" s="84"/>
+      <c r="E59" s="84"/>
+      <c r="F59" s="84"/>
+      <c r="G59" s="84"/>
+      <c r="H59" s="84"/>
+      <c r="I59" s="84"/>
     </row>
     <row r="60" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="29" t="s">
@@ -6569,14 +6575,14 @@
       <c r="A61" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="B61" s="82"/>
-      <c r="C61" s="82"/>
-      <c r="D61" s="82"/>
-      <c r="E61" s="82"/>
-      <c r="F61" s="82"/>
-      <c r="G61" s="82"/>
-      <c r="H61" s="82"/>
-      <c r="I61" s="82"/>
+      <c r="B61" s="84"/>
+      <c r="C61" s="84"/>
+      <c r="D61" s="84"/>
+      <c r="E61" s="84"/>
+      <c r="F61" s="84"/>
+      <c r="G61" s="84"/>
+      <c r="H61" s="84"/>
+      <c r="I61" s="84"/>
     </row>
     <row r="62" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="29" t="s">
@@ -6595,14 +6601,14 @@
       <c r="A63" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="B63" s="82"/>
-      <c r="C63" s="82"/>
-      <c r="D63" s="82"/>
-      <c r="E63" s="82"/>
-      <c r="F63" s="82"/>
-      <c r="G63" s="82"/>
-      <c r="H63" s="82"/>
-      <c r="I63" s="82"/>
+      <c r="B63" s="84"/>
+      <c r="C63" s="84"/>
+      <c r="D63" s="84"/>
+      <c r="E63" s="84"/>
+      <c r="F63" s="84"/>
+      <c r="G63" s="84"/>
+      <c r="H63" s="84"/>
+      <c r="I63" s="84"/>
     </row>
     <row r="64" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="29" t="s">
@@ -6621,14 +6627,14 @@
       <c r="A65" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B65" s="82"/>
-      <c r="C65" s="82"/>
-      <c r="D65" s="82"/>
-      <c r="E65" s="82"/>
-      <c r="F65" s="82"/>
-      <c r="G65" s="82"/>
-      <c r="H65" s="82"/>
-      <c r="I65" s="82"/>
+      <c r="B65" s="84"/>
+      <c r="C65" s="84"/>
+      <c r="D65" s="84"/>
+      <c r="E65" s="84"/>
+      <c r="F65" s="84"/>
+      <c r="G65" s="84"/>
+      <c r="H65" s="84"/>
+      <c r="I65" s="84"/>
     </row>
     <row r="66" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="29" t="s">
@@ -6647,14 +6653,14 @@
       <c r="A67" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="B67" s="82"/>
-      <c r="C67" s="82"/>
-      <c r="D67" s="82"/>
-      <c r="E67" s="82"/>
-      <c r="F67" s="82"/>
-      <c r="G67" s="82"/>
-      <c r="H67" s="82"/>
-      <c r="I67" s="82"/>
+      <c r="B67" s="84"/>
+      <c r="C67" s="84"/>
+      <c r="D67" s="84"/>
+      <c r="E67" s="84"/>
+      <c r="F67" s="84"/>
+      <c r="G67" s="84"/>
+      <c r="H67" s="84"/>
+      <c r="I67" s="84"/>
     </row>
     <row r="68" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="29" t="s">
@@ -6673,14 +6679,14 @@
       <c r="A69" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B69" s="82"/>
-      <c r="C69" s="82"/>
-      <c r="D69" s="82"/>
-      <c r="E69" s="82"/>
-      <c r="F69" s="82"/>
-      <c r="G69" s="82"/>
-      <c r="H69" s="82"/>
-      <c r="I69" s="82"/>
+      <c r="B69" s="84"/>
+      <c r="C69" s="84"/>
+      <c r="D69" s="84"/>
+      <c r="E69" s="84"/>
+      <c r="F69" s="84"/>
+      <c r="G69" s="84"/>
+      <c r="H69" s="84"/>
+      <c r="I69" s="84"/>
     </row>
     <row r="70" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="29" t="s">
@@ -6699,14 +6705,14 @@
       <c r="A71" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="B71" s="82"/>
-      <c r="C71" s="82"/>
-      <c r="D71" s="82"/>
-      <c r="E71" s="82"/>
-      <c r="F71" s="82"/>
-      <c r="G71" s="82"/>
-      <c r="H71" s="82"/>
-      <c r="I71" s="82"/>
+      <c r="B71" s="84"/>
+      <c r="C71" s="84"/>
+      <c r="D71" s="84"/>
+      <c r="E71" s="84"/>
+      <c r="F71" s="84"/>
+      <c r="G71" s="84"/>
+      <c r="H71" s="84"/>
+      <c r="I71" s="84"/>
     </row>
     <row r="72" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="29" t="s">
@@ -6725,14 +6731,14 @@
       <c r="A73" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="B73" s="82"/>
-      <c r="C73" s="82"/>
-      <c r="D73" s="82"/>
-      <c r="E73" s="82"/>
-      <c r="F73" s="82"/>
-      <c r="G73" s="82"/>
-      <c r="H73" s="82"/>
-      <c r="I73" s="82"/>
+      <c r="B73" s="84"/>
+      <c r="C73" s="84"/>
+      <c r="D73" s="84"/>
+      <c r="E73" s="84"/>
+      <c r="F73" s="84"/>
+      <c r="G73" s="84"/>
+      <c r="H73" s="84"/>
+      <c r="I73" s="84"/>
     </row>
     <row r="74" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="29" t="s">
@@ -6751,14 +6757,14 @@
       <c r="A75" s="12" t="s">
         <v>191</v>
       </c>
-      <c r="B75" s="82"/>
-      <c r="C75" s="82"/>
-      <c r="D75" s="82"/>
-      <c r="E75" s="82"/>
-      <c r="F75" s="82"/>
-      <c r="G75" s="82"/>
-      <c r="H75" s="82"/>
-      <c r="I75" s="82"/>
+      <c r="B75" s="84"/>
+      <c r="C75" s="84"/>
+      <c r="D75" s="84"/>
+      <c r="E75" s="84"/>
+      <c r="F75" s="84"/>
+      <c r="G75" s="84"/>
+      <c r="H75" s="84"/>
+      <c r="I75" s="84"/>
     </row>
     <row r="76" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="29" t="s">
@@ -6777,14 +6783,14 @@
       <c r="A77" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B77" s="82"/>
-      <c r="C77" s="82"/>
-      <c r="D77" s="82"/>
-      <c r="E77" s="82"/>
-      <c r="F77" s="82"/>
-      <c r="G77" s="82"/>
-      <c r="H77" s="82"/>
-      <c r="I77" s="82"/>
+      <c r="B77" s="84"/>
+      <c r="C77" s="84"/>
+      <c r="D77" s="84"/>
+      <c r="E77" s="84"/>
+      <c r="F77" s="84"/>
+      <c r="G77" s="84"/>
+      <c r="H77" s="84"/>
+      <c r="I77" s="84"/>
     </row>
     <row r="78" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="29" t="s">
@@ -6803,14 +6809,14 @@
       <c r="A79" s="12" t="s">
         <v>195</v>
       </c>
-      <c r="B79" s="82"/>
-      <c r="C79" s="82"/>
-      <c r="D79" s="82"/>
-      <c r="E79" s="82"/>
-      <c r="F79" s="82"/>
-      <c r="G79" s="82"/>
-      <c r="H79" s="82"/>
-      <c r="I79" s="82"/>
+      <c r="B79" s="84"/>
+      <c r="C79" s="84"/>
+      <c r="D79" s="84"/>
+      <c r="E79" s="84"/>
+      <c r="F79" s="84"/>
+      <c r="G79" s="84"/>
+      <c r="H79" s="84"/>
+      <c r="I79" s="84"/>
     </row>
     <row r="80" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="29" t="s">
@@ -6829,14 +6835,14 @@
       <c r="A81" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="B81" s="82"/>
-      <c r="C81" s="82"/>
-      <c r="D81" s="82"/>
-      <c r="E81" s="82"/>
-      <c r="F81" s="82"/>
-      <c r="G81" s="82"/>
-      <c r="H81" s="82"/>
-      <c r="I81" s="82"/>
+      <c r="B81" s="84"/>
+      <c r="C81" s="84"/>
+      <c r="D81" s="84"/>
+      <c r="E81" s="84"/>
+      <c r="F81" s="84"/>
+      <c r="G81" s="84"/>
+      <c r="H81" s="84"/>
+      <c r="I81" s="84"/>
     </row>
     <row r="82" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="29" t="s">
@@ -6855,14 +6861,14 @@
       <c r="A83" s="12" t="s">
         <v>199</v>
       </c>
-      <c r="B83" s="82"/>
-      <c r="C83" s="82"/>
-      <c r="D83" s="82"/>
-      <c r="E83" s="82"/>
-      <c r="F83" s="82"/>
-      <c r="G83" s="82"/>
-      <c r="H83" s="82"/>
-      <c r="I83" s="82"/>
+      <c r="B83" s="84"/>
+      <c r="C83" s="84"/>
+      <c r="D83" s="84"/>
+      <c r="E83" s="84"/>
+      <c r="F83" s="84"/>
+      <c r="G83" s="84"/>
+      <c r="H83" s="84"/>
+      <c r="I83" s="84"/>
     </row>
     <row r="84" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="29" t="s">
@@ -6881,14 +6887,14 @@
       <c r="A85" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="B85" s="82"/>
-      <c r="C85" s="82"/>
-      <c r="D85" s="82"/>
-      <c r="E85" s="82"/>
-      <c r="F85" s="82"/>
-      <c r="G85" s="82"/>
-      <c r="H85" s="82"/>
-      <c r="I85" s="82"/>
+      <c r="B85" s="84"/>
+      <c r="C85" s="84"/>
+      <c r="D85" s="84"/>
+      <c r="E85" s="84"/>
+      <c r="F85" s="84"/>
+      <c r="G85" s="84"/>
+      <c r="H85" s="84"/>
+      <c r="I85" s="84"/>
     </row>
     <row r="86" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="29" t="s">
@@ -6907,14 +6913,14 @@
       <c r="A87" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="B87" s="82"/>
-      <c r="C87" s="82"/>
-      <c r="D87" s="82"/>
-      <c r="E87" s="82"/>
-      <c r="F87" s="82"/>
-      <c r="G87" s="82"/>
-      <c r="H87" s="82"/>
-      <c r="I87" s="82"/>
+      <c r="B87" s="84"/>
+      <c r="C87" s="84"/>
+      <c r="D87" s="84"/>
+      <c r="E87" s="84"/>
+      <c r="F87" s="84"/>
+      <c r="G87" s="84"/>
+      <c r="H87" s="84"/>
+      <c r="I87" s="84"/>
     </row>
     <row r="88" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="29" t="s">
@@ -6933,14 +6939,14 @@
       <c r="A89" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="B89" s="82"/>
-      <c r="C89" s="82"/>
-      <c r="D89" s="82"/>
-      <c r="E89" s="82"/>
-      <c r="F89" s="82"/>
-      <c r="G89" s="82"/>
-      <c r="H89" s="82"/>
-      <c r="I89" s="82"/>
+      <c r="B89" s="84"/>
+      <c r="C89" s="84"/>
+      <c r="D89" s="84"/>
+      <c r="E89" s="84"/>
+      <c r="F89" s="84"/>
+      <c r="G89" s="84"/>
+      <c r="H89" s="84"/>
+      <c r="I89" s="84"/>
     </row>
     <row r="90" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="29" t="s">
@@ -6959,14 +6965,14 @@
       <c r="A91" s="12" t="s">
         <v>206</v>
       </c>
-      <c r="B91" s="82"/>
-      <c r="C91" s="82"/>
-      <c r="D91" s="82"/>
-      <c r="E91" s="82"/>
-      <c r="F91" s="82"/>
-      <c r="G91" s="82"/>
-      <c r="H91" s="82"/>
-      <c r="I91" s="82"/>
+      <c r="B91" s="84"/>
+      <c r="C91" s="84"/>
+      <c r="D91" s="84"/>
+      <c r="E91" s="84"/>
+      <c r="F91" s="84"/>
+      <c r="G91" s="84"/>
+      <c r="H91" s="84"/>
+      <c r="I91" s="84"/>
     </row>
     <row r="92" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="29" t="s">
@@ -6985,14 +6991,14 @@
       <c r="A93" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="B93" s="82"/>
-      <c r="C93" s="82"/>
-      <c r="D93" s="82"/>
-      <c r="E93" s="82"/>
-      <c r="F93" s="82"/>
-      <c r="G93" s="82"/>
-      <c r="H93" s="82"/>
-      <c r="I93" s="82"/>
+      <c r="B93" s="84"/>
+      <c r="C93" s="84"/>
+      <c r="D93" s="84"/>
+      <c r="E93" s="84"/>
+      <c r="F93" s="84"/>
+      <c r="G93" s="84"/>
+      <c r="H93" s="84"/>
+      <c r="I93" s="84"/>
     </row>
     <row r="94" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="29" t="s">
@@ -7036,7 +7042,7 @@
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A1" s="86">
+      <c r="A1" s="88">
         <v>46286</v>
       </c>
       <c r="B1" s="1">
@@ -7493,38 +7499,38 @@
       <c r="AF5" s="23"/>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A6" s="85"/>
-      <c r="B6" s="85"/>
-      <c r="C6" s="85"/>
-      <c r="D6" s="85"/>
-      <c r="E6" s="85"/>
-      <c r="F6" s="85"/>
-      <c r="G6" s="85"/>
-      <c r="H6" s="85"/>
-      <c r="I6" s="85"/>
-      <c r="J6" s="85"/>
-      <c r="K6" s="85"/>
-      <c r="L6" s="85"/>
-      <c r="M6" s="85"/>
-      <c r="N6" s="85"/>
-      <c r="O6" s="85"/>
-      <c r="P6" s="85"/>
-      <c r="Q6" s="85"/>
-      <c r="R6" s="85"/>
-      <c r="S6" s="85"/>
-      <c r="T6" s="85"/>
-      <c r="U6" s="85"/>
-      <c r="V6" s="85"/>
-      <c r="W6" s="85"/>
-      <c r="X6" s="85"/>
-      <c r="Y6" s="85"/>
-      <c r="Z6" s="85"/>
-      <c r="AA6" s="85"/>
-      <c r="AB6" s="85"/>
-      <c r="AC6" s="85"/>
-      <c r="AD6" s="85"/>
-      <c r="AE6" s="85"/>
-      <c r="AF6" s="85"/>
+      <c r="A6" s="87"/>
+      <c r="B6" s="87"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="F6" s="87"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="87"/>
+      <c r="I6" s="87"/>
+      <c r="J6" s="87"/>
+      <c r="K6" s="87"/>
+      <c r="L6" s="87"/>
+      <c r="M6" s="87"/>
+      <c r="N6" s="87"/>
+      <c r="O6" s="87"/>
+      <c r="P6" s="87"/>
+      <c r="Q6" s="87"/>
+      <c r="R6" s="87"/>
+      <c r="S6" s="87"/>
+      <c r="T6" s="87"/>
+      <c r="U6" s="87"/>
+      <c r="V6" s="87"/>
+      <c r="W6" s="87"/>
+      <c r="X6" s="87"/>
+      <c r="Y6" s="87"/>
+      <c r="Z6" s="87"/>
+      <c r="AA6" s="87"/>
+      <c r="AB6" s="87"/>
+      <c r="AC6" s="87"/>
+      <c r="AD6" s="87"/>
+      <c r="AE6" s="87"/>
+      <c r="AF6" s="87"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
@@ -23144,22 +23150,22 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="78" t="s">
         <v>93</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="27">
         <v>5</v>
       </c>
-      <c r="D7" s="8">
+      <c r="D7" s="27">
         <v>3</v>
       </c>
-      <c r="E7" s="64">
+      <c r="E7" s="79">
         <v>4464</v>
       </c>
-      <c r="F7" s="64">
+      <c r="F7" s="79">
         <v>0</v>
       </c>
       <c r="G7" s="64">
@@ -23168,22 +23174,22 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="80" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="32">
         <v>3</v>
       </c>
-      <c r="D8" s="11">
+      <c r="D8" s="32">
         <v>2</v>
       </c>
-      <c r="E8" s="59">
+      <c r="E8" s="81">
         <v>612</v>
       </c>
-      <c r="F8" s="59">
+      <c r="F8" s="81">
         <v>0</v>
       </c>
       <c r="G8" s="59">
@@ -23192,22 +23198,22 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="78" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="25" t="s">
         <v>94</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="27">
         <v>3</v>
       </c>
-      <c r="D9" s="8">
+      <c r="D9" s="27">
         <v>2</v>
       </c>
-      <c r="E9" s="64">
+      <c r="E9" s="79">
         <v>936</v>
       </c>
-      <c r="F9" s="64">
+      <c r="F9" s="79">
         <v>0</v>
       </c>
       <c r="G9" s="64">
@@ -23216,22 +23222,22 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="29" t="s">
+      <c r="A10" s="80" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="30" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="11">
-        <v>1</v>
-      </c>
-      <c r="D10" s="11">
+      <c r="C10" s="32">
+        <v>1</v>
+      </c>
+      <c r="D10" s="32">
         <v>32</v>
       </c>
-      <c r="E10" s="59">
+      <c r="E10" s="81">
         <v>1160</v>
       </c>
-      <c r="F10" s="59">
+      <c r="F10" s="81">
         <v>0</v>
       </c>
       <c r="G10" s="59">
@@ -23346,7 +23352,7 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="78" t="s">
         <v>103</v>
       </c>
       <c r="B7" s="27">
@@ -23355,7 +23361,7 @@
       <c r="C7" s="27">
         <v>1500</v>
       </c>
-      <c r="D7" s="78">
+      <c r="D7" s="79">
         <v>0.76</v>
       </c>
       <c r="E7" s="64">
@@ -23468,7 +23474,7 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="78" t="s">
         <v>106</v>
       </c>
       <c r="B7" s="25" t="s">
@@ -23477,7 +23483,7 @@
       <c r="C7" s="27">
         <v>3.5</v>
       </c>
-      <c r="D7" s="78">
+      <c r="D7" s="79">
         <v>1000</v>
       </c>
       <c r="E7" s="64">
@@ -23486,7 +23492,7 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="80" t="s">
         <v>108</v>
       </c>
       <c r="B8" s="30" t="s">
@@ -23495,7 +23501,7 @@
       <c r="C8" s="32">
         <v>1</v>
       </c>
-      <c r="D8" s="79">
+      <c r="D8" s="81">
         <v>1200</v>
       </c>
       <c r="E8" s="59">
@@ -23504,7 +23510,7 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="78" t="s">
         <v>110</v>
       </c>
       <c r="B9" s="25" t="s">
@@ -23513,7 +23519,7 @@
       <c r="C9" s="27">
         <v>1</v>
       </c>
-      <c r="D9" s="78">
+      <c r="D9" s="79">
         <v>6000</v>
       </c>
       <c r="E9" s="64">

</xml_diff>

<commit_message>
Unlock Subcontractor inputs and group craft sheets Days then Nights.
Cost-sheet estimator cells stay editable on a protected sheet. Craft tabs emit every DAYSHIFT block first, then NIGHTSHIFT, without changing clock math.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -242,34 +242,34 @@
     <t>PD</t>
   </si>
   <si>
+    <t>COORDINATOR QA-QC 1</t>
+  </si>
+  <si>
+    <t>cr-1787762352222-vw0iw|day</t>
+  </si>
+  <si>
+    <t>COORDINATOR SAFETY 01</t>
+  </si>
+  <si>
+    <t>cr-1787762351054-x15wg|day</t>
+  </si>
+  <si>
+    <t>Pipefitter General Foreman</t>
+  </si>
+  <si>
+    <t>cr-1787763765587-o1zgp|day</t>
+  </si>
+  <si>
     <t>NIGHTSHIFT</t>
   </si>
   <si>
     <t>cr-1787760932966-c9m84|night</t>
   </si>
   <si>
-    <t>COORDINATOR QA-QC 1</t>
-  </si>
-  <si>
-    <t>cr-1787762352222-vw0iw|day</t>
-  </si>
-  <si>
     <t>cr-1787762352222-vw0iw|night</t>
   </si>
   <si>
-    <t>COORDINATOR SAFETY 01</t>
-  </si>
-  <si>
-    <t>cr-1787762351054-x15wg|day</t>
-  </si>
-  <si>
     <t>cr-1787762351054-x15wg|night</t>
-  </si>
-  <si>
-    <t>Pipefitter General Foreman</t>
-  </si>
-  <si>
-    <t>cr-1787763765587-o1zgp|day</t>
   </si>
   <si>
     <t>cr-1787763765587-o1zgp|night</t>
@@ -2338,7 +2338,7 @@
     </row>
     <row r="8" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="29" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B8" s="59">
         <v>64</v>
@@ -2358,7 +2358,7 @@
     </row>
     <row r="9" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B9" s="64">
         <v>52.5</v>
@@ -2378,7 +2378,7 @@
     </row>
     <row r="10" ht="16" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B10" s="59">
         <v>58.84</v>
@@ -5881,7 +5881,7 @@
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B19" s="84"/>
       <c r="C19" s="6" t="s">
@@ -7002,7 +7002,7 @@
     </row>
     <row r="94" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="29" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B94" s="20"/>
       <c r="C94" s="20"/>
@@ -9227,21 +9227,21 @@
       <c r="AP14" s="71"/>
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A15" s="72" t="s">
+      <c r="A15" s="43" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" s="44" t="s">
         <v>63</v>
-      </c>
-      <c r="B15" s="44" t="s">
-        <v>55</v>
       </c>
       <c r="C15" s="45">
         <f>J15</f>
-        <v>30005.120000000003</v>
+        <v>33109.96000000001</v>
       </c>
       <c r="D15" s="46"/>
       <c r="E15" s="46"/>
       <c r="F15" s="47">
         <f>SUM(K18:AP18)</f>
-        <v>164</v>
+        <v>212</v>
       </c>
       <c r="G15" s="47">
         <f>SUM(K19:AP19)</f>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="J15" s="48">
         <f>C18+C19+C20</f>
-        <v>30005.120000000003</v>
+        <v>33109.96000000001</v>
       </c>
       <c r="K15" s="49"/>
       <c r="L15" s="50"/>
@@ -9296,7 +9296,7 @@
       </c>
     </row>
     <row r="16" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A16" s="72"/>
+      <c r="A16" s="43"/>
       <c r="B16" s="44"/>
       <c r="C16" s="45"/>
       <c r="D16" s="46"/>
@@ -9381,10 +9381,10 @@
         <v>1</v>
       </c>
       <c r="AI16" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ16" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK16" s="56">
         <v>0</v>
@@ -9393,23 +9393,23 @@
         <v>0</v>
       </c>
       <c r="AM16" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN16" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO16" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP16" s="57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="OU16" s="58" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A17" s="72"/>
+      <c r="A17" s="43"/>
       <c r="B17" s="44"/>
       <c r="C17" s="45"/>
       <c r="D17" s="46"/>
@@ -9494,10 +9494,10 @@
         <v>12</v>
       </c>
       <c r="AI17" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AJ17" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AK17" s="56">
         <v>0</v>
@@ -9506,31 +9506,31 @@
         <v>0</v>
       </c>
       <c r="AM17" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AN17" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AO17" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AP17" s="57">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="OU17" s="58" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A18" s="72"/>
+      <c r="A18" s="43"/>
       <c r="B18" s="44"/>
       <c r="C18" s="59">
         <f>F15*N(D18)</f>
-        <v>18313.88</v>
+        <v>22421.120000000003</v>
       </c>
       <c r="D18" s="59">
         <f>IF(TRIM(B15)="","No rate",IFERROR(INDEX('Rate Tables'!C$7:C$161,MATCH(B15,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>111.67</v>
+        <v>105.76</v>
       </c>
       <c r="E18" s="53" t="s">
         <v>59</v>
@@ -9637,51 +9637,51 @@
         <v>10</v>
       </c>
       <c r="AI18" s="61">
-        <f>IF(AND(AI16=0,AI17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI17)*AI16)),MAX(0,40*MAX(1,AI16)-(0))))</f>
-        <v>0</v>
+        <f>IF(AND(AI16=1,AI17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI17)*AI16)),MAX(0,40*MAX(1,AI16)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="AJ18" s="61">
-        <f>IF(AND(AJ16=0,AJ17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ17)*AJ16)),MAX(0,40*MAX(1,AJ16)-(AI18))))</f>
-        <v>0</v>
+        <f>IF(AND(AJ16=1,AJ17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ17)*AJ16)),MAX(0,40*MAX(1,AJ16)-(AI18))))</f>
+        <v>8</v>
       </c>
       <c r="AK18" s="62">
-        <f>IF(AND(AK16=0,AK17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK17)*AK16)),MAX(0,40*MAX(1,AK16)-(AI18+AJ18))))</f>
+        <f>IF(AND(AK16=0,AK17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK17)*AK16)),MAX(0,40*MAX(1,AK16)-(0))))</f>
         <v>0</v>
       </c>
       <c r="AL18" s="62">
-        <f>IF(AND(AL16=0,AL17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL17)*AL16)),MAX(0,40*MAX(1,AL16)-(AI18+AJ18+AK18))))</f>
+        <f>IF(AND(AL16=0,AL17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL17)*AL16)),MAX(0,40*MAX(1,AL16)-(AK18))))</f>
         <v>0</v>
       </c>
       <c r="AM18" s="61">
-        <f>IF(AND(AM16=0,AM17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM17)*AM16)),MAX(0,40*MAX(1,AM16)-(0))))</f>
-        <v>0</v>
+        <f>IF(AND(AM16=1,AM17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM17)*AM16)),MAX(0,40*MAX(1,AM16)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="AN18" s="61">
-        <f>IF(AND(AN16=0,AN17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN17)*AN16)),MAX(0,40*MAX(1,AN16)-(AM18))))</f>
-        <v>0</v>
+        <f>IF(AND(AN16=1,AN17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN17)*AN16)),MAX(0,40*MAX(1,AN16)-(AM18))))</f>
+        <v>8</v>
       </c>
       <c r="AO18" s="61">
-        <f>IF(AND(AO16=0,AO17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO17)*AO16)),MAX(0,40*MAX(1,AO16)-(AM18+AN18))))</f>
-        <v>0</v>
+        <f>IF(AND(AO16=1,AO17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO17)*AO16)),MAX(0,40*MAX(1,AO16)-(AM18+AN18))))</f>
+        <v>8</v>
       </c>
       <c r="AP18" s="63">
-        <f>IF(AND(AP16=0,AP17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP17)*AP16)),MAX(0,40*MAX(1,AP16)-(AM18+AN18+AO18))))</f>
-        <v>0</v>
+        <f>IF(AND(AP16=1,AP17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP17)*AP16)),MAX(0,40*MAX(1,AP16)-(AM18+AN18+AO18))))</f>
+        <v>8</v>
       </c>
       <c r="OU18" s="28" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A19" s="72"/>
+      <c r="A19" s="43"/>
       <c r="B19" s="44"/>
       <c r="C19" s="64">
         <f>G15*N(D19)</f>
-        <v>6873.240000000001</v>
+        <v>6325.88</v>
       </c>
       <c r="D19" s="64">
         <f>IF(TRIM(B15)="","No rate",IFERROR(INDEX('Rate Tables'!D$7:D$161,MATCH(B15,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>156.21</v>
+        <v>143.77</v>
       </c>
       <c r="E19" s="53" t="s">
         <v>60</v>
@@ -9788,35 +9788,35 @@
         <v>2</v>
       </c>
       <c r="AI19" s="61">
-        <f>IF(AND(AI16=0,AI17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MAX(0,AI17-(IF('_JobDays'!Y3,8,10)))*AI16))+((IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI17)*AI16)))-MIN(IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI17)*AI16)),MAX(0,40*MAX(1,AI16)-(0)))))</f>
+        <f>IF(AND(AI16=1,AI17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MAX(0,AI17-(IF('_JobDays'!Y3,8,10)))*AI16))+((IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI17)*AI16)))-MIN(IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI17)*AI16)),MAX(0,40*MAX(1,AI16)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AJ19" s="61">
-        <f>IF(AND(AJ16=0,AJ17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MAX(0,AJ17-(IF('_JobDays'!Z3,8,10)))*AJ16))+((IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ17)*AJ16)))-MIN(IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ17)*AJ16)),MAX(0,40*MAX(1,AJ16)-(AI18)))))</f>
+        <f>IF(AND(AJ16=1,AJ17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MAX(0,AJ17-(IF('_JobDays'!Z3,8,10)))*AJ16))+((IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ17)*AJ16)))-MIN(IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ17)*AJ16)),MAX(0,40*MAX(1,AJ16)-(AI18)))))</f>
         <v>0</v>
       </c>
       <c r="AK19" s="62">
-        <f>IF(AND(AK16=0,AK17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MAX(0,AK17-(IF('_JobDays'!AA3,8,10)))*AK16))+((IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK17)*AK16)))-MIN(IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK17)*AK16)),MAX(0,40*MAX(1,AK16)-(AI18+AJ18)))))</f>
+        <f>IF(AND(AK16=0,AK17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MAX(0,AK17-(IF('_JobDays'!AA3,8,10)))*AK16))+((IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK17)*AK16)))-MIN(IF(OR(AK16&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK17)*AK16)),MAX(0,40*MAX(1,AK16)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AL19" s="62">
-        <f>IF(AND(AL16=0,AL17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MAX(0,AL17-(IF('_JobDays'!AB3,8,10)))*AL16))+((IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL17)*AL16)))-MIN(IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL17)*AL16)),MAX(0,40*MAX(1,AL16)-(AI18+AJ18+AK18)))))</f>
+        <f>IF(AND(AL16=0,AL17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MAX(0,AL17-(IF('_JobDays'!AB3,8,10)))*AL16))+((IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL17)*AL16)))-MIN(IF(OR(AL16&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL17)*AL16)),MAX(0,40*MAX(1,AL16)-(AK18)))))</f>
         <v>0</v>
       </c>
       <c r="AM19" s="61">
-        <f>IF(AND(AM16=0,AM17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MAX(0,AM17-(IF('_JobDays'!AC3,8,10)))*AM16))+((IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM17)*AM16)))-MIN(IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM17)*AM16)),MAX(0,40*MAX(1,AM16)-(0)))))</f>
+        <f>IF(AND(AM16=1,AM17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MAX(0,AM17-(IF('_JobDays'!AC3,8,10)))*AM16))+((IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM17)*AM16)))-MIN(IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM17)*AM16)),MAX(0,40*MAX(1,AM16)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AN19" s="61">
-        <f>IF(AND(AN16=0,AN17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MAX(0,AN17-(IF('_JobDays'!AD3,8,10)))*AN16))+((IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN17)*AN16)))-MIN(IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN17)*AN16)),MAX(0,40*MAX(1,AN16)-(AM18)))))</f>
+        <f>IF(AND(AN16=1,AN17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MAX(0,AN17-(IF('_JobDays'!AD3,8,10)))*AN16))+((IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN17)*AN16)))-MIN(IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN17)*AN16)),MAX(0,40*MAX(1,AN16)-(AM18)))))</f>
         <v>0</v>
       </c>
       <c r="AO19" s="61">
-        <f>IF(AND(AO16=0,AO17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MAX(0,AO17-(IF('_JobDays'!AE3,8,10)))*AO16))+((IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO17)*AO16)))-MIN(IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO17)*AO16)),MAX(0,40*MAX(1,AO16)-(AM18+AN18)))))</f>
+        <f>IF(AND(AO16=1,AO17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MAX(0,AO17-(IF('_JobDays'!AE3,8,10)))*AO16))+((IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO17)*AO16)))-MIN(IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO17)*AO16)),MAX(0,40*MAX(1,AO16)-(AM18+AN18)))))</f>
         <v>0</v>
       </c>
       <c r="AP19" s="63">
-        <f>IF(AND(AP16=0,AP17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MAX(0,AP17-(IF('_JobDays'!AF3,8,10)))*AP16))+((IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP17)*AP16)))-MIN(IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP17)*AP16)),MAX(0,40*MAX(1,AP16)-(AM18+AN18+AO18)))))</f>
+        <f>IF(AND(AP16=1,AP17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MAX(0,AP17-(IF('_JobDays'!AF3,8,10)))*AP16))+((IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP17)*AP16)))-MIN(IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP17)*AP16)),MAX(0,40*MAX(1,AP16)-(AM18+AN18+AO18)))))</f>
         <v>0</v>
       </c>
       <c r="OU19" s="28" t="s">
@@ -9824,15 +9824,15 @@
       </c>
     </row>
     <row r="20" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A20" s="72"/>
+      <c r="A20" s="43"/>
       <c r="B20" s="44"/>
       <c r="C20" s="59">
         <f>H15*N(D20)</f>
-        <v>4818</v>
+        <v>4362.96</v>
       </c>
       <c r="D20" s="59">
         <f>IF(TRIM(B15)="","No rate",IFERROR(INDEX('Rate Tables'!E$7:E$161,MATCH(B15,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>200.75</v>
+        <v>181.79</v>
       </c>
       <c r="E20" s="53" t="s">
         <v>61</v>
@@ -9939,11 +9939,11 @@
         <v>0</v>
       </c>
       <c r="AI20" s="61">
-        <f>IF(AND(AI16=0,AI17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI16*AI17,0)))</f>
+        <f>IF(AND(AI16=1,AI17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI16&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI16*AI17,0)))</f>
         <v>0</v>
       </c>
       <c r="AJ20" s="61">
-        <f>IF(AND(AJ16=0,AJ17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ16*AJ17,0)))</f>
+        <f>IF(AND(AJ16=1,AJ17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ16&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ16*AJ17,0)))</f>
         <v>0</v>
       </c>
       <c r="AK20" s="62">
@@ -9955,19 +9955,19 @@
         <v>0</v>
       </c>
       <c r="AM20" s="61">
-        <f>IF(AND(AM16=0,AM17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM16*AM17,0)))</f>
+        <f>IF(AND(AM16=1,AM17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM16&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM16*AM17,0)))</f>
         <v>0</v>
       </c>
       <c r="AN20" s="61">
-        <f>IF(AND(AN16=0,AN17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN16*AN17,0)))</f>
+        <f>IF(AND(AN16=1,AN17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN16&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN16*AN17,0)))</f>
         <v>0</v>
       </c>
       <c r="AO20" s="61">
-        <f>IF(AND(AO16=0,AO17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO16*AO17,0)))</f>
+        <f>IF(AND(AO16=1,AO17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO16&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO16*AO17,0)))</f>
         <v>0</v>
       </c>
       <c r="AP20" s="63">
-        <f>IF(AND(AP16=0,AP17=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP16*AP17,0)))</f>
+        <f>IF(AND(AP16=1,AP17=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP16&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP16*AP17,0)))</f>
         <v>0</v>
       </c>
       <c r="OU20" s="28" t="s">
@@ -9975,7 +9975,7 @@
       </c>
     </row>
     <row r="21" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A21" s="72"/>
+      <c r="A21" s="43"/>
       <c r="B21" s="44"/>
       <c r="C21" s="65">
         <f>I15*D21</f>
@@ -10145,7 +10145,7 @@
       </c>
       <c r="C23" s="45">
         <f>J23</f>
-        <v>33109.96000000001</v>
+        <v>28354.399999999998</v>
       </c>
       <c r="D23" s="46"/>
       <c r="E23" s="46"/>
@@ -10167,7 +10167,7 @@
       </c>
       <c r="J23" s="48">
         <f>C26+C27+C28</f>
-        <v>33109.96000000001</v>
+        <v>28354.399999999998</v>
       </c>
       <c r="K23" s="49"/>
       <c r="L23" s="50"/>
@@ -10436,11 +10436,11 @@
       <c r="B26" s="44"/>
       <c r="C26" s="59">
         <f>F23*N(D26)</f>
-        <v>22421.120000000003</v>
+        <v>19296.239999999998</v>
       </c>
       <c r="D26" s="59">
         <f>IF(TRIM(B23)="","No rate",IFERROR(INDEX('Rate Tables'!C$7:C$161,MATCH(B23,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>105.76</v>
+        <v>91.02</v>
       </c>
       <c r="E26" s="53" t="s">
         <v>59</v>
@@ -10587,11 +10587,11 @@
       <c r="B27" s="44"/>
       <c r="C27" s="64">
         <f>G23*N(D27)</f>
-        <v>6325.88</v>
+        <v>5376.8</v>
       </c>
       <c r="D27" s="64">
         <f>IF(TRIM(B23)="","No rate",IFERROR(INDEX('Rate Tables'!D$7:D$161,MATCH(B23,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>143.77</v>
+        <v>122.2</v>
       </c>
       <c r="E27" s="53" t="s">
         <v>60</v>
@@ -10738,11 +10738,11 @@
       <c r="B28" s="44"/>
       <c r="C28" s="59">
         <f>H23*N(D28)</f>
-        <v>4362.96</v>
+        <v>3681.3599999999997</v>
       </c>
       <c r="D28" s="59">
         <f>IF(TRIM(B23)="","No rate",IFERROR(INDEX('Rate Tables'!E$7:E$161,MATCH(B23,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>181.79</v>
+        <v>153.39</v>
       </c>
       <c r="E28" s="53" t="s">
         <v>61</v>
@@ -11047,25 +11047,25 @@
       <c r="AP30" s="71"/>
     </row>
     <row r="31" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A31" s="72" t="s">
-        <v>63</v>
+      <c r="A31" s="43" t="s">
+        <v>54</v>
       </c>
       <c r="B31" s="44" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C31" s="45">
         <f>J31</f>
-        <v>28033.48</v>
+        <v>36191.68</v>
       </c>
       <c r="D31" s="46"/>
       <c r="E31" s="46"/>
       <c r="F31" s="47">
         <f>SUM(K34:AP34)</f>
-        <v>164</v>
+        <v>192</v>
       </c>
       <c r="G31" s="47">
         <f>SUM(K35:AP35)</f>
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="H31" s="47">
         <f>SUM(K36:AP36)</f>
@@ -11077,7 +11077,7 @@
       </c>
       <c r="J31" s="48">
         <f>C34+C35+C36</f>
-        <v>28033.48</v>
+        <v>36191.68</v>
       </c>
       <c r="K31" s="49"/>
       <c r="L31" s="50"/>
@@ -11112,11 +11112,11 @@
       <c r="AO31" s="50"/>
       <c r="AP31" s="52"/>
       <c r="OU31" s="28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A32" s="72"/>
+      <c r="A32" s="43"/>
       <c r="B32" s="44"/>
       <c r="C32" s="45"/>
       <c r="D32" s="46"/>
@@ -11201,10 +11201,10 @@
         <v>1</v>
       </c>
       <c r="AI32" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ32" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AK32" s="56">
         <v>0</v>
@@ -11213,23 +11213,23 @@
         <v>0</v>
       </c>
       <c r="AM32" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN32" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO32" s="55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP32" s="57">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="OU32" s="58" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A33" s="72"/>
+      <c r="A33" s="43"/>
       <c r="B33" s="44"/>
       <c r="C33" s="45"/>
       <c r="D33" s="46"/>
@@ -11314,10 +11314,10 @@
         <v>12</v>
       </c>
       <c r="AI33" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AJ33" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AK33" s="56">
         <v>0</v>
@@ -11326,31 +11326,31 @@
         <v>0</v>
       </c>
       <c r="AM33" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AN33" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AO33" s="55">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AP33" s="57">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="OU33" s="58" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A34" s="72"/>
+      <c r="A34" s="43"/>
       <c r="B34" s="44"/>
       <c r="C34" s="59">
         <f>F31*N(D34)</f>
-        <v>17344.64</v>
+        <v>21354.239999999998</v>
       </c>
       <c r="D34" s="59">
         <f>IF(TRIM(B31)="","No rate",IFERROR(INDEX('Rate Tables'!C$7:C$161,MATCH(B31,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>105.76</v>
+        <v>111.22</v>
       </c>
       <c r="E34" s="53" t="s">
         <v>59</v>
@@ -11361,147 +11361,147 @@
       <c r="I34" s="47"/>
       <c r="J34" s="48"/>
       <c r="K34" s="60">
-        <f>IF(AND(K32=1,K33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MIN(IF('_JobDays'!A3,8,10),K33)*K32)),MAX(0,40*MAX(1,K32)-(0))))</f>
+        <f>IF(AND(K32=1,K33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,0,IF('_JobDays'!A3,MIN(8,K33)*K32,K32*K33)))),MAX(0,40*MAX(1,K32)-(0))))</f>
         <v>8</v>
       </c>
       <c r="L34" s="61">
-        <f>IF(AND(L32=1,L33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MIN(IF('_JobDays'!B3,8,10),L33)*L32)),MAX(0,40*MAX(1,L32)-(K34))))</f>
+        <f>IF(AND(L32=1,L33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,0,IF('_JobDays'!B3,MIN(8,L33)*L32,L32*L33)))),MAX(0,40*MAX(1,L32)-(K34))))</f>
         <v>8</v>
       </c>
       <c r="M34" s="61">
-        <f>IF(AND(M32=1,M33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MIN(IF('_JobDays'!C3,8,10),M33)*M32)),MAX(0,40*MAX(1,M32)-(K34+L34))))</f>
+        <f>IF(AND(M32=1,M33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,0,IF('_JobDays'!C3,MIN(8,M33)*M32,M32*M33)))),MAX(0,40*MAX(1,M32)-(K34+L34))))</f>
         <v>8</v>
       </c>
       <c r="N34" s="61">
-        <f>IF(AND(N32=1,N33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MIN(IF('_JobDays'!D3,8,10),N33)*N32)),MAX(0,40*MAX(1,N32)-(K34+L34+M34))))</f>
+        <f>IF(AND(N32=1,N33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,0,IF('_JobDays'!D3,MIN(8,N33)*N32,N32*N33)))),MAX(0,40*MAX(1,N32)-(K34+L34+M34))))</f>
         <v>8</v>
       </c>
       <c r="O34" s="61">
-        <f>IF(AND(O32=1,O33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MIN(IF('_JobDays'!E3,8,10),O33)*O32)),MAX(0,40*MAX(1,O32)-(K34+L34+M34+N34))))</f>
+        <f>IF(AND(O32=1,O33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,0,IF('_JobDays'!E3,MIN(8,O33)*O32,O32*O33)))),MAX(0,40*MAX(1,O32)-(K34+L34+M34+N34))))</f>
         <v>8</v>
       </c>
       <c r="P34" s="62">
-        <f>IF(AND(P32=0,P33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MIN(IF('_JobDays'!F3,8,10),P33)*P32)),MAX(0,40*MAX(1,P32)-(0))))</f>
+        <f>IF(AND(P32=0,P33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,0,IF('_JobDays'!F3,MIN(8,P33)*P32,P32*P33)))),MAX(0,40*MAX(1,P32)-(0))))</f>
         <v>0</v>
       </c>
       <c r="Q34" s="62">
-        <f>IF(AND(Q32=0,Q33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MIN(IF('_JobDays'!G3,8,10),Q33)*Q32)),MAX(0,40*MAX(1,Q32)-(P34))))</f>
+        <f>IF(AND(Q32=0,Q33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,0,IF('_JobDays'!G3,MIN(8,Q33)*Q32,Q32*Q33)))),MAX(0,40*MAX(1,Q32)-(P34))))</f>
         <v>0</v>
       </c>
       <c r="R34" s="61">
-        <f>IF(AND(R32=1,R33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MIN(IF('_JobDays'!H3,8,10),R33)*R32)),MAX(0,40*MAX(1,R32)-(0))))</f>
+        <f>IF(AND(R32=1,R33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,0,IF('_JobDays'!H3,MIN(8,R33)*R32,R32*R33)))),MAX(0,40*MAX(1,R32)-(0))))</f>
         <v>8</v>
       </c>
       <c r="S34" s="61">
-        <f>IF(AND(S32=1,S33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MIN(IF('_JobDays'!I3,8,10),S33)*S32)),MAX(0,40*MAX(1,S32)-(R34))))</f>
+        <f>IF(AND(S32=1,S33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,0,IF('_JobDays'!I3,MIN(8,S33)*S32,S32*S33)))),MAX(0,40*MAX(1,S32)-(R34))))</f>
         <v>8</v>
       </c>
       <c r="T34" s="61">
-        <f>IF(AND(T32=1,T33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MIN(IF('_JobDays'!J3,8,10),T33)*T32)),MAX(0,40*MAX(1,T32)-(R34+S34))))</f>
+        <f>IF(AND(T32=1,T33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,0,IF('_JobDays'!J3,MIN(8,T33)*T32,T32*T33)))),MAX(0,40*MAX(1,T32)-(R34+S34))))</f>
         <v>8</v>
       </c>
       <c r="U34" s="61">
-        <f>IF(AND(U32=1,U33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MIN(IF('_JobDays'!K3,8,10),U33)*U32)),MAX(0,40*MAX(1,U32)-(0))))</f>
-        <v>10</v>
+        <f>IF(AND(U32=1,U33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,0,IF('_JobDays'!K3,MIN(8,U33)*U32,U32*U33)))),MAX(0,40*MAX(1,U32)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="V34" s="61">
-        <f>IF(AND(V32=1,V33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MIN(IF('_JobDays'!L3,8,10),V33)*V32)),MAX(0,40*MAX(1,V32)-(U34))))</f>
-        <v>10</v>
+        <f>IF(AND(V32=1,V33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,0,IF('_JobDays'!L3,MIN(8,V33)*V32,V32*V33)))),MAX(0,40*MAX(1,V32)-(U34))))</f>
+        <v>8</v>
       </c>
       <c r="W34" s="62">
-        <f>IF(AND(W32=1,W33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MIN(IF('_JobDays'!M3,8,10),W33)*W32)),MAX(0,40*MAX(1,W32)-(U34+V34))))</f>
-        <v>10</v>
+        <f>IF(AND(W32=1,W33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,0,IF('_JobDays'!M3,MIN(8,W33)*W32,W32*W33)))),MAX(0,40*MAX(1,W32)-(U34+V34))))</f>
+        <v>0</v>
       </c>
       <c r="X34" s="62">
-        <f>IF(AND(X32=1,X33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MIN(IF('_JobDays'!N3,8,10),X33)*X32)),MAX(0,40*MAX(1,X32)-(U34+V34+W34))))</f>
+        <f>IF(AND(X32=1,X33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,0,IF('_JobDays'!N3,MIN(8,X33)*X32,X32*X33)))),MAX(0,40*MAX(1,X32)-(U34+V34+W34))))</f>
         <v>0</v>
       </c>
       <c r="Y34" s="61">
-        <f>IF(AND(Y32=1,Y33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MIN(IF('_JobDays'!O3,8,10),Y33)*Y32)),MAX(0,40*MAX(1,Y32)-(0))))</f>
-        <v>10</v>
+        <f>IF(AND(Y32=1,Y33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,0,IF('_JobDays'!O3,MIN(8,Y33)*Y32,Y32*Y33)))),MAX(0,40*MAX(1,Y32)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="Z34" s="61">
-        <f>IF(AND(Z32=1,Z33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MIN(IF('_JobDays'!P3,8,10),Z33)*Z32)),MAX(0,40*MAX(1,Z32)-(Y34))))</f>
-        <v>10</v>
+        <f>IF(AND(Z32=1,Z33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,0,IF('_JobDays'!P3,MIN(8,Z33)*Z32,Z32*Z33)))),MAX(0,40*MAX(1,Z32)-(Y34))))</f>
+        <v>8</v>
       </c>
       <c r="AA34" s="61">
-        <f>IF(AND(AA32=1,AA33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MIN(IF('_JobDays'!Q3,8,10),AA33)*AA32)),MAX(0,40*MAX(1,AA32)-(Y34+Z34))))</f>
-        <v>10</v>
+        <f>IF(AND(AA32=1,AA33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,0,IF('_JobDays'!Q3,MIN(8,AA33)*AA32,AA32*AA33)))),MAX(0,40*MAX(1,AA32)-(Y34+Z34))))</f>
+        <v>8</v>
       </c>
       <c r="AB34" s="61">
-        <f>IF(AND(AB32=1,AB33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MIN(IF('_JobDays'!R3,8,10),AB33)*AB32)),MAX(0,40*MAX(1,AB32)-(Y34+Z34+AA34))))</f>
-        <v>10</v>
+        <f>IF(AND(AB32=1,AB33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,0,IF('_JobDays'!R3,MIN(8,AB33)*AB32,AB32*AB33)))),MAX(0,40*MAX(1,AB32)-(Y34+Z34+AA34))))</f>
+        <v>8</v>
       </c>
       <c r="AC34" s="61">
-        <f>IF(AND(AC32=1,AC33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MIN(IF('_JobDays'!S3,8,10),AC33)*AC32)),MAX(0,40*MAX(1,AC32)-(Y34+Z34+AA34+AB34))))</f>
-        <v>0</v>
+        <f>IF(AND(AC32=1,AC33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,0,IF('_JobDays'!S3,MIN(8,AC33)*AC32,AC32*AC33)))),MAX(0,40*MAX(1,AC32)-(Y34+Z34+AA34+AB34))))</f>
+        <v>8</v>
       </c>
       <c r="AD34" s="62">
-        <f>IF(AND(AD32=1,AD33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MIN(IF('_JobDays'!T3,8,10),AD33)*AD32)),MAX(0,40*MAX(1,AD32)-(Y34+Z34+AA34+AB34+AC34))))</f>
+        <f>IF(AND(AD32=1,AD33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,0,IF('_JobDays'!T3,MIN(8,AD33)*AD32,AD32*AD33)))),MAX(0,40*MAX(1,AD32)-(Y34+Z34+AA34+AB34+AC34))))</f>
         <v>0</v>
       </c>
       <c r="AE34" s="62">
-        <f>IF(AND(AE32=1,AE33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MIN(IF('_JobDays'!U3,8,10),AE33)*AE32)),MAX(0,40*MAX(1,AE32)-(Y34+Z34+AA34+AB34+AC34+AD34))))</f>
+        <f>IF(AND(AE32=1,AE33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,0,IF('_JobDays'!U3,MIN(8,AE33)*AE32,AE32*AE33)))),MAX(0,40*MAX(1,AE32)-(Y34+Z34+AA34+AB34+AC34+AD34))))</f>
         <v>0</v>
       </c>
       <c r="AF34" s="61">
-        <f>IF(AND(AF32=1,AF33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MIN(IF('_JobDays'!V3,8,10),AF33)*AF32)),MAX(0,40*MAX(1,AF32)-(0))))</f>
-        <v>10</v>
+        <f>IF(AND(AF32=1,AF33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,0,IF('_JobDays'!V3,MIN(8,AF33)*AF32,AF32*AF33)))),MAX(0,40*MAX(1,AF32)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="AG34" s="61">
-        <f>IF(AND(AG32=1,AG33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MIN(IF('_JobDays'!W3,8,10),AG33)*AG32)),MAX(0,40*MAX(1,AG32)-(AF34))))</f>
-        <v>10</v>
+        <f>IF(AND(AG32=1,AG33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,0,IF('_JobDays'!W3,MIN(8,AG33)*AG32,AG32*AG33)))),MAX(0,40*MAX(1,AG32)-(AF34))))</f>
+        <v>8</v>
       </c>
       <c r="AH34" s="61">
-        <f>IF(AND(AH32=1,AH33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MIN(IF('_JobDays'!X3,8,10),AH33)*AH32)),MAX(0,40*MAX(1,AH32)-(AF34+AG34))))</f>
-        <v>10</v>
+        <f>IF(AND(AH32=1,AH33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,0,IF('_JobDays'!X3,MIN(8,AH33)*AH32,AH32*AH33)))),MAX(0,40*MAX(1,AH32)-(AF34+AG34))))</f>
+        <v>8</v>
       </c>
       <c r="AI34" s="61">
-        <f>IF(AND(AI32=0,AI33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI33)*AI32)),MAX(0,40*MAX(1,AI32)-(0))))</f>
-        <v>0</v>
+        <f>IF(AND(AI32=1,AI33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,0,IF('_JobDays'!Y3,MIN(8,AI33)*AI32,AI32*AI33)))),MAX(0,40*MAX(1,AI32)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="AJ34" s="61">
-        <f>IF(AND(AJ32=0,AJ33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ33)*AJ32)),MAX(0,40*MAX(1,AJ32)-(AI34))))</f>
-        <v>0</v>
+        <f>IF(AND(AJ32=1,AJ33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,0,IF('_JobDays'!Z3,MIN(8,AJ33)*AJ32,AJ32*AJ33)))),MAX(0,40*MAX(1,AJ32)-(AI34))))</f>
+        <v>8</v>
       </c>
       <c r="AK34" s="62">
-        <f>IF(AND(AK32=0,AK33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK33)*AK32)),MAX(0,40*MAX(1,AK32)-(AI34+AJ34))))</f>
+        <f>IF(AND(AK32=0,AK33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,0,IF('_JobDays'!AA3,MIN(8,AK33)*AK32,AK32*AK33)))),MAX(0,40*MAX(1,AK32)-(0))))</f>
         <v>0</v>
       </c>
       <c r="AL34" s="62">
-        <f>IF(AND(AL32=0,AL33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL33)*AL32)),MAX(0,40*MAX(1,AL32)-(AI34+AJ34+AK34))))</f>
+        <f>IF(AND(AL32=0,AL33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,0,IF('_JobDays'!AB3,MIN(8,AL33)*AL32,AL32*AL33)))),MAX(0,40*MAX(1,AL32)-(AK34))))</f>
         <v>0</v>
       </c>
       <c r="AM34" s="61">
-        <f>IF(AND(AM32=0,AM33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM33)*AM32)),MAX(0,40*MAX(1,AM32)-(0))))</f>
-        <v>0</v>
+        <f>IF(AND(AM32=1,AM33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,0,IF('_JobDays'!AC3,MIN(8,AM33)*AM32,AM32*AM33)))),MAX(0,40*MAX(1,AM32)-(0))))</f>
+        <v>8</v>
       </c>
       <c r="AN34" s="61">
-        <f>IF(AND(AN32=0,AN33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN33)*AN32)),MAX(0,40*MAX(1,AN32)-(AM34))))</f>
-        <v>0</v>
+        <f>IF(AND(AN32=1,AN33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,0,IF('_JobDays'!AD3,MIN(8,AN33)*AN32,AN32*AN33)))),MAX(0,40*MAX(1,AN32)-(AM34))))</f>
+        <v>8</v>
       </c>
       <c r="AO34" s="61">
-        <f>IF(AND(AO32=0,AO33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO33)*AO32)),MAX(0,40*MAX(1,AO32)-(AM34+AN34))))</f>
-        <v>0</v>
+        <f>IF(AND(AO32=1,AO33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,0,IF('_JobDays'!AE3,MIN(8,AO33)*AO32,AO32*AO33)))),MAX(0,40*MAX(1,AO32)-(AM34+AN34))))</f>
+        <v>8</v>
       </c>
       <c r="AP34" s="63">
-        <f>IF(AND(AP32=0,AP33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP33)*AP32)),MAX(0,40*MAX(1,AP32)-(AM34+AN34+AO34))))</f>
-        <v>0</v>
+        <f>IF(AND(AP32=1,AP33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,0,IF('_JobDays'!AF3,MIN(8,AP33)*AP32,AP32*AP33)))),MAX(0,40*MAX(1,AP32)-(AM34+AN34+AO34))))</f>
+        <v>8</v>
       </c>
       <c r="OU34" s="28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A35" s="72"/>
+      <c r="A35" s="43"/>
       <c r="B35" s="44"/>
       <c r="C35" s="64">
         <f>G31*N(D35)</f>
-        <v>6325.88</v>
+        <v>10003.84</v>
       </c>
       <c r="D35" s="64">
         <f>IF(TRIM(B31)="","No rate",IFERROR(INDEX('Rate Tables'!D$7:D$161,MATCH(B31,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>143.77</v>
+        <v>156.31</v>
       </c>
       <c r="E35" s="53" t="s">
         <v>60</v>
@@ -11512,147 +11512,147 @@
       <c r="I35" s="47"/>
       <c r="J35" s="48"/>
       <c r="K35" s="60">
-        <f>IF(AND(K32=1,K33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),0,IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MAX(0,K33-(IF('_JobDays'!A3,8,10)))*K32))+((IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MIN(IF('_JobDays'!A3,8,10),K33)*K32)))-MIN(IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MIN(IF('_JobDays'!A3,8,10),K33)*K32)),MAX(0,40*MAX(1,K32)-(0)))))</f>
+        <f>IF(AND(K32=1,K33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),0,IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,K32*K33,IF('_JobDays'!A3,MAX(0,K33-8)*K32,0))))+((IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,0,IF('_JobDays'!A3,MIN(8,K33)*K32,K32*K33)))))-MIN(IF(OR(K32&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,0,IF('_JobDays'!A3,MIN(8,K33)*K32,K32*K33)))),MAX(0,40*MAX(1,K32)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="L35" s="61">
-        <f>IF(AND(L32=1,L33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),0,IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MAX(0,L33-(IF('_JobDays'!B3,8,10)))*L32))+((IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MIN(IF('_JobDays'!B3,8,10),L33)*L32)))-MIN(IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MIN(IF('_JobDays'!B3,8,10),L33)*L32)),MAX(0,40*MAX(1,L32)-(K34)))))</f>
+        <f>IF(AND(L32=1,L33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),0,IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L32*L33,IF('_JobDays'!B3,MAX(0,L33-8)*L32,0))))+((IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,0,IF('_JobDays'!B3,MIN(8,L33)*L32,L32*L33)))))-MIN(IF(OR(L32&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,0,IF('_JobDays'!B3,MIN(8,L33)*L32,L32*L33)))),MAX(0,40*MAX(1,L32)-(K34)))))</f>
         <v>0</v>
       </c>
       <c r="M35" s="61">
-        <f>IF(AND(M32=1,M33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),0,IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MAX(0,M33-(IF('_JobDays'!C3,8,10)))*M32))+((IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MIN(IF('_JobDays'!C3,8,10),M33)*M32)))-MIN(IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MIN(IF('_JobDays'!C3,8,10),M33)*M32)),MAX(0,40*MAX(1,M32)-(K34+L34)))))</f>
+        <f>IF(AND(M32=1,M33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),0,IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,M32*M33,IF('_JobDays'!C3,MAX(0,M33-8)*M32,0))))+((IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,0,IF('_JobDays'!C3,MIN(8,M33)*M32,M32*M33)))))-MIN(IF(OR(M32&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,0,IF('_JobDays'!C3,MIN(8,M33)*M32,M32*M33)))),MAX(0,40*MAX(1,M32)-(K34+L34)))))</f>
         <v>0</v>
       </c>
       <c r="N35" s="61">
-        <f>IF(AND(N32=1,N33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),0,IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MAX(0,N33-(IF('_JobDays'!D3,8,10)))*N32))+((IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MIN(IF('_JobDays'!D3,8,10),N33)*N32)))-MIN(IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MIN(IF('_JobDays'!D3,8,10),N33)*N32)),MAX(0,40*MAX(1,N32)-(K34+L34+M34)))))</f>
+        <f>IF(AND(N32=1,N33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),0,IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,N32*N33,IF('_JobDays'!D3,MAX(0,N33-8)*N32,0))))+((IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,0,IF('_JobDays'!D3,MIN(8,N33)*N32,N32*N33)))))-MIN(IF(OR(N32&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,0,IF('_JobDays'!D3,MIN(8,N33)*N32,N32*N33)))),MAX(0,40*MAX(1,N32)-(K34+L34+M34)))))</f>
         <v>0</v>
       </c>
       <c r="O35" s="61">
-        <f>IF(AND(O32=1,O33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),0,IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MAX(0,O33-(IF('_JobDays'!E3,8,10)))*O32))+((IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MIN(IF('_JobDays'!E3,8,10),O33)*O32)))-MIN(IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MIN(IF('_JobDays'!E3,8,10),O33)*O32)),MAX(0,40*MAX(1,O32)-(K34+L34+M34+N34)))))</f>
+        <f>IF(AND(O32=1,O33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),0,IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,O32*O33,IF('_JobDays'!E3,MAX(0,O33-8)*O32,0))))+((IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,0,IF('_JobDays'!E3,MIN(8,O33)*O32,O32*O33)))))-MIN(IF(OR(O32&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,0,IF('_JobDays'!E3,MIN(8,O33)*O32,O32*O33)))),MAX(0,40*MAX(1,O32)-(K34+L34+M34+N34)))))</f>
         <v>0</v>
       </c>
       <c r="P35" s="62">
-        <f>IF(AND(P32=0,P33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MAX(0,P33-(IF('_JobDays'!F3,8,10)))*P32))+((IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MIN(IF('_JobDays'!F3,8,10),P33)*P32)))-MIN(IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MIN(IF('_JobDays'!F3,8,10),P33)*P32)),MAX(0,40*MAX(1,P32)-(0)))))</f>
+        <f>IF(AND(P32=0,P33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,P32*P33,IF('_JobDays'!F3,MAX(0,P33-8)*P32,0))))+((IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,0,IF('_JobDays'!F3,MIN(8,P33)*P32,P32*P33)))))-MIN(IF(OR(P32&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,0,IF('_JobDays'!F3,MIN(8,P33)*P32,P32*P33)))),MAX(0,40*MAX(1,P32)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="Q35" s="62">
-        <f>IF(AND(Q32=0,Q33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MAX(0,Q33-(IF('_JobDays'!G3,8,10)))*Q32))+((IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MIN(IF('_JobDays'!G3,8,10),Q33)*Q32)))-MIN(IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MIN(IF('_JobDays'!G3,8,10),Q33)*Q32)),MAX(0,40*MAX(1,Q32)-(P34)))))</f>
+        <f>IF(AND(Q32=0,Q33=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,Q32*Q33,IF('_JobDays'!G3,MAX(0,Q33-8)*Q32,0))))+((IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,0,IF('_JobDays'!G3,MIN(8,Q33)*Q32,Q32*Q33)))))-MIN(IF(OR(Q32&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,0,IF('_JobDays'!G3,MIN(8,Q33)*Q32,Q32*Q33)))),MAX(0,40*MAX(1,Q32)-(P34)))))</f>
         <v>0</v>
       </c>
       <c r="R35" s="61">
-        <f>IF(AND(R32=1,R33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),0,IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MAX(0,R33-(IF('_JobDays'!H3,8,10)))*R32))+((IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MIN(IF('_JobDays'!H3,8,10),R33)*R32)))-MIN(IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MIN(IF('_JobDays'!H3,8,10),R33)*R32)),MAX(0,40*MAX(1,R32)-(0)))))</f>
+        <f>IF(AND(R32=1,R33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),0,IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R32*R33,IF('_JobDays'!H3,MAX(0,R33-8)*R32,0))))+((IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,0,IF('_JobDays'!H3,MIN(8,R33)*R32,R32*R33)))))-MIN(IF(OR(R32&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,0,IF('_JobDays'!H3,MIN(8,R33)*R32,R32*R33)))),MAX(0,40*MAX(1,R32)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="S35" s="61">
-        <f>IF(AND(S32=1,S33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),0,IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MAX(0,S33-(IF('_JobDays'!I3,8,10)))*S32))+((IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MIN(IF('_JobDays'!I3,8,10),S33)*S32)))-MIN(IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MIN(IF('_JobDays'!I3,8,10),S33)*S32)),MAX(0,40*MAX(1,S32)-(R34)))))</f>
+        <f>IF(AND(S32=1,S33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),0,IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,S32*S33,IF('_JobDays'!I3,MAX(0,S33-8)*S32,0))))+((IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,0,IF('_JobDays'!I3,MIN(8,S33)*S32,S32*S33)))))-MIN(IF(OR(S32&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,0,IF('_JobDays'!I3,MIN(8,S33)*S32,S32*S33)))),MAX(0,40*MAX(1,S32)-(R34)))))</f>
         <v>0</v>
       </c>
       <c r="T35" s="61">
-        <f>IF(AND(T32=1,T33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),0,IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MAX(0,T33-(IF('_JobDays'!J3,8,10)))*T32))+((IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MIN(IF('_JobDays'!J3,8,10),T33)*T32)))-MIN(IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MIN(IF('_JobDays'!J3,8,10),T33)*T32)),MAX(0,40*MAX(1,T32)-(R34+S34)))))</f>
+        <f>IF(AND(T32=1,T33=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),0,IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,T32*T33,IF('_JobDays'!J3,MAX(0,T33-8)*T32,0))))+((IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,0,IF('_JobDays'!J3,MIN(8,T33)*T32,T32*T33)))))-MIN(IF(OR(T32&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,0,IF('_JobDays'!J3,MIN(8,T33)*T32,T32*T33)))),MAX(0,40*MAX(1,T32)-(R34+S34)))))</f>
         <v>0</v>
       </c>
       <c r="U35" s="61">
-        <f>IF(AND(U32=1,U33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),2,IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MAX(0,U33-(IF('_JobDays'!K3,8,10)))*U32))+((IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MIN(IF('_JobDays'!K3,8,10),U33)*U32)))-MIN(IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MIN(IF('_JobDays'!K3,8,10),U33)*U32)),MAX(0,40*MAX(1,U32)-(0)))))</f>
-        <v>2</v>
+        <f>IF(AND(U32=1,U33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),4,IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,U32*U33,IF('_JobDays'!K3,MAX(0,U33-8)*U32,0))))+((IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,0,IF('_JobDays'!K3,MIN(8,U33)*U32,U32*U33)))))-MIN(IF(OR(U32&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,0,IF('_JobDays'!K3,MIN(8,U33)*U32,U32*U33)))),MAX(0,40*MAX(1,U32)-(0)))))</f>
+        <v>4</v>
       </c>
       <c r="V35" s="61">
-        <f>IF(AND(V32=1,V33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),2,IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MAX(0,V33-(IF('_JobDays'!L3,8,10)))*V32))+((IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MIN(IF('_JobDays'!L3,8,10),V33)*V32)))-MIN(IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MIN(IF('_JobDays'!L3,8,10),V33)*V32)),MAX(0,40*MAX(1,V32)-(U34)))))</f>
-        <v>2</v>
+        <f>IF(AND(V32=1,V33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),4,IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,V32*V33,IF('_JobDays'!L3,MAX(0,V33-8)*V32,0))))+((IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,0,IF('_JobDays'!L3,MIN(8,V33)*V32,V32*V33)))))-MIN(IF(OR(V32&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,0,IF('_JobDays'!L3,MIN(8,V33)*V32,V32*V33)))),MAX(0,40*MAX(1,V32)-(U34)))))</f>
+        <v>4</v>
       </c>
       <c r="W35" s="62">
-        <f>IF(AND(W32=1,W33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),2,IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MAX(0,W33-(IF('_JobDays'!M3,8,10)))*W32))+((IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MIN(IF('_JobDays'!M3,8,10),W33)*W32)))-MIN(IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MIN(IF('_JobDays'!M3,8,10),W33)*W32)),MAX(0,40*MAX(1,W32)-(U34+V34)))))</f>
-        <v>2</v>
+        <f>IF(AND(W32=1,W33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),12,IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,W32*W33,IF('_JobDays'!M3,MAX(0,W33-8)*W32,0))))+((IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,0,IF('_JobDays'!M3,MIN(8,W33)*W32,W32*W33)))))-MIN(IF(OR(W32&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,0,IF('_JobDays'!M3,MIN(8,W33)*W32,W32*W33)))),MAX(0,40*MAX(1,W32)-(U34+V34)))))</f>
+        <v>12</v>
       </c>
       <c r="X35" s="62">
-        <f>IF(AND(X32=1,X33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MAX(0,X33-(IF('_JobDays'!N3,8,10)))*X32))+((IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MIN(IF('_JobDays'!N3,8,10),X33)*X32)))-MIN(IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MIN(IF('_JobDays'!N3,8,10),X33)*X32)),MAX(0,40*MAX(1,X32)-(U34+V34+W34)))))</f>
+        <f>IF(AND(X32=1,X33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,X32*X33,IF('_JobDays'!N3,MAX(0,X33-8)*X32,0))))+((IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,0,IF('_JobDays'!N3,MIN(8,X33)*X32,X32*X33)))))-MIN(IF(OR(X32&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,0,IF('_JobDays'!N3,MIN(8,X33)*X32,X32*X33)))),MAX(0,40*MAX(1,X32)-(U34+V34+W34)))))</f>
         <v>0</v>
       </c>
       <c r="Y35" s="61">
-        <f>IF(AND(Y32=1,Y33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),2,IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MAX(0,Y33-(IF('_JobDays'!O3,8,10)))*Y32))+((IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MIN(IF('_JobDays'!O3,8,10),Y33)*Y32)))-MIN(IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MIN(IF('_JobDays'!O3,8,10),Y33)*Y32)),MAX(0,40*MAX(1,Y32)-(0)))))</f>
-        <v>2</v>
+        <f>IF(AND(Y32=1,Y33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),4,IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,Y32*Y33,IF('_JobDays'!O3,MAX(0,Y33-8)*Y32,0))))+((IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,0,IF('_JobDays'!O3,MIN(8,Y33)*Y32,Y32*Y33)))))-MIN(IF(OR(Y32&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,0,IF('_JobDays'!O3,MIN(8,Y33)*Y32,Y32*Y33)))),MAX(0,40*MAX(1,Y32)-(0)))))</f>
+        <v>4</v>
       </c>
       <c r="Z35" s="61">
-        <f>IF(AND(Z32=1,Z33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),2,IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MAX(0,Z33-(IF('_JobDays'!P3,8,10)))*Z32))+((IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MIN(IF('_JobDays'!P3,8,10),Z33)*Z32)))-MIN(IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MIN(IF('_JobDays'!P3,8,10),Z33)*Z32)),MAX(0,40*MAX(1,Z32)-(Y34)))))</f>
-        <v>2</v>
+        <f>IF(AND(Z32=1,Z33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),4,IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,Z32*Z33,IF('_JobDays'!P3,MAX(0,Z33-8)*Z32,0))))+((IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,0,IF('_JobDays'!P3,MIN(8,Z33)*Z32,Z32*Z33)))))-MIN(IF(OR(Z32&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,0,IF('_JobDays'!P3,MIN(8,Z33)*Z32,Z32*Z33)))),MAX(0,40*MAX(1,Z32)-(Y34)))))</f>
+        <v>4</v>
       </c>
       <c r="AA35" s="61">
-        <f>IF(AND(AA32=1,AA33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),2,IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MAX(0,AA33-(IF('_JobDays'!Q3,8,10)))*AA32))+((IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MIN(IF('_JobDays'!Q3,8,10),AA33)*AA32)))-MIN(IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MIN(IF('_JobDays'!Q3,8,10),AA33)*AA32)),MAX(0,40*MAX(1,AA32)-(Y34+Z34)))))</f>
-        <v>2</v>
+        <f>IF(AND(AA32=1,AA33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),4,IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,AA32*AA33,IF('_JobDays'!Q3,MAX(0,AA33-8)*AA32,0))))+((IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,0,IF('_JobDays'!Q3,MIN(8,AA33)*AA32,AA32*AA33)))))-MIN(IF(OR(AA32&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,0,IF('_JobDays'!Q3,MIN(8,AA33)*AA32,AA32*AA33)))),MAX(0,40*MAX(1,AA32)-(Y34+Z34)))))</f>
+        <v>4</v>
       </c>
       <c r="AB35" s="61">
-        <f>IF(AND(AB32=1,AB33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),2,IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MAX(0,AB33-(IF('_JobDays'!R3,8,10)))*AB32))+((IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MIN(IF('_JobDays'!R3,8,10),AB33)*AB32)))-MIN(IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MIN(IF('_JobDays'!R3,8,10),AB33)*AB32)),MAX(0,40*MAX(1,AB32)-(Y34+Z34+AA34)))))</f>
-        <v>2</v>
+        <f>IF(AND(AB32=1,AB33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),4,IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,AB32*AB33,IF('_JobDays'!R3,MAX(0,AB33-8)*AB32,0))))+((IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,0,IF('_JobDays'!R3,MIN(8,AB33)*AB32,AB32*AB33)))))-MIN(IF(OR(AB32&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,0,IF('_JobDays'!R3,MIN(8,AB33)*AB32,AB32*AB33)))),MAX(0,40*MAX(1,AB32)-(Y34+Z34+AA34)))))</f>
+        <v>4</v>
       </c>
       <c r="AC35" s="61">
-        <f>IF(AND(AC32=1,AC33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),12,IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MAX(0,AC33-(IF('_JobDays'!S3,8,10)))*AC32))+((IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MIN(IF('_JobDays'!S3,8,10),AC33)*AC32)))-MIN(IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MIN(IF('_JobDays'!S3,8,10),AC33)*AC32)),MAX(0,40*MAX(1,AC32)-(Y34+Z34+AA34+AB34)))))</f>
-        <v>12</v>
+        <f>IF(AND(AC32=1,AC33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),4,IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,AC32*AC33,IF('_JobDays'!S3,MAX(0,AC33-8)*AC32,0))))+((IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,0,IF('_JobDays'!S3,MIN(8,AC33)*AC32,AC32*AC33)))))-MIN(IF(OR(AC32&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,0,IF('_JobDays'!S3,MIN(8,AC33)*AC32,AC32*AC33)))),MAX(0,40*MAX(1,AC32)-(Y34+Z34+AA34+AB34)))))</f>
+        <v>4</v>
       </c>
       <c r="AD35" s="62">
-        <f>IF(AND(AD32=1,AD33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),12,IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MAX(0,AD33-(IF('_JobDays'!T3,8,10)))*AD32))+((IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MIN(IF('_JobDays'!T3,8,10),AD33)*AD32)))-MIN(IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MIN(IF('_JobDays'!T3,8,10),AD33)*AD32)),MAX(0,40*MAX(1,AD32)-(Y34+Z34+AA34+AB34+AC34)))))</f>
+        <f>IF(AND(AD32=1,AD33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),12,IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,AD32*AD33,IF('_JobDays'!T3,MAX(0,AD33-8)*AD32,0))))+((IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,0,IF('_JobDays'!T3,MIN(8,AD33)*AD32,AD32*AD33)))))-MIN(IF(OR(AD32&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,0,IF('_JobDays'!T3,MIN(8,AD33)*AD32,AD32*AD33)))),MAX(0,40*MAX(1,AD32)-(Y34+Z34+AA34+AB34+AC34)))))</f>
         <v>12</v>
       </c>
       <c r="AE35" s="62">
-        <f>IF(AND(AE32=1,AE33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MAX(0,AE33-(IF('_JobDays'!U3,8,10)))*AE32))+((IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MIN(IF('_JobDays'!U3,8,10),AE33)*AE32)))-MIN(IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MIN(IF('_JobDays'!U3,8,10),AE33)*AE32)),MAX(0,40*MAX(1,AE32)-(Y34+Z34+AA34+AB34+AC34+AD34)))))</f>
+        <f>IF(AND(AE32=1,AE33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,AE32*AE33,IF('_JobDays'!U3,MAX(0,AE33-8)*AE32,0))))+((IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,0,IF('_JobDays'!U3,MIN(8,AE33)*AE32,AE32*AE33)))))-MIN(IF(OR(AE32&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,0,IF('_JobDays'!U3,MIN(8,AE33)*AE32,AE32*AE33)))),MAX(0,40*MAX(1,AE32)-(Y34+Z34+AA34+AB34+AC34+AD34)))))</f>
         <v>0</v>
       </c>
       <c r="AF35" s="61">
-        <f>IF(AND(AF32=1,AF33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),2,IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MAX(0,AF33-(IF('_JobDays'!V3,8,10)))*AF32))+((IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MIN(IF('_JobDays'!V3,8,10),AF33)*AF32)))-MIN(IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MIN(IF('_JobDays'!V3,8,10),AF33)*AF32)),MAX(0,40*MAX(1,AF32)-(0)))))</f>
-        <v>2</v>
+        <f>IF(AND(AF32=1,AF33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),4,IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,AF32*AF33,IF('_JobDays'!V3,MAX(0,AF33-8)*AF32,0))))+((IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,0,IF('_JobDays'!V3,MIN(8,AF33)*AF32,AF32*AF33)))))-MIN(IF(OR(AF32&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,0,IF('_JobDays'!V3,MIN(8,AF33)*AF32,AF32*AF33)))),MAX(0,40*MAX(1,AF32)-(0)))))</f>
+        <v>4</v>
       </c>
       <c r="AG35" s="61">
-        <f>IF(AND(AG32=1,AG33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),2,IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MAX(0,AG33-(IF('_JobDays'!W3,8,10)))*AG32))+((IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MIN(IF('_JobDays'!W3,8,10),AG33)*AG32)))-MIN(IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MIN(IF('_JobDays'!W3,8,10),AG33)*AG32)),MAX(0,40*MAX(1,AG32)-(AF34)))))</f>
-        <v>2</v>
+        <f>IF(AND(AG32=1,AG33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),4,IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,AG32*AG33,IF('_JobDays'!W3,MAX(0,AG33-8)*AG32,0))))+((IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,0,IF('_JobDays'!W3,MIN(8,AG33)*AG32,AG32*AG33)))))-MIN(IF(OR(AG32&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,0,IF('_JobDays'!W3,MIN(8,AG33)*AG32,AG32*AG33)))),MAX(0,40*MAX(1,AG32)-(AF34)))))</f>
+        <v>4</v>
       </c>
       <c r="AH35" s="61">
-        <f>IF(AND(AH32=1,AH33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),2,IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MAX(0,AH33-(IF('_JobDays'!X3,8,10)))*AH32))+((IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MIN(IF('_JobDays'!X3,8,10),AH33)*AH32)))-MIN(IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MIN(IF('_JobDays'!X3,8,10),AH33)*AH32)),MAX(0,40*MAX(1,AH32)-(AF34+AG34)))))</f>
-        <v>2</v>
+        <f>IF(AND(AH32=1,AH33=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),4,IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,AH32*AH33,IF('_JobDays'!X3,MAX(0,AH33-8)*AH32,0))))+((IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,0,IF('_JobDays'!X3,MIN(8,AH33)*AH32,AH32*AH33)))))-MIN(IF(OR(AH32&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,0,IF('_JobDays'!X3,MIN(8,AH33)*AH32,AH32*AH33)))),MAX(0,40*MAX(1,AH32)-(AF34+AG34)))))</f>
+        <v>4</v>
       </c>
       <c r="AI35" s="61">
-        <f>IF(AND(AI32=0,AI33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MAX(0,AI33-(IF('_JobDays'!Y3,8,10)))*AI32))+((IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI33)*AI32)))-MIN(IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI33)*AI32)),MAX(0,40*MAX(1,AI32)-(0)))))</f>
+        <f>IF(AND(AI32=1,AI33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,AI32*AI33,IF('_JobDays'!Y3,MAX(0,AI33-8)*AI32,0))))+((IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,0,IF('_JobDays'!Y3,MIN(8,AI33)*AI32,AI32*AI33)))))-MIN(IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,0,IF('_JobDays'!Y3,MIN(8,AI33)*AI32,AI32*AI33)))),MAX(0,40*MAX(1,AI32)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AJ35" s="61">
-        <f>IF(AND(AJ32=0,AJ33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MAX(0,AJ33-(IF('_JobDays'!Z3,8,10)))*AJ32))+((IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ33)*AJ32)))-MIN(IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ33)*AJ32)),MAX(0,40*MAX(1,AJ32)-(AI34)))))</f>
+        <f>IF(AND(AJ32=1,AJ33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,AJ32*AJ33,IF('_JobDays'!Z3,MAX(0,AJ33-8)*AJ32,0))))+((IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,0,IF('_JobDays'!Z3,MIN(8,AJ33)*AJ32,AJ32*AJ33)))))-MIN(IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,0,IF('_JobDays'!Z3,MIN(8,AJ33)*AJ32,AJ32*AJ33)))),MAX(0,40*MAX(1,AJ32)-(AI34)))))</f>
         <v>0</v>
       </c>
       <c r="AK35" s="62">
-        <f>IF(AND(AK32=0,AK33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MAX(0,AK33-(IF('_JobDays'!AA3,8,10)))*AK32))+((IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK33)*AK32)))-MIN(IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK33)*AK32)),MAX(0,40*MAX(1,AK32)-(AI34+AJ34)))))</f>
+        <f>IF(AND(AK32=0,AK33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,AK32*AK33,IF('_JobDays'!AA3,MAX(0,AK33-8)*AK32,0))))+((IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,0,IF('_JobDays'!AA3,MIN(8,AK33)*AK32,AK32*AK33)))))-MIN(IF(OR(AK32&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,0,IF('_JobDays'!AA3,MIN(8,AK33)*AK32,AK32*AK33)))),MAX(0,40*MAX(1,AK32)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AL35" s="62">
-        <f>IF(AND(AL32=0,AL33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MAX(0,AL33-(IF('_JobDays'!AB3,8,10)))*AL32))+((IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL33)*AL32)))-MIN(IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL33)*AL32)),MAX(0,40*MAX(1,AL32)-(AI34+AJ34+AK34)))))</f>
+        <f>IF(AND(AL32=0,AL33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,AL32*AL33,IF('_JobDays'!AB3,MAX(0,AL33-8)*AL32,0))))+((IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,0,IF('_JobDays'!AB3,MIN(8,AL33)*AL32,AL32*AL33)))))-MIN(IF(OR(AL32&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,0,IF('_JobDays'!AB3,MIN(8,AL33)*AL32,AL32*AL33)))),MAX(0,40*MAX(1,AL32)-(AK34)))))</f>
         <v>0</v>
       </c>
       <c r="AM35" s="61">
-        <f>IF(AND(AM32=0,AM33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MAX(0,AM33-(IF('_JobDays'!AC3,8,10)))*AM32))+((IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM33)*AM32)))-MIN(IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM33)*AM32)),MAX(0,40*MAX(1,AM32)-(0)))))</f>
+        <f>IF(AND(AM32=1,AM33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,AM32*AM33,IF('_JobDays'!AC3,MAX(0,AM33-8)*AM32,0))))+((IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,0,IF('_JobDays'!AC3,MIN(8,AM33)*AM32,AM32*AM33)))))-MIN(IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,0,IF('_JobDays'!AC3,MIN(8,AM33)*AM32,AM32*AM33)))),MAX(0,40*MAX(1,AM32)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AN35" s="61">
-        <f>IF(AND(AN32=0,AN33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MAX(0,AN33-(IF('_JobDays'!AD3,8,10)))*AN32))+((IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN33)*AN32)))-MIN(IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN33)*AN32)),MAX(0,40*MAX(1,AN32)-(AM34)))))</f>
+        <f>IF(AND(AN32=1,AN33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,AN32*AN33,IF('_JobDays'!AD3,MAX(0,AN33-8)*AN32,0))))+((IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,0,IF('_JobDays'!AD3,MIN(8,AN33)*AN32,AN32*AN33)))))-MIN(IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,0,IF('_JobDays'!AD3,MIN(8,AN33)*AN32,AN32*AN33)))),MAX(0,40*MAX(1,AN32)-(AM34)))))</f>
         <v>0</v>
       </c>
       <c r="AO35" s="61">
-        <f>IF(AND(AO32=0,AO33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MAX(0,AO33-(IF('_JobDays'!AE3,8,10)))*AO32))+((IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO33)*AO32)))-MIN(IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO33)*AO32)),MAX(0,40*MAX(1,AO32)-(AM34+AN34)))))</f>
+        <f>IF(AND(AO32=1,AO33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,AO32*AO33,IF('_JobDays'!AE3,MAX(0,AO33-8)*AO32,0))))+((IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,0,IF('_JobDays'!AE3,MIN(8,AO33)*AO32,AO32*AO33)))))-MIN(IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,0,IF('_JobDays'!AE3,MIN(8,AO33)*AO32,AO32*AO33)))),MAX(0,40*MAX(1,AO32)-(AM34+AN34)))))</f>
         <v>0</v>
       </c>
       <c r="AP35" s="63">
-        <f>IF(AND(AP32=0,AP33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MAX(0,AP33-(IF('_JobDays'!AF3,8,10)))*AP32))+((IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP33)*AP32)))-MIN(IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP33)*AP32)),MAX(0,40*MAX(1,AP32)-(AM34+AN34+AO34)))))</f>
+        <f>IF(AND(AP32=1,AP33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,AP32*AP33,IF('_JobDays'!AF3,MAX(0,AP33-8)*AP32,0))))+((IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,0,IF('_JobDays'!AF3,MIN(8,AP33)*AP32,AP32*AP33)))))-MIN(IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,0,IF('_JobDays'!AF3,MIN(8,AP33)*AP32,AP32*AP33)))),MAX(0,40*MAX(1,AP32)-(AM34+AN34+AO34)))))</f>
         <v>0</v>
       </c>
       <c r="OU35" s="28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A36" s="72"/>
+      <c r="A36" s="43"/>
       <c r="B36" s="44"/>
       <c r="C36" s="59">
         <f>H31*N(D36)</f>
-        <v>4362.96</v>
+        <v>4833.6</v>
       </c>
       <c r="D36" s="59">
         <f>IF(TRIM(B31)="","No rate",IFERROR(INDEX('Rate Tables'!E$7:E$161,MATCH(B31,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>181.79</v>
+        <v>201.4</v>
       </c>
       <c r="E36" s="53" t="s">
         <v>61</v>
@@ -11759,11 +11759,11 @@
         <v>0</v>
       </c>
       <c r="AI36" s="61">
-        <f>IF(AND(AI32=0,AI33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI32*AI33,0)))</f>
+        <f>IF(AND(AI32=1,AI33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI32&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI32*AI33,0)))</f>
         <v>0</v>
       </c>
       <c r="AJ36" s="61">
-        <f>IF(AND(AJ32=0,AJ33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ32*AJ33,0)))</f>
+        <f>IF(AND(AJ32=1,AJ33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ32&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ32*AJ33,0)))</f>
         <v>0</v>
       </c>
       <c r="AK36" s="62">
@@ -11775,27 +11775,27 @@
         <v>0</v>
       </c>
       <c r="AM36" s="61">
-        <f>IF(AND(AM32=0,AM33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM32*AM33,0)))</f>
+        <f>IF(AND(AM32=1,AM33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM32&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM32*AM33,0)))</f>
         <v>0</v>
       </c>
       <c r="AN36" s="61">
-        <f>IF(AND(AN32=0,AN33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN32*AN33,0)))</f>
+        <f>IF(AND(AN32=1,AN33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN32&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN32*AN33,0)))</f>
         <v>0</v>
       </c>
       <c r="AO36" s="61">
-        <f>IF(AND(AO32=0,AO33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO32*AO33,0)))</f>
+        <f>IF(AND(AO32=1,AO33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO32&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO32*AO33,0)))</f>
         <v>0</v>
       </c>
       <c r="AP36" s="63">
-        <f>IF(AND(AP32=0,AP33=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP32*AP33,0)))</f>
+        <f>IF(AND(AP32=1,AP33=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP32&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP32*AP33,0)))</f>
         <v>0</v>
       </c>
       <c r="OU36" s="28" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A37" s="72"/>
+      <c r="A37" s="43"/>
       <c r="B37" s="44"/>
       <c r="C37" s="65">
         <f>I31*D37</f>
@@ -11909,7 +11909,7 @@
         <v>0</v>
       </c>
       <c r="OU37" s="58" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="38" ht="8" customHeight="1" spans="1:42" x14ac:dyDescent="0.25">
@@ -11957,21 +11957,21 @@
       <c r="AP38" s="71"/>
     </row>
     <row r="39" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A39" s="43" t="s">
-        <v>54</v>
+      <c r="A39" s="72" t="s">
+        <v>69</v>
       </c>
       <c r="B39" s="44" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="C39" s="45">
         <f>J39</f>
-        <v>28354.399999999998</v>
+        <v>30005.120000000003</v>
       </c>
       <c r="D39" s="46"/>
       <c r="E39" s="46"/>
       <c r="F39" s="47">
         <f>SUM(K42:AP42)</f>
-        <v>212</v>
+        <v>164</v>
       </c>
       <c r="G39" s="47">
         <f>SUM(K43:AP43)</f>
@@ -11987,7 +11987,7 @@
       </c>
       <c r="J39" s="48">
         <f>C42+C43+C44</f>
-        <v>28354.399999999998</v>
+        <v>30005.120000000003</v>
       </c>
       <c r="K39" s="49"/>
       <c r="L39" s="50"/>
@@ -12022,11 +12022,11 @@
       <c r="AO39" s="50"/>
       <c r="AP39" s="52"/>
       <c r="OU39" s="28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A40" s="43"/>
+      <c r="A40" s="72"/>
       <c r="B40" s="44"/>
       <c r="C40" s="45"/>
       <c r="D40" s="46"/>
@@ -12111,10 +12111,10 @@
         <v>1</v>
       </c>
       <c r="AI40" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ40" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK40" s="56">
         <v>0</v>
@@ -12123,23 +12123,23 @@
         <v>0</v>
       </c>
       <c r="AM40" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN40" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO40" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP40" s="57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="OU40" s="58" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A41" s="43"/>
+      <c r="A41" s="72"/>
       <c r="B41" s="44"/>
       <c r="C41" s="45"/>
       <c r="D41" s="46"/>
@@ -12224,10 +12224,10 @@
         <v>12</v>
       </c>
       <c r="AI41" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AJ41" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AK41" s="56">
         <v>0</v>
@@ -12236,31 +12236,31 @@
         <v>0</v>
       </c>
       <c r="AM41" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AN41" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AO41" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AP41" s="57">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="OU41" s="58" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A42" s="43"/>
+      <c r="A42" s="72"/>
       <c r="B42" s="44"/>
       <c r="C42" s="59">
         <f>F39*N(D42)</f>
-        <v>19296.239999999998</v>
+        <v>18313.88</v>
       </c>
       <c r="D42" s="59">
         <f>IF(TRIM(B39)="","No rate",IFERROR(INDEX('Rate Tables'!C$7:C$161,MATCH(B39,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>91.02</v>
+        <v>111.67</v>
       </c>
       <c r="E42" s="53" t="s">
         <v>59</v>
@@ -12367,51 +12367,51 @@
         <v>10</v>
       </c>
       <c r="AI42" s="61">
-        <f>IF(AND(AI40=1,AI41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI41)*AI40)),MAX(0,40*MAX(1,AI40)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(AI40=0,AI41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI41)*AI40)),MAX(0,40*MAX(1,AI40)-(0))))</f>
+        <v>0</v>
       </c>
       <c r="AJ42" s="61">
-        <f>IF(AND(AJ40=1,AJ41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ41)*AJ40)),MAX(0,40*MAX(1,AJ40)-(AI42))))</f>
-        <v>8</v>
+        <f>IF(AND(AJ40=0,AJ41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ41)*AJ40)),MAX(0,40*MAX(1,AJ40)-(AI42))))</f>
+        <v>0</v>
       </c>
       <c r="AK42" s="62">
-        <f>IF(AND(AK40=0,AK41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK41)*AK40)),MAX(0,40*MAX(1,AK40)-(0))))</f>
+        <f>IF(AND(AK40=0,AK41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK41)*AK40)),MAX(0,40*MAX(1,AK40)-(AI42+AJ42))))</f>
         <v>0</v>
       </c>
       <c r="AL42" s="62">
-        <f>IF(AND(AL40=0,AL41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL41)*AL40)),MAX(0,40*MAX(1,AL40)-(AK42))))</f>
+        <f>IF(AND(AL40=0,AL41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL41)*AL40)),MAX(0,40*MAX(1,AL40)-(AI42+AJ42+AK42))))</f>
         <v>0</v>
       </c>
       <c r="AM42" s="61">
-        <f>IF(AND(AM40=1,AM41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM41)*AM40)),MAX(0,40*MAX(1,AM40)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(AM40=0,AM41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM41)*AM40)),MAX(0,40*MAX(1,AM40)-(0))))</f>
+        <v>0</v>
       </c>
       <c r="AN42" s="61">
-        <f>IF(AND(AN40=1,AN41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN41)*AN40)),MAX(0,40*MAX(1,AN40)-(AM42))))</f>
-        <v>8</v>
+        <f>IF(AND(AN40=0,AN41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN41)*AN40)),MAX(0,40*MAX(1,AN40)-(AM42))))</f>
+        <v>0</v>
       </c>
       <c r="AO42" s="61">
-        <f>IF(AND(AO40=1,AO41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO41)*AO40)),MAX(0,40*MAX(1,AO40)-(AM42+AN42))))</f>
-        <v>8</v>
+        <f>IF(AND(AO40=0,AO41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO41)*AO40)),MAX(0,40*MAX(1,AO40)-(AM42+AN42))))</f>
+        <v>0</v>
       </c>
       <c r="AP42" s="63">
-        <f>IF(AND(AP40=1,AP41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP41)*AP40)),MAX(0,40*MAX(1,AP40)-(AM42+AN42+AO42))))</f>
-        <v>8</v>
+        <f>IF(AND(AP40=0,AP41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP41)*AP40)),MAX(0,40*MAX(1,AP40)-(AM42+AN42+AO42))))</f>
+        <v>0</v>
       </c>
       <c r="OU42" s="28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A43" s="43"/>
+      <c r="A43" s="72"/>
       <c r="B43" s="44"/>
       <c r="C43" s="64">
         <f>G39*N(D43)</f>
-        <v>5376.8</v>
+        <v>6873.240000000001</v>
       </c>
       <c r="D43" s="64">
         <f>IF(TRIM(B39)="","No rate",IFERROR(INDEX('Rate Tables'!D$7:D$161,MATCH(B39,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>122.2</v>
+        <v>156.21</v>
       </c>
       <c r="E43" s="53" t="s">
         <v>60</v>
@@ -12518,51 +12518,51 @@
         <v>2</v>
       </c>
       <c r="AI43" s="61">
-        <f>IF(AND(AI40=1,AI41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MAX(0,AI41-(IF('_JobDays'!Y3,8,10)))*AI40))+((IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI41)*AI40)))-MIN(IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI41)*AI40)),MAX(0,40*MAX(1,AI40)-(0)))))</f>
+        <f>IF(AND(AI40=0,AI41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MAX(0,AI41-(IF('_JobDays'!Y3,8,10)))*AI40))+((IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI41)*AI40)))-MIN(IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI41)*AI40)),MAX(0,40*MAX(1,AI40)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AJ43" s="61">
-        <f>IF(AND(AJ40=1,AJ41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MAX(0,AJ41-(IF('_JobDays'!Z3,8,10)))*AJ40))+((IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ41)*AJ40)))-MIN(IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ41)*AJ40)),MAX(0,40*MAX(1,AJ40)-(AI42)))))</f>
+        <f>IF(AND(AJ40=0,AJ41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MAX(0,AJ41-(IF('_JobDays'!Z3,8,10)))*AJ40))+((IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ41)*AJ40)))-MIN(IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ41)*AJ40)),MAX(0,40*MAX(1,AJ40)-(AI42)))))</f>
         <v>0</v>
       </c>
       <c r="AK43" s="62">
-        <f>IF(AND(AK40=0,AK41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MAX(0,AK41-(IF('_JobDays'!AA3,8,10)))*AK40))+((IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK41)*AK40)))-MIN(IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK41)*AK40)),MAX(0,40*MAX(1,AK40)-(0)))))</f>
+        <f>IF(AND(AK40=0,AK41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MAX(0,AK41-(IF('_JobDays'!AA3,8,10)))*AK40))+((IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK41)*AK40)))-MIN(IF(OR(AK40&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK41)*AK40)),MAX(0,40*MAX(1,AK40)-(AI42+AJ42)))))</f>
         <v>0</v>
       </c>
       <c r="AL43" s="62">
-        <f>IF(AND(AL40=0,AL41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MAX(0,AL41-(IF('_JobDays'!AB3,8,10)))*AL40))+((IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL41)*AL40)))-MIN(IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL41)*AL40)),MAX(0,40*MAX(1,AL40)-(AK42)))))</f>
+        <f>IF(AND(AL40=0,AL41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MAX(0,AL41-(IF('_JobDays'!AB3,8,10)))*AL40))+((IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL41)*AL40)))-MIN(IF(OR(AL40&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL41)*AL40)),MAX(0,40*MAX(1,AL40)-(AI42+AJ42+AK42)))))</f>
         <v>0</v>
       </c>
       <c r="AM43" s="61">
-        <f>IF(AND(AM40=1,AM41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MAX(0,AM41-(IF('_JobDays'!AC3,8,10)))*AM40))+((IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM41)*AM40)))-MIN(IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM41)*AM40)),MAX(0,40*MAX(1,AM40)-(0)))))</f>
+        <f>IF(AND(AM40=0,AM41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MAX(0,AM41-(IF('_JobDays'!AC3,8,10)))*AM40))+((IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM41)*AM40)))-MIN(IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM41)*AM40)),MAX(0,40*MAX(1,AM40)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AN43" s="61">
-        <f>IF(AND(AN40=1,AN41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MAX(0,AN41-(IF('_JobDays'!AD3,8,10)))*AN40))+((IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN41)*AN40)))-MIN(IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN41)*AN40)),MAX(0,40*MAX(1,AN40)-(AM42)))))</f>
+        <f>IF(AND(AN40=0,AN41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MAX(0,AN41-(IF('_JobDays'!AD3,8,10)))*AN40))+((IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN41)*AN40)))-MIN(IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN41)*AN40)),MAX(0,40*MAX(1,AN40)-(AM42)))))</f>
         <v>0</v>
       </c>
       <c r="AO43" s="61">
-        <f>IF(AND(AO40=1,AO41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MAX(0,AO41-(IF('_JobDays'!AE3,8,10)))*AO40))+((IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO41)*AO40)))-MIN(IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO41)*AO40)),MAX(0,40*MAX(1,AO40)-(AM42+AN42)))))</f>
+        <f>IF(AND(AO40=0,AO41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MAX(0,AO41-(IF('_JobDays'!AE3,8,10)))*AO40))+((IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO41)*AO40)))-MIN(IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO41)*AO40)),MAX(0,40*MAX(1,AO40)-(AM42+AN42)))))</f>
         <v>0</v>
       </c>
       <c r="AP43" s="63">
-        <f>IF(AND(AP40=1,AP41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MAX(0,AP41-(IF('_JobDays'!AF3,8,10)))*AP40))+((IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP41)*AP40)))-MIN(IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP41)*AP40)),MAX(0,40*MAX(1,AP40)-(AM42+AN42+AO42)))))</f>
+        <f>IF(AND(AP40=0,AP41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MAX(0,AP41-(IF('_JobDays'!AF3,8,10)))*AP40))+((IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP41)*AP40)))-MIN(IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP41)*AP40)),MAX(0,40*MAX(1,AP40)-(AM42+AN42+AO42)))))</f>
         <v>0</v>
       </c>
       <c r="OU43" s="28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A44" s="43"/>
+      <c r="A44" s="72"/>
       <c r="B44" s="44"/>
       <c r="C44" s="59">
         <f>H39*N(D44)</f>
-        <v>3681.3599999999997</v>
+        <v>4818</v>
       </c>
       <c r="D44" s="59">
         <f>IF(TRIM(B39)="","No rate",IFERROR(INDEX('Rate Tables'!E$7:E$161,MATCH(B39,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>153.39</v>
+        <v>200.75</v>
       </c>
       <c r="E44" s="53" t="s">
         <v>61</v>
@@ -12669,11 +12669,11 @@
         <v>0</v>
       </c>
       <c r="AI44" s="61">
-        <f>IF(AND(AI40=1,AI41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI40*AI41,0)))</f>
+        <f>IF(AND(AI40=0,AI41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI40&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI40*AI41,0)))</f>
         <v>0</v>
       </c>
       <c r="AJ44" s="61">
-        <f>IF(AND(AJ40=1,AJ41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ40*AJ41,0)))</f>
+        <f>IF(AND(AJ40=0,AJ41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ40&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ40*AJ41,0)))</f>
         <v>0</v>
       </c>
       <c r="AK44" s="62">
@@ -12685,27 +12685,27 @@
         <v>0</v>
       </c>
       <c r="AM44" s="61">
-        <f>IF(AND(AM40=1,AM41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM40*AM41,0)))</f>
+        <f>IF(AND(AM40=0,AM41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM40&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM40*AM41,0)))</f>
         <v>0</v>
       </c>
       <c r="AN44" s="61">
-        <f>IF(AND(AN40=1,AN41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN40*AN41,0)))</f>
+        <f>IF(AND(AN40=0,AN41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN40&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN40*AN41,0)))</f>
         <v>0</v>
       </c>
       <c r="AO44" s="61">
-        <f>IF(AND(AO40=1,AO41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO40*AO41,0)))</f>
+        <f>IF(AND(AO40=0,AO41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO40&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO40*AO41,0)))</f>
         <v>0</v>
       </c>
       <c r="AP44" s="63">
-        <f>IF(AND(AP40=1,AP41=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP40*AP41,0)))</f>
+        <f>IF(AND(AP40=0,AP41=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP40&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP40*AP41,0)))</f>
         <v>0</v>
       </c>
       <c r="OU44" s="28" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A45" s="43"/>
+      <c r="A45" s="72"/>
       <c r="B45" s="44"/>
       <c r="C45" s="65">
         <f>I39*D45</f>
@@ -12819,7 +12819,7 @@
         <v>0</v>
       </c>
       <c r="OU45" s="58" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" ht="8" customHeight="1" spans="1:42" x14ac:dyDescent="0.25">
@@ -12868,14 +12868,14 @@
     </row>
     <row r="47" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
       <c r="A47" s="72" t="s">
+        <v>69</v>
+      </c>
+      <c r="B47" s="44" t="s">
         <v>63</v>
-      </c>
-      <c r="B47" s="44" t="s">
-        <v>68</v>
       </c>
       <c r="C47" s="45">
         <f>J47</f>
-        <v>23985.44</v>
+        <v>28033.48</v>
       </c>
       <c r="D47" s="46"/>
       <c r="E47" s="46"/>
@@ -12897,7 +12897,7 @@
       </c>
       <c r="J47" s="48">
         <f>C50+C51+C52</f>
-        <v>23985.44</v>
+        <v>28033.48</v>
       </c>
       <c r="K47" s="49"/>
       <c r="L47" s="50"/>
@@ -12932,7 +12932,7 @@
       <c r="AO47" s="50"/>
       <c r="AP47" s="52"/>
       <c r="OU47" s="28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
@@ -13045,7 +13045,7 @@
         <v>0</v>
       </c>
       <c r="OU48" s="58" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
@@ -13158,7 +13158,7 @@
         <v>0</v>
       </c>
       <c r="OU49" s="58" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
@@ -13166,11 +13166,11 @@
       <c r="B50" s="44"/>
       <c r="C50" s="59">
         <f>F47*N(D50)</f>
-        <v>14927.279999999999</v>
+        <v>17344.64</v>
       </c>
       <c r="D50" s="59">
         <f>IF(TRIM(B47)="","No rate",IFERROR(INDEX('Rate Tables'!C$7:C$161,MATCH(B47,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>91.02</v>
+        <v>105.76</v>
       </c>
       <c r="E50" s="53" t="s">
         <v>59</v>
@@ -13309,7 +13309,7 @@
         <v>0</v>
       </c>
       <c r="OU50" s="28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
@@ -13317,11 +13317,11 @@
       <c r="B51" s="44"/>
       <c r="C51" s="64">
         <f>G47*N(D51)</f>
-        <v>5376.8</v>
+        <v>6325.88</v>
       </c>
       <c r="D51" s="64">
         <f>IF(TRIM(B47)="","No rate",IFERROR(INDEX('Rate Tables'!D$7:D$161,MATCH(B47,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>122.2</v>
+        <v>143.77</v>
       </c>
       <c r="E51" s="53" t="s">
         <v>60</v>
@@ -13460,7 +13460,7 @@
         <v>0</v>
       </c>
       <c r="OU51" s="28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
@@ -13468,11 +13468,11 @@
       <c r="B52" s="44"/>
       <c r="C52" s="59">
         <f>H47*N(D52)</f>
-        <v>3681.3599999999997</v>
+        <v>4362.96</v>
       </c>
       <c r="D52" s="59">
         <f>IF(TRIM(B47)="","No rate",IFERROR(INDEX('Rate Tables'!E$7:E$161,MATCH(B47,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>153.39</v>
+        <v>181.79</v>
       </c>
       <c r="E52" s="53" t="s">
         <v>61</v>
@@ -13611,7 +13611,7 @@
         <v>0</v>
       </c>
       <c r="OU52" s="28" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
@@ -13729,7 +13729,7 @@
         <v>0</v>
       </c>
       <c r="OU53" s="58" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="54" ht="8" customHeight="1" spans="1:42" x14ac:dyDescent="0.25">
@@ -13777,25 +13777,25 @@
       <c r="AP54" s="71"/>
     </row>
     <row r="55" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A55" s="43" t="s">
-        <v>54</v>
+      <c r="A55" s="72" t="s">
+        <v>69</v>
       </c>
       <c r="B55" s="44" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C55" s="45">
         <f>J55</f>
-        <v>36191.68</v>
+        <v>23985.44</v>
       </c>
       <c r="D55" s="46"/>
       <c r="E55" s="46"/>
       <c r="F55" s="47">
         <f>SUM(K58:AP58)</f>
-        <v>192</v>
+        <v>164</v>
       </c>
       <c r="G55" s="47">
         <f>SUM(K59:AP59)</f>
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="H55" s="47">
         <f>SUM(K60:AP60)</f>
@@ -13807,7 +13807,7 @@
       </c>
       <c r="J55" s="48">
         <f>C58+C59+C60</f>
-        <v>36191.68</v>
+        <v>23985.44</v>
       </c>
       <c r="K55" s="49"/>
       <c r="L55" s="50"/>
@@ -13846,7 +13846,7 @@
       </c>
     </row>
     <row r="56" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A56" s="43"/>
+      <c r="A56" s="72"/>
       <c r="B56" s="44"/>
       <c r="C56" s="45"/>
       <c r="D56" s="46"/>
@@ -13931,10 +13931,10 @@
         <v>1</v>
       </c>
       <c r="AI56" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ56" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AK56" s="56">
         <v>0</v>
@@ -13943,23 +13943,23 @@
         <v>0</v>
       </c>
       <c r="AM56" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN56" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AO56" s="55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP56" s="57">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="OU56" s="58" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A57" s="43"/>
+      <c r="A57" s="72"/>
       <c r="B57" s="44"/>
       <c r="C57" s="45"/>
       <c r="D57" s="46"/>
@@ -14044,10 +14044,10 @@
         <v>12</v>
       </c>
       <c r="AI57" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AJ57" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AK57" s="56">
         <v>0</v>
@@ -14056,31 +14056,31 @@
         <v>0</v>
       </c>
       <c r="AM57" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AN57" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AO57" s="55">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AP57" s="57">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="OU57" s="58" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A58" s="43"/>
+      <c r="A58" s="72"/>
       <c r="B58" s="44"/>
       <c r="C58" s="59">
         <f>F55*N(D58)</f>
-        <v>21354.239999999998</v>
+        <v>14927.279999999999</v>
       </c>
       <c r="D58" s="59">
         <f>IF(TRIM(B55)="","No rate",IFERROR(INDEX('Rate Tables'!C$7:C$161,MATCH(B55,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>111.22</v>
+        <v>91.02</v>
       </c>
       <c r="E58" s="53" t="s">
         <v>59</v>
@@ -14091,147 +14091,147 @@
       <c r="I58" s="47"/>
       <c r="J58" s="48"/>
       <c r="K58" s="60">
-        <f>IF(AND(K56=1,K57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,0,IF('_JobDays'!A3,MIN(8,K57)*K56,K56*K57)))),MAX(0,40*MAX(1,K56)-(0))))</f>
+        <f>IF(AND(K56=1,K57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MIN(IF('_JobDays'!A3,8,10),K57)*K56)),MAX(0,40*MAX(1,K56)-(0))))</f>
         <v>8</v>
       </c>
       <c r="L58" s="61">
-        <f>IF(AND(L56=1,L57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,0,IF('_JobDays'!B3,MIN(8,L57)*L56,L56*L57)))),MAX(0,40*MAX(1,L56)-(K58))))</f>
+        <f>IF(AND(L56=1,L57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MIN(IF('_JobDays'!B3,8,10),L57)*L56)),MAX(0,40*MAX(1,L56)-(K58))))</f>
         <v>8</v>
       </c>
       <c r="M58" s="61">
-        <f>IF(AND(M56=1,M57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,0,IF('_JobDays'!C3,MIN(8,M57)*M56,M56*M57)))),MAX(0,40*MAX(1,M56)-(K58+L58))))</f>
+        <f>IF(AND(M56=1,M57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MIN(IF('_JobDays'!C3,8,10),M57)*M56)),MAX(0,40*MAX(1,M56)-(K58+L58))))</f>
         <v>8</v>
       </c>
       <c r="N58" s="61">
-        <f>IF(AND(N56=1,N57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,0,IF('_JobDays'!D3,MIN(8,N57)*N56,N56*N57)))),MAX(0,40*MAX(1,N56)-(K58+L58+M58))))</f>
+        <f>IF(AND(N56=1,N57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MIN(IF('_JobDays'!D3,8,10),N57)*N56)),MAX(0,40*MAX(1,N56)-(K58+L58+M58))))</f>
         <v>8</v>
       </c>
       <c r="O58" s="61">
-        <f>IF(AND(O56=1,O57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,0,IF('_JobDays'!E3,MIN(8,O57)*O56,O56*O57)))),MAX(0,40*MAX(1,O56)-(K58+L58+M58+N58))))</f>
+        <f>IF(AND(O56=1,O57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MIN(IF('_JobDays'!E3,8,10),O57)*O56)),MAX(0,40*MAX(1,O56)-(K58+L58+M58+N58))))</f>
         <v>8</v>
       </c>
       <c r="P58" s="62">
-        <f>IF(AND(P56=0,P57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,0,IF('_JobDays'!F3,MIN(8,P57)*P56,P56*P57)))),MAX(0,40*MAX(1,P56)-(0))))</f>
+        <f>IF(AND(P56=0,P57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MIN(IF('_JobDays'!F3,8,10),P57)*P56)),MAX(0,40*MAX(1,P56)-(0))))</f>
         <v>0</v>
       </c>
       <c r="Q58" s="62">
-        <f>IF(AND(Q56=0,Q57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,0,IF('_JobDays'!G3,MIN(8,Q57)*Q56,Q56*Q57)))),MAX(0,40*MAX(1,Q56)-(P58))))</f>
+        <f>IF(AND(Q56=0,Q57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,MIN(IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MIN(IF('_JobDays'!G3,8,10),Q57)*Q56)),MAX(0,40*MAX(1,Q56)-(P58))))</f>
         <v>0</v>
       </c>
       <c r="R58" s="61">
-        <f>IF(AND(R56=1,R57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,0,IF('_JobDays'!H3,MIN(8,R57)*R56,R56*R57)))),MAX(0,40*MAX(1,R56)-(0))))</f>
+        <f>IF(AND(R56=1,R57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MIN(IF('_JobDays'!H3,8,10),R57)*R56)),MAX(0,40*MAX(1,R56)-(0))))</f>
         <v>8</v>
       </c>
       <c r="S58" s="61">
-        <f>IF(AND(S56=1,S57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,0,IF('_JobDays'!I3,MIN(8,S57)*S56,S56*S57)))),MAX(0,40*MAX(1,S56)-(R58))))</f>
+        <f>IF(AND(S56=1,S57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MIN(IF('_JobDays'!I3,8,10),S57)*S56)),MAX(0,40*MAX(1,S56)-(R58))))</f>
         <v>8</v>
       </c>
       <c r="T58" s="61">
-        <f>IF(AND(T56=1,T57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,0,IF('_JobDays'!J3,MIN(8,T57)*T56,T56*T57)))),MAX(0,40*MAX(1,T56)-(R58+S58))))</f>
+        <f>IF(AND(T56=1,T57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),8,MIN(IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MIN(IF('_JobDays'!J3,8,10),T57)*T56)),MAX(0,40*MAX(1,T56)-(R58+S58))))</f>
         <v>8</v>
       </c>
       <c r="U58" s="61">
-        <f>IF(AND(U56=1,U57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,0,IF('_JobDays'!K3,MIN(8,U57)*U56,U56*U57)))),MAX(0,40*MAX(1,U56)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(U56=1,U57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MIN(IF('_JobDays'!K3,8,10),U57)*U56)),MAX(0,40*MAX(1,U56)-(0))))</f>
+        <v>10</v>
       </c>
       <c r="V58" s="61">
-        <f>IF(AND(V56=1,V57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,0,IF('_JobDays'!L3,MIN(8,V57)*V56,V56*V57)))),MAX(0,40*MAX(1,V56)-(U58))))</f>
-        <v>8</v>
+        <f>IF(AND(V56=1,V57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MIN(IF('_JobDays'!L3,8,10),V57)*V56)),MAX(0,40*MAX(1,V56)-(U58))))</f>
+        <v>10</v>
       </c>
       <c r="W58" s="62">
-        <f>IF(AND(W56=1,W57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,0,IF('_JobDays'!M3,MIN(8,W57)*W56,W56*W57)))),MAX(0,40*MAX(1,W56)-(U58+V58))))</f>
-        <v>0</v>
+        <f>IF(AND(W56=1,W57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MIN(IF('_JobDays'!M3,8,10),W57)*W56)),MAX(0,40*MAX(1,W56)-(U58+V58))))</f>
+        <v>10</v>
       </c>
       <c r="X58" s="62">
-        <f>IF(AND(X56=1,X57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,0,IF('_JobDays'!N3,MIN(8,X57)*X56,X56*X57)))),MAX(0,40*MAX(1,X56)-(U58+V58+W58))))</f>
+        <f>IF(AND(X56=1,X57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MIN(IF('_JobDays'!N3,8,10),X57)*X56)),MAX(0,40*MAX(1,X56)-(U58+V58+W58))))</f>
         <v>0</v>
       </c>
       <c r="Y58" s="61">
-        <f>IF(AND(Y56=1,Y57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,0,IF('_JobDays'!O3,MIN(8,Y57)*Y56,Y56*Y57)))),MAX(0,40*MAX(1,Y56)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(Y56=1,Y57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MIN(IF('_JobDays'!O3,8,10),Y57)*Y56)),MAX(0,40*MAX(1,Y56)-(0))))</f>
+        <v>10</v>
       </c>
       <c r="Z58" s="61">
-        <f>IF(AND(Z56=1,Z57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,0,IF('_JobDays'!P3,MIN(8,Z57)*Z56,Z56*Z57)))),MAX(0,40*MAX(1,Z56)-(Y58))))</f>
-        <v>8</v>
+        <f>IF(AND(Z56=1,Z57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MIN(IF('_JobDays'!P3,8,10),Z57)*Z56)),MAX(0,40*MAX(1,Z56)-(Y58))))</f>
+        <v>10</v>
       </c>
       <c r="AA58" s="61">
-        <f>IF(AND(AA56=1,AA57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,0,IF('_JobDays'!Q3,MIN(8,AA57)*AA56,AA56*AA57)))),MAX(0,40*MAX(1,AA56)-(Y58+Z58))))</f>
-        <v>8</v>
+        <f>IF(AND(AA56=1,AA57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MIN(IF('_JobDays'!Q3,8,10),AA57)*AA56)),MAX(0,40*MAX(1,AA56)-(Y58+Z58))))</f>
+        <v>10</v>
       </c>
       <c r="AB58" s="61">
-        <f>IF(AND(AB56=1,AB57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,0,IF('_JobDays'!R3,MIN(8,AB57)*AB56,AB56*AB57)))),MAX(0,40*MAX(1,AB56)-(Y58+Z58+AA58))))</f>
-        <v>8</v>
+        <f>IF(AND(AB56=1,AB57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MIN(IF('_JobDays'!R3,8,10),AB57)*AB56)),MAX(0,40*MAX(1,AB56)-(Y58+Z58+AA58))))</f>
+        <v>10</v>
       </c>
       <c r="AC58" s="61">
-        <f>IF(AND(AC56=1,AC57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,0,IF('_JobDays'!S3,MIN(8,AC57)*AC56,AC56*AC57)))),MAX(0,40*MAX(1,AC56)-(Y58+Z58+AA58+AB58))))</f>
-        <v>8</v>
+        <f>IF(AND(AC56=1,AC57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MIN(IF('_JobDays'!S3,8,10),AC57)*AC56)),MAX(0,40*MAX(1,AC56)-(Y58+Z58+AA58+AB58))))</f>
+        <v>0</v>
       </c>
       <c r="AD58" s="62">
-        <f>IF(AND(AD56=1,AD57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,0,IF('_JobDays'!T3,MIN(8,AD57)*AD56,AD56*AD57)))),MAX(0,40*MAX(1,AD56)-(Y58+Z58+AA58+AB58+AC58))))</f>
+        <f>IF(AND(AD56=1,AD57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MIN(IF('_JobDays'!T3,8,10),AD57)*AD56)),MAX(0,40*MAX(1,AD56)-(Y58+Z58+AA58+AB58+AC58))))</f>
         <v>0</v>
       </c>
       <c r="AE58" s="62">
-        <f>IF(AND(AE56=1,AE57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,0,IF('_JobDays'!U3,MIN(8,AE57)*AE56,AE56*AE57)))),MAX(0,40*MAX(1,AE56)-(Y58+Z58+AA58+AB58+AC58+AD58))))</f>
+        <f>IF(AND(AE56=1,AE57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,MIN(IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MIN(IF('_JobDays'!U3,8,10),AE57)*AE56)),MAX(0,40*MAX(1,AE56)-(Y58+Z58+AA58+AB58+AC58+AD58))))</f>
         <v>0</v>
       </c>
       <c r="AF58" s="61">
-        <f>IF(AND(AF56=1,AF57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,0,IF('_JobDays'!V3,MIN(8,AF57)*AF56,AF56*AF57)))),MAX(0,40*MAX(1,AF56)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(AF56=1,AF57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MIN(IF('_JobDays'!V3,8,10),AF57)*AF56)),MAX(0,40*MAX(1,AF56)-(0))))</f>
+        <v>10</v>
       </c>
       <c r="AG58" s="61">
-        <f>IF(AND(AG56=1,AG57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,0,IF('_JobDays'!W3,MIN(8,AG57)*AG56,AG56*AG57)))),MAX(0,40*MAX(1,AG56)-(AF58))))</f>
-        <v>8</v>
+        <f>IF(AND(AG56=1,AG57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MIN(IF('_JobDays'!W3,8,10),AG57)*AG56)),MAX(0,40*MAX(1,AG56)-(AF58))))</f>
+        <v>10</v>
       </c>
       <c r="AH58" s="61">
-        <f>IF(AND(AH56=1,AH57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),8,MIN(IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,0,IF('_JobDays'!X3,MIN(8,AH57)*AH56,AH56*AH57)))),MAX(0,40*MAX(1,AH56)-(AF58+AG58))))</f>
-        <v>8</v>
+        <f>IF(AND(AH56=1,AH57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),10,MIN(IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MIN(IF('_JobDays'!X3,8,10),AH57)*AH56)),MAX(0,40*MAX(1,AH56)-(AF58+AG58))))</f>
+        <v>10</v>
       </c>
       <c r="AI58" s="61">
-        <f>IF(AND(AI56=1,AI57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,0,IF('_JobDays'!Y3,MIN(8,AI57)*AI56,AI56*AI57)))),MAX(0,40*MAX(1,AI56)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(AI56=0,AI57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI57)*AI56)),MAX(0,40*MAX(1,AI56)-(0))))</f>
+        <v>0</v>
       </c>
       <c r="AJ58" s="61">
-        <f>IF(AND(AJ56=1,AJ57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,0,IF('_JobDays'!Z3,MIN(8,AJ57)*AJ56,AJ56*AJ57)))),MAX(0,40*MAX(1,AJ56)-(AI58))))</f>
-        <v>8</v>
+        <f>IF(AND(AJ56=0,AJ57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ57)*AJ56)),MAX(0,40*MAX(1,AJ56)-(AI58))))</f>
+        <v>0</v>
       </c>
       <c r="AK58" s="62">
-        <f>IF(AND(AK56=0,AK57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,0,IF('_JobDays'!AA3,MIN(8,AK57)*AK56,AK56*AK57)))),MAX(0,40*MAX(1,AK56)-(0))))</f>
+        <f>IF(AND(AK56=0,AK57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK57)*AK56)),MAX(0,40*MAX(1,AK56)-(AI58+AJ58))))</f>
         <v>0</v>
       </c>
       <c r="AL58" s="62">
-        <f>IF(AND(AL56=0,AL57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,0,IF('_JobDays'!AB3,MIN(8,AL57)*AL56,AL56*AL57)))),MAX(0,40*MAX(1,AL56)-(AK58))))</f>
+        <f>IF(AND(AL56=0,AL57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL57)*AL56)),MAX(0,40*MAX(1,AL56)-(AI58+AJ58+AK58))))</f>
         <v>0</v>
       </c>
       <c r="AM58" s="61">
-        <f>IF(AND(AM56=1,AM57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,0,IF('_JobDays'!AC3,MIN(8,AM57)*AM56,AM56*AM57)))),MAX(0,40*MAX(1,AM56)-(0))))</f>
-        <v>8</v>
+        <f>IF(AND(AM56=0,AM57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM57)*AM56)),MAX(0,40*MAX(1,AM56)-(0))))</f>
+        <v>0</v>
       </c>
       <c r="AN58" s="61">
-        <f>IF(AND(AN56=1,AN57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,0,IF('_JobDays'!AD3,MIN(8,AN57)*AN56,AN56*AN57)))),MAX(0,40*MAX(1,AN56)-(AM58))))</f>
-        <v>8</v>
+        <f>IF(AND(AN56=0,AN57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN57)*AN56)),MAX(0,40*MAX(1,AN56)-(AM58))))</f>
+        <v>0</v>
       </c>
       <c r="AO58" s="61">
-        <f>IF(AND(AO56=1,AO57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,0,IF('_JobDays'!AE3,MIN(8,AO57)*AO56,AO56*AO57)))),MAX(0,40*MAX(1,AO56)-(AM58+AN58))))</f>
-        <v>8</v>
+        <f>IF(AND(AO56=0,AO57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO57)*AO56)),MAX(0,40*MAX(1,AO56)-(AM58+AN58))))</f>
+        <v>0</v>
       </c>
       <c r="AP58" s="63">
-        <f>IF(AND(AP56=1,AP57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),8,MIN(IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,0,IF('_JobDays'!AF3,MIN(8,AP57)*AP56,AP56*AP57)))),MAX(0,40*MAX(1,AP56)-(AM58+AN58+AO58))))</f>
-        <v>8</v>
+        <f>IF(AND(AP56=0,AP57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,MIN(IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP57)*AP56)),MAX(0,40*MAX(1,AP56)-(AM58+AN58+AO58))))</f>
+        <v>0</v>
       </c>
       <c r="OU58" s="28" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A59" s="43"/>
+      <c r="A59" s="72"/>
       <c r="B59" s="44"/>
       <c r="C59" s="64">
         <f>G55*N(D59)</f>
-        <v>10003.84</v>
+        <v>5376.8</v>
       </c>
       <c r="D59" s="64">
         <f>IF(TRIM(B55)="","No rate",IFERROR(INDEX('Rate Tables'!D$7:D$161,MATCH(B55,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>156.31</v>
+        <v>122.2</v>
       </c>
       <c r="E59" s="53" t="s">
         <v>60</v>
@@ -14242,131 +14242,131 @@
       <c r="I59" s="47"/>
       <c r="J59" s="48"/>
       <c r="K59" s="60">
-        <f>IF(AND(K56=1,K57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),0,IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,K56*K57,IF('_JobDays'!A3,MAX(0,K57-8)*K56,0))))+((IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,0,IF('_JobDays'!A3,MIN(8,K57)*K56,K56*K57)))))-MIN(IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,IF(WEEKDAY(K$6,1)=7,0,IF('_JobDays'!A3,MIN(8,K57)*K56,K56*K57)))),MAX(0,40*MAX(1,K56)-(0)))))</f>
+        <f>IF(AND(K56=1,K57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=K$6,'Job setup'!$D$7&gt;=K$6,'Job setup'!$G$7="YES")),0,IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MAX(0,K57-(IF('_JobDays'!A3,8,10)))*K56))+((IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MIN(IF('_JobDays'!A3,8,10),K57)*K56)))-MIN(IF(OR(K56&lt;=0,NOT('_JobDays'!A2)),0,IF(WEEKDAY(K$6,1)=1,0,MIN(IF('_JobDays'!A3,8,10),K57)*K56)),MAX(0,40*MAX(1,K56)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="L59" s="61">
-        <f>IF(AND(L56=1,L57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),0,IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,L56*L57,IF('_JobDays'!B3,MAX(0,L57-8)*L56,0))))+((IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,0,IF('_JobDays'!B3,MIN(8,L57)*L56,L56*L57)))))-MIN(IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,IF(WEEKDAY(L$6,1)=7,0,IF('_JobDays'!B3,MIN(8,L57)*L56,L56*L57)))),MAX(0,40*MAX(1,L56)-(K58)))))</f>
+        <f>IF(AND(L56=1,L57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=L$6,'Job setup'!$D$7&gt;=L$6,'Job setup'!$G$7="YES")),0,IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MAX(0,L57-(IF('_JobDays'!B3,8,10)))*L56))+((IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MIN(IF('_JobDays'!B3,8,10),L57)*L56)))-MIN(IF(OR(L56&lt;=0,NOT('_JobDays'!B2)),0,IF(WEEKDAY(L$6,1)=1,0,MIN(IF('_JobDays'!B3,8,10),L57)*L56)),MAX(0,40*MAX(1,L56)-(K58)))))</f>
         <v>0</v>
       </c>
       <c r="M59" s="61">
-        <f>IF(AND(M56=1,M57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),0,IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,M56*M57,IF('_JobDays'!C3,MAX(0,M57-8)*M56,0))))+((IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,0,IF('_JobDays'!C3,MIN(8,M57)*M56,M56*M57)))))-MIN(IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,IF(WEEKDAY(M$6,1)=7,0,IF('_JobDays'!C3,MIN(8,M57)*M56,M56*M57)))),MAX(0,40*MAX(1,M56)-(K58+L58)))))</f>
+        <f>IF(AND(M56=1,M57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=M$6,'Job setup'!$D$7&gt;=M$6,'Job setup'!$G$7="YES")),0,IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MAX(0,M57-(IF('_JobDays'!C3,8,10)))*M56))+((IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MIN(IF('_JobDays'!C3,8,10),M57)*M56)))-MIN(IF(OR(M56&lt;=0,NOT('_JobDays'!C2)),0,IF(WEEKDAY(M$6,1)=1,0,MIN(IF('_JobDays'!C3,8,10),M57)*M56)),MAX(0,40*MAX(1,M56)-(K58+L58)))))</f>
         <v>0</v>
       </c>
       <c r="N59" s="61">
-        <f>IF(AND(N56=1,N57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),0,IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,N56*N57,IF('_JobDays'!D3,MAX(0,N57-8)*N56,0))))+((IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,0,IF('_JobDays'!D3,MIN(8,N57)*N56,N56*N57)))))-MIN(IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,IF(WEEKDAY(N$6,1)=7,0,IF('_JobDays'!D3,MIN(8,N57)*N56,N56*N57)))),MAX(0,40*MAX(1,N56)-(K58+L58+M58)))))</f>
+        <f>IF(AND(N56=1,N57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=N$6,'Job setup'!$D$7&gt;=N$6,'Job setup'!$G$7="YES")),0,IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MAX(0,N57-(IF('_JobDays'!D3,8,10)))*N56))+((IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MIN(IF('_JobDays'!D3,8,10),N57)*N56)))-MIN(IF(OR(N56&lt;=0,NOT('_JobDays'!D2)),0,IF(WEEKDAY(N$6,1)=1,0,MIN(IF('_JobDays'!D3,8,10),N57)*N56)),MAX(0,40*MAX(1,N56)-(K58+L58+M58)))))</f>
         <v>0</v>
       </c>
       <c r="O59" s="61">
-        <f>IF(AND(O56=1,O57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),0,IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,O56*O57,IF('_JobDays'!E3,MAX(0,O57-8)*O56,0))))+((IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,0,IF('_JobDays'!E3,MIN(8,O57)*O56,O56*O57)))))-MIN(IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,IF(WEEKDAY(O$6,1)=7,0,IF('_JobDays'!E3,MIN(8,O57)*O56,O56*O57)))),MAX(0,40*MAX(1,O56)-(K58+L58+M58+N58)))))</f>
+        <f>IF(AND(O56=1,O57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=O$6,'Job setup'!$D$7&gt;=O$6,'Job setup'!$G$7="YES")),0,IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MAX(0,O57-(IF('_JobDays'!E3,8,10)))*O56))+((IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MIN(IF('_JobDays'!E3,8,10),O57)*O56)))-MIN(IF(OR(O56&lt;=0,NOT('_JobDays'!E2)),0,IF(WEEKDAY(O$6,1)=1,0,MIN(IF('_JobDays'!E3,8,10),O57)*O56)),MAX(0,40*MAX(1,O56)-(K58+L58+M58+N58)))))</f>
         <v>0</v>
       </c>
       <c r="P59" s="62">
-        <f>IF(AND(P56=0,P57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,P56*P57,IF('_JobDays'!F3,MAX(0,P57-8)*P56,0))))+((IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,0,IF('_JobDays'!F3,MIN(8,P57)*P56,P56*P57)))))-MIN(IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,IF(WEEKDAY(P$6,1)=7,0,IF('_JobDays'!F3,MIN(8,P57)*P56,P56*P57)))),MAX(0,40*MAX(1,P56)-(0)))))</f>
+        <f>IF(AND(P56=0,P57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=P$6,'Job setup'!$D$7&gt;=P$6,'Job setup'!$G$7="YES")),0,IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MAX(0,P57-(IF('_JobDays'!F3,8,10)))*P56))+((IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MIN(IF('_JobDays'!F3,8,10),P57)*P56)))-MIN(IF(OR(P56&lt;=0,NOT('_JobDays'!F2)),0,IF(WEEKDAY(P$6,1)=1,0,MIN(IF('_JobDays'!F3,8,10),P57)*P56)),MAX(0,40*MAX(1,P56)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="Q59" s="62">
-        <f>IF(AND(Q56=0,Q57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,Q56*Q57,IF('_JobDays'!G3,MAX(0,Q57-8)*Q56,0))))+((IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,0,IF('_JobDays'!G3,MIN(8,Q57)*Q56,Q56*Q57)))))-MIN(IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,IF(WEEKDAY(Q$6,1)=7,0,IF('_JobDays'!G3,MIN(8,Q57)*Q56,Q56*Q57)))),MAX(0,40*MAX(1,Q56)-(P58)))))</f>
+        <f>IF(AND(Q56=0,Q57=0,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=Q$6,'Job setup'!$D$7&gt;=Q$6,'Job setup'!$G$7="YES")),0,IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MAX(0,Q57-(IF('_JobDays'!G3,8,10)))*Q56))+((IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MIN(IF('_JobDays'!G3,8,10),Q57)*Q56)))-MIN(IF(OR(Q56&lt;=0,NOT('_JobDays'!G2)),0,IF(WEEKDAY(Q$6,1)=1,0,MIN(IF('_JobDays'!G3,8,10),Q57)*Q56)),MAX(0,40*MAX(1,Q56)-(P58)))))</f>
         <v>0</v>
       </c>
       <c r="R59" s="61">
-        <f>IF(AND(R56=1,R57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),0,IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,R56*R57,IF('_JobDays'!H3,MAX(0,R57-8)*R56,0))))+((IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,0,IF('_JobDays'!H3,MIN(8,R57)*R56,R56*R57)))))-MIN(IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,IF(WEEKDAY(R$6,1)=7,0,IF('_JobDays'!H3,MIN(8,R57)*R56,R56*R57)))),MAX(0,40*MAX(1,R56)-(0)))))</f>
+        <f>IF(AND(R56=1,R57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=R$6,'Job setup'!$D$7&gt;=R$6,'Job setup'!$G$7="YES")),0,IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MAX(0,R57-(IF('_JobDays'!H3,8,10)))*R56))+((IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MIN(IF('_JobDays'!H3,8,10),R57)*R56)))-MIN(IF(OR(R56&lt;=0,NOT('_JobDays'!H2)),0,IF(WEEKDAY(R$6,1)=1,0,MIN(IF('_JobDays'!H3,8,10),R57)*R56)),MAX(0,40*MAX(1,R56)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="S59" s="61">
-        <f>IF(AND(S56=1,S57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),0,IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,S56*S57,IF('_JobDays'!I3,MAX(0,S57-8)*S56,0))))+((IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,0,IF('_JobDays'!I3,MIN(8,S57)*S56,S56*S57)))))-MIN(IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,IF(WEEKDAY(S$6,1)=7,0,IF('_JobDays'!I3,MIN(8,S57)*S56,S56*S57)))),MAX(0,40*MAX(1,S56)-(R58)))))</f>
+        <f>IF(AND(S56=1,S57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=S$6,'Job setup'!$D$7&gt;=S$6,'Job setup'!$G$7="YES")),0,IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MAX(0,S57-(IF('_JobDays'!I3,8,10)))*S56))+((IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MIN(IF('_JobDays'!I3,8,10),S57)*S56)))-MIN(IF(OR(S56&lt;=0,NOT('_JobDays'!I2)),0,IF(WEEKDAY(S$6,1)=1,0,MIN(IF('_JobDays'!I3,8,10),S57)*S56)),MAX(0,40*MAX(1,S56)-(R58)))))</f>
         <v>0</v>
       </c>
       <c r="T59" s="61">
-        <f>IF(AND(T56=1,T57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),0,IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,T56*T57,IF('_JobDays'!J3,MAX(0,T57-8)*T56,0))))+((IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,0,IF('_JobDays'!J3,MIN(8,T57)*T56,T56*T57)))))-MIN(IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,IF(WEEKDAY(T$6,1)=7,0,IF('_JobDays'!J3,MIN(8,T57)*T56,T56*T57)))),MAX(0,40*MAX(1,T56)-(R58+S58)))))</f>
+        <f>IF(AND(T56=1,T57=8,AND('Job setup'!$B$7="ON",'Job setup'!$C$7&lt;=T$6,'Job setup'!$D$7&gt;=T$6,'Job setup'!$G$7="YES")),0,IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MAX(0,T57-(IF('_JobDays'!J3,8,10)))*T56))+((IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MIN(IF('_JobDays'!J3,8,10),T57)*T56)))-MIN(IF(OR(T56&lt;=0,NOT('_JobDays'!J2)),0,IF(WEEKDAY(T$6,1)=1,0,MIN(IF('_JobDays'!J3,8,10),T57)*T56)),MAX(0,40*MAX(1,T56)-(R58+S58)))))</f>
         <v>0</v>
       </c>
       <c r="U59" s="61">
-        <f>IF(AND(U56=1,U57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),4,IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,U56*U57,IF('_JobDays'!K3,MAX(0,U57-8)*U56,0))))+((IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,0,IF('_JobDays'!K3,MIN(8,U57)*U56,U56*U57)))))-MIN(IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,IF(WEEKDAY(U$6,1)=7,0,IF('_JobDays'!K3,MIN(8,U57)*U56,U56*U57)))),MAX(0,40*MAX(1,U56)-(0)))))</f>
-        <v>4</v>
+        <f>IF(AND(U56=1,U57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=U$6,'Job setup'!$D$9&gt;=U$6,'Job setup'!$G$9="NO")),2,IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MAX(0,U57-(IF('_JobDays'!K3,8,10)))*U56))+((IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MIN(IF('_JobDays'!K3,8,10),U57)*U56)))-MIN(IF(OR(U56&lt;=0,NOT('_JobDays'!K2)),0,IF(WEEKDAY(U$6,1)=1,0,MIN(IF('_JobDays'!K3,8,10),U57)*U56)),MAX(0,40*MAX(1,U56)-(0)))))</f>
+        <v>2</v>
       </c>
       <c r="V59" s="61">
-        <f>IF(AND(V56=1,V57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),4,IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,V56*V57,IF('_JobDays'!L3,MAX(0,V57-8)*V56,0))))+((IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,0,IF('_JobDays'!L3,MIN(8,V57)*V56,V56*V57)))))-MIN(IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,IF(WEEKDAY(V$6,1)=7,0,IF('_JobDays'!L3,MIN(8,V57)*V56,V56*V57)))),MAX(0,40*MAX(1,V56)-(U58)))))</f>
-        <v>4</v>
+        <f>IF(AND(V56=1,V57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=V$6,'Job setup'!$D$9&gt;=V$6,'Job setup'!$G$9="NO")),2,IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MAX(0,V57-(IF('_JobDays'!L3,8,10)))*V56))+((IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MIN(IF('_JobDays'!L3,8,10),V57)*V56)))-MIN(IF(OR(V56&lt;=0,NOT('_JobDays'!L2)),0,IF(WEEKDAY(V$6,1)=1,0,MIN(IF('_JobDays'!L3,8,10),V57)*V56)),MAX(0,40*MAX(1,V56)-(U58)))))</f>
+        <v>2</v>
       </c>
       <c r="W59" s="62">
-        <f>IF(AND(W56=1,W57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),12,IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,W56*W57,IF('_JobDays'!M3,MAX(0,W57-8)*W56,0))))+((IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,0,IF('_JobDays'!M3,MIN(8,W57)*W56,W56*W57)))))-MIN(IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,IF(WEEKDAY(W$6,1)=7,0,IF('_JobDays'!M3,MIN(8,W57)*W56,W56*W57)))),MAX(0,40*MAX(1,W56)-(U58+V58)))))</f>
-        <v>12</v>
+        <f>IF(AND(W56=1,W57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=W$6,'Job setup'!$D$9&gt;=W$6,'Job setup'!$G$9="NO")),2,IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MAX(0,W57-(IF('_JobDays'!M3,8,10)))*W56))+((IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MIN(IF('_JobDays'!M3,8,10),W57)*W56)))-MIN(IF(OR(W56&lt;=0,NOT('_JobDays'!M2)),0,IF(WEEKDAY(W$6,1)=1,0,MIN(IF('_JobDays'!M3,8,10),W57)*W56)),MAX(0,40*MAX(1,W56)-(U58+V58)))))</f>
+        <v>2</v>
       </c>
       <c r="X59" s="62">
-        <f>IF(AND(X56=1,X57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,X56*X57,IF('_JobDays'!N3,MAX(0,X57-8)*X56,0))))+((IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,0,IF('_JobDays'!N3,MIN(8,X57)*X56,X56*X57)))))-MIN(IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,IF(WEEKDAY(X$6,1)=7,0,IF('_JobDays'!N3,MIN(8,X57)*X56,X56*X57)))),MAX(0,40*MAX(1,X56)-(U58+V58+W58)))))</f>
+        <f>IF(AND(X56=1,X57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=X$6,'Job setup'!$D$9&gt;=X$6,'Job setup'!$G$9="NO")),0,IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MAX(0,X57-(IF('_JobDays'!N3,8,10)))*X56))+((IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MIN(IF('_JobDays'!N3,8,10),X57)*X56)))-MIN(IF(OR(X56&lt;=0,NOT('_JobDays'!N2)),0,IF(WEEKDAY(X$6,1)=1,0,MIN(IF('_JobDays'!N3,8,10),X57)*X56)),MAX(0,40*MAX(1,X56)-(U58+V58+W58)))))</f>
         <v>0</v>
       </c>
       <c r="Y59" s="61">
-        <f>IF(AND(Y56=1,Y57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),4,IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,Y56*Y57,IF('_JobDays'!O3,MAX(0,Y57-8)*Y56,0))))+((IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,0,IF('_JobDays'!O3,MIN(8,Y57)*Y56,Y56*Y57)))))-MIN(IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,IF(WEEKDAY(Y$6,1)=7,0,IF('_JobDays'!O3,MIN(8,Y57)*Y56,Y56*Y57)))),MAX(0,40*MAX(1,Y56)-(0)))))</f>
-        <v>4</v>
+        <f>IF(AND(Y56=1,Y57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Y$6,'Job setup'!$D$9&gt;=Y$6,'Job setup'!$G$9="NO")),2,IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MAX(0,Y57-(IF('_JobDays'!O3,8,10)))*Y56))+((IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MIN(IF('_JobDays'!O3,8,10),Y57)*Y56)))-MIN(IF(OR(Y56&lt;=0,NOT('_JobDays'!O2)),0,IF(WEEKDAY(Y$6,1)=1,0,MIN(IF('_JobDays'!O3,8,10),Y57)*Y56)),MAX(0,40*MAX(1,Y56)-(0)))))</f>
+        <v>2</v>
       </c>
       <c r="Z59" s="61">
-        <f>IF(AND(Z56=1,Z57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),4,IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,Z56*Z57,IF('_JobDays'!P3,MAX(0,Z57-8)*Z56,0))))+((IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,0,IF('_JobDays'!P3,MIN(8,Z57)*Z56,Z56*Z57)))))-MIN(IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,IF(WEEKDAY(Z$6,1)=7,0,IF('_JobDays'!P3,MIN(8,Z57)*Z56,Z56*Z57)))),MAX(0,40*MAX(1,Z56)-(Y58)))))</f>
-        <v>4</v>
+        <f>IF(AND(Z56=1,Z57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=Z$6,'Job setup'!$D$9&gt;=Z$6,'Job setup'!$G$9="NO")),2,IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MAX(0,Z57-(IF('_JobDays'!P3,8,10)))*Z56))+((IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MIN(IF('_JobDays'!P3,8,10),Z57)*Z56)))-MIN(IF(OR(Z56&lt;=0,NOT('_JobDays'!P2)),0,IF(WEEKDAY(Z$6,1)=1,0,MIN(IF('_JobDays'!P3,8,10),Z57)*Z56)),MAX(0,40*MAX(1,Z56)-(Y58)))))</f>
+        <v>2</v>
       </c>
       <c r="AA59" s="61">
-        <f>IF(AND(AA56=1,AA57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),4,IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,AA56*AA57,IF('_JobDays'!Q3,MAX(0,AA57-8)*AA56,0))))+((IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,0,IF('_JobDays'!Q3,MIN(8,AA57)*AA56,AA56*AA57)))))-MIN(IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,IF(WEEKDAY(AA$6,1)=7,0,IF('_JobDays'!Q3,MIN(8,AA57)*AA56,AA56*AA57)))),MAX(0,40*MAX(1,AA56)-(Y58+Z58)))))</f>
-        <v>4</v>
+        <f>IF(AND(AA56=1,AA57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AA$6,'Job setup'!$D$9&gt;=AA$6,'Job setup'!$G$9="NO")),2,IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MAX(0,AA57-(IF('_JobDays'!Q3,8,10)))*AA56))+((IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MIN(IF('_JobDays'!Q3,8,10),AA57)*AA56)))-MIN(IF(OR(AA56&lt;=0,NOT('_JobDays'!Q2)),0,IF(WEEKDAY(AA$6,1)=1,0,MIN(IF('_JobDays'!Q3,8,10),AA57)*AA56)),MAX(0,40*MAX(1,AA56)-(Y58+Z58)))))</f>
+        <v>2</v>
       </c>
       <c r="AB59" s="61">
-        <f>IF(AND(AB56=1,AB57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),4,IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,AB56*AB57,IF('_JobDays'!R3,MAX(0,AB57-8)*AB56,0))))+((IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,0,IF('_JobDays'!R3,MIN(8,AB57)*AB56,AB56*AB57)))))-MIN(IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,IF(WEEKDAY(AB$6,1)=7,0,IF('_JobDays'!R3,MIN(8,AB57)*AB56,AB56*AB57)))),MAX(0,40*MAX(1,AB56)-(Y58+Z58+AA58)))))</f>
-        <v>4</v>
+        <f>IF(AND(AB56=1,AB57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AB$6,'Job setup'!$D$9&gt;=AB$6,'Job setup'!$G$9="NO")),2,IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MAX(0,AB57-(IF('_JobDays'!R3,8,10)))*AB56))+((IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MIN(IF('_JobDays'!R3,8,10),AB57)*AB56)))-MIN(IF(OR(AB56&lt;=0,NOT('_JobDays'!R2)),0,IF(WEEKDAY(AB$6,1)=1,0,MIN(IF('_JobDays'!R3,8,10),AB57)*AB56)),MAX(0,40*MAX(1,AB56)-(Y58+Z58+AA58)))))</f>
+        <v>2</v>
       </c>
       <c r="AC59" s="61">
-        <f>IF(AND(AC56=1,AC57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),4,IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,AC56*AC57,IF('_JobDays'!S3,MAX(0,AC57-8)*AC56,0))))+((IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,0,IF('_JobDays'!S3,MIN(8,AC57)*AC56,AC56*AC57)))))-MIN(IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,IF(WEEKDAY(AC$6,1)=7,0,IF('_JobDays'!S3,MIN(8,AC57)*AC56,AC56*AC57)))),MAX(0,40*MAX(1,AC56)-(Y58+Z58+AA58+AB58)))))</f>
-        <v>4</v>
+        <f>IF(AND(AC56=1,AC57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AC$6,'Job setup'!$D$9&gt;=AC$6,'Job setup'!$G$9="NO")),12,IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MAX(0,AC57-(IF('_JobDays'!S3,8,10)))*AC56))+((IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MIN(IF('_JobDays'!S3,8,10),AC57)*AC56)))-MIN(IF(OR(AC56&lt;=0,NOT('_JobDays'!S2)),0,IF(WEEKDAY(AC$6,1)=1,0,MIN(IF('_JobDays'!S3,8,10),AC57)*AC56)),MAX(0,40*MAX(1,AC56)-(Y58+Z58+AA58+AB58)))))</f>
+        <v>12</v>
       </c>
       <c r="AD59" s="62">
-        <f>IF(AND(AD56=1,AD57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),12,IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,AD56*AD57,IF('_JobDays'!T3,MAX(0,AD57-8)*AD56,0))))+((IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,0,IF('_JobDays'!T3,MIN(8,AD57)*AD56,AD56*AD57)))))-MIN(IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,IF(WEEKDAY(AD$6,1)=7,0,IF('_JobDays'!T3,MIN(8,AD57)*AD56,AD56*AD57)))),MAX(0,40*MAX(1,AD56)-(Y58+Z58+AA58+AB58+AC58)))))</f>
+        <f>IF(AND(AD56=1,AD57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AD$6,'Job setup'!$D$9&gt;=AD$6,'Job setup'!$G$9="NO")),12,IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MAX(0,AD57-(IF('_JobDays'!T3,8,10)))*AD56))+((IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MIN(IF('_JobDays'!T3,8,10),AD57)*AD56)))-MIN(IF(OR(AD56&lt;=0,NOT('_JobDays'!T2)),0,IF(WEEKDAY(AD$6,1)=1,0,MIN(IF('_JobDays'!T3,8,10),AD57)*AD56)),MAX(0,40*MAX(1,AD56)-(Y58+Z58+AA58+AB58+AC58)))))</f>
         <v>12</v>
       </c>
       <c r="AE59" s="62">
-        <f>IF(AND(AE56=1,AE57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,AE56*AE57,IF('_JobDays'!U3,MAX(0,AE57-8)*AE56,0))))+((IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,0,IF('_JobDays'!U3,MIN(8,AE57)*AE56,AE56*AE57)))))-MIN(IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,IF(WEEKDAY(AE$6,1)=7,0,IF('_JobDays'!U3,MIN(8,AE57)*AE56,AE56*AE57)))),MAX(0,40*MAX(1,AE56)-(Y58+Z58+AA58+AB58+AC58+AD58)))))</f>
+        <f>IF(AND(AE56=1,AE57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AE$6,'Job setup'!$D$9&gt;=AE$6,'Job setup'!$G$9="NO")),0,IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MAX(0,AE57-(IF('_JobDays'!U3,8,10)))*AE56))+((IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MIN(IF('_JobDays'!U3,8,10),AE57)*AE56)))-MIN(IF(OR(AE56&lt;=0,NOT('_JobDays'!U2)),0,IF(WEEKDAY(AE$6,1)=1,0,MIN(IF('_JobDays'!U3,8,10),AE57)*AE56)),MAX(0,40*MAX(1,AE56)-(Y58+Z58+AA58+AB58+AC58+AD58)))))</f>
         <v>0</v>
       </c>
       <c r="AF59" s="61">
-        <f>IF(AND(AF56=1,AF57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),4,IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,AF56*AF57,IF('_JobDays'!V3,MAX(0,AF57-8)*AF56,0))))+((IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,0,IF('_JobDays'!V3,MIN(8,AF57)*AF56,AF56*AF57)))))-MIN(IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,IF(WEEKDAY(AF$6,1)=7,0,IF('_JobDays'!V3,MIN(8,AF57)*AF56,AF56*AF57)))),MAX(0,40*MAX(1,AF56)-(0)))))</f>
-        <v>4</v>
+        <f>IF(AND(AF56=1,AF57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AF$6,'Job setup'!$D$9&gt;=AF$6,'Job setup'!$G$9="NO")),2,IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MAX(0,AF57-(IF('_JobDays'!V3,8,10)))*AF56))+((IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MIN(IF('_JobDays'!V3,8,10),AF57)*AF56)))-MIN(IF(OR(AF56&lt;=0,NOT('_JobDays'!V2)),0,IF(WEEKDAY(AF$6,1)=1,0,MIN(IF('_JobDays'!V3,8,10),AF57)*AF56)),MAX(0,40*MAX(1,AF56)-(0)))))</f>
+        <v>2</v>
       </c>
       <c r="AG59" s="61">
-        <f>IF(AND(AG56=1,AG57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),4,IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,AG56*AG57,IF('_JobDays'!W3,MAX(0,AG57-8)*AG56,0))))+((IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,0,IF('_JobDays'!W3,MIN(8,AG57)*AG56,AG56*AG57)))))-MIN(IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,IF(WEEKDAY(AG$6,1)=7,0,IF('_JobDays'!W3,MIN(8,AG57)*AG56,AG56*AG57)))),MAX(0,40*MAX(1,AG56)-(AF58)))))</f>
-        <v>4</v>
+        <f>IF(AND(AG56=1,AG57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AG$6,'Job setup'!$D$9&gt;=AG$6,'Job setup'!$G$9="NO")),2,IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MAX(0,AG57-(IF('_JobDays'!W3,8,10)))*AG56))+((IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MIN(IF('_JobDays'!W3,8,10),AG57)*AG56)))-MIN(IF(OR(AG56&lt;=0,NOT('_JobDays'!W2)),0,IF(WEEKDAY(AG$6,1)=1,0,MIN(IF('_JobDays'!W3,8,10),AG57)*AG56)),MAX(0,40*MAX(1,AG56)-(AF58)))))</f>
+        <v>2</v>
       </c>
       <c r="AH59" s="61">
-        <f>IF(AND(AH56=1,AH57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),4,IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,AH56*AH57,IF('_JobDays'!X3,MAX(0,AH57-8)*AH56,0))))+((IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,0,IF('_JobDays'!X3,MIN(8,AH57)*AH56,AH56*AH57)))))-MIN(IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,IF(WEEKDAY(AH$6,1)=7,0,IF('_JobDays'!X3,MIN(8,AH57)*AH56,AH56*AH57)))),MAX(0,40*MAX(1,AH56)-(AF58+AG58)))))</f>
-        <v>4</v>
+        <f>IF(AND(AH56=1,AH57=12,AND('Job setup'!$B$9="ON",'Job setup'!$C$9&lt;=AH$6,'Job setup'!$D$9&gt;=AH$6,'Job setup'!$G$9="NO")),2,IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MAX(0,AH57-(IF('_JobDays'!X3,8,10)))*AH56))+((IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MIN(IF('_JobDays'!X3,8,10),AH57)*AH56)))-MIN(IF(OR(AH56&lt;=0,NOT('_JobDays'!X2)),0,IF(WEEKDAY(AH$6,1)=1,0,MIN(IF('_JobDays'!X3,8,10),AH57)*AH56)),MAX(0,40*MAX(1,AH56)-(AF58+AG58)))))</f>
+        <v>2</v>
       </c>
       <c r="AI59" s="61">
-        <f>IF(AND(AI56=1,AI57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,AI56*AI57,IF('_JobDays'!Y3,MAX(0,AI57-8)*AI56,0))))+((IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,0,IF('_JobDays'!Y3,MIN(8,AI57)*AI56,AI56*AI57)))))-MIN(IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,IF(WEEKDAY(AI$6,1)=7,0,IF('_JobDays'!Y3,MIN(8,AI57)*AI56,AI56*AI57)))),MAX(0,40*MAX(1,AI56)-(0)))))</f>
+        <f>IF(AND(AI56=0,AI57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MAX(0,AI57-(IF('_JobDays'!Y3,8,10)))*AI56))+((IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI57)*AI56)))-MIN(IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,0,MIN(IF('_JobDays'!Y3,8,10),AI57)*AI56)),MAX(0,40*MAX(1,AI56)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AJ59" s="61">
-        <f>IF(AND(AJ56=1,AJ57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,AJ56*AJ57,IF('_JobDays'!Z3,MAX(0,AJ57-8)*AJ56,0))))+((IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,0,IF('_JobDays'!Z3,MIN(8,AJ57)*AJ56,AJ56*AJ57)))))-MIN(IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,IF(WEEKDAY(AJ$6,1)=7,0,IF('_JobDays'!Z3,MIN(8,AJ57)*AJ56,AJ56*AJ57)))),MAX(0,40*MAX(1,AJ56)-(AI58)))))</f>
+        <f>IF(AND(AJ56=0,AJ57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MAX(0,AJ57-(IF('_JobDays'!Z3,8,10)))*AJ56))+((IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ57)*AJ56)))-MIN(IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,0,MIN(IF('_JobDays'!Z3,8,10),AJ57)*AJ56)),MAX(0,40*MAX(1,AJ56)-(AI58)))))</f>
         <v>0</v>
       </c>
       <c r="AK59" s="62">
-        <f>IF(AND(AK56=0,AK57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,AK56*AK57,IF('_JobDays'!AA3,MAX(0,AK57-8)*AK56,0))))+((IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,0,IF('_JobDays'!AA3,MIN(8,AK57)*AK56,AK56*AK57)))))-MIN(IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,IF(WEEKDAY(AK$6,1)=7,0,IF('_JobDays'!AA3,MIN(8,AK57)*AK56,AK56*AK57)))),MAX(0,40*MAX(1,AK56)-(0)))))</f>
+        <f>IF(AND(AK56=0,AK57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AK$6,'Job setup'!$D$11&gt;=AK$6,'Job setup'!$G$11="YES")),0,IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MAX(0,AK57-(IF('_JobDays'!AA3,8,10)))*AK56))+((IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK57)*AK56)))-MIN(IF(OR(AK56&lt;=0,NOT('_JobDays'!AA2)),0,IF(WEEKDAY(AK$6,1)=1,0,MIN(IF('_JobDays'!AA3,8,10),AK57)*AK56)),MAX(0,40*MAX(1,AK56)-(AI58+AJ58)))))</f>
         <v>0</v>
       </c>
       <c r="AL59" s="62">
-        <f>IF(AND(AL56=0,AL57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,AL56*AL57,IF('_JobDays'!AB3,MAX(0,AL57-8)*AL56,0))))+((IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,0,IF('_JobDays'!AB3,MIN(8,AL57)*AL56,AL56*AL57)))))-MIN(IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,IF(WEEKDAY(AL$6,1)=7,0,IF('_JobDays'!AB3,MIN(8,AL57)*AL56,AL56*AL57)))),MAX(0,40*MAX(1,AL56)-(AK58)))))</f>
+        <f>IF(AND(AL56=0,AL57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AL$6,'Job setup'!$D$11&gt;=AL$6,'Job setup'!$G$11="YES")),0,IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MAX(0,AL57-(IF('_JobDays'!AB3,8,10)))*AL56))+((IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL57)*AL56)))-MIN(IF(OR(AL56&lt;=0,NOT('_JobDays'!AB2)),0,IF(WEEKDAY(AL$6,1)=1,0,MIN(IF('_JobDays'!AB3,8,10),AL57)*AL56)),MAX(0,40*MAX(1,AL56)-(AI58+AJ58+AK58)))))</f>
         <v>0</v>
       </c>
       <c r="AM59" s="61">
-        <f>IF(AND(AM56=1,AM57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,AM56*AM57,IF('_JobDays'!AC3,MAX(0,AM57-8)*AM56,0))))+((IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,0,IF('_JobDays'!AC3,MIN(8,AM57)*AM56,AM56*AM57)))))-MIN(IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,IF(WEEKDAY(AM$6,1)=7,0,IF('_JobDays'!AC3,MIN(8,AM57)*AM56,AM56*AM57)))),MAX(0,40*MAX(1,AM56)-(0)))))</f>
+        <f>IF(AND(AM56=0,AM57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MAX(0,AM57-(IF('_JobDays'!AC3,8,10)))*AM56))+((IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM57)*AM56)))-MIN(IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,0,MIN(IF('_JobDays'!AC3,8,10),AM57)*AM56)),MAX(0,40*MAX(1,AM56)-(0)))))</f>
         <v>0</v>
       </c>
       <c r="AN59" s="61">
-        <f>IF(AND(AN56=1,AN57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,AN56*AN57,IF('_JobDays'!AD3,MAX(0,AN57-8)*AN56,0))))+((IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,0,IF('_JobDays'!AD3,MIN(8,AN57)*AN56,AN56*AN57)))))-MIN(IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,IF(WEEKDAY(AN$6,1)=7,0,IF('_JobDays'!AD3,MIN(8,AN57)*AN56,AN56*AN57)))),MAX(0,40*MAX(1,AN56)-(AM58)))))</f>
+        <f>IF(AND(AN56=0,AN57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MAX(0,AN57-(IF('_JobDays'!AD3,8,10)))*AN56))+((IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN57)*AN56)))-MIN(IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,0,MIN(IF('_JobDays'!AD3,8,10),AN57)*AN56)),MAX(0,40*MAX(1,AN56)-(AM58)))))</f>
         <v>0</v>
       </c>
       <c r="AO59" s="61">
-        <f>IF(AND(AO56=1,AO57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,AO56*AO57,IF('_JobDays'!AE3,MAX(0,AO57-8)*AO56,0))))+((IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,0,IF('_JobDays'!AE3,MIN(8,AO57)*AO56,AO56*AO57)))))-MIN(IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,IF(WEEKDAY(AO$6,1)=7,0,IF('_JobDays'!AE3,MIN(8,AO57)*AO56,AO56*AO57)))),MAX(0,40*MAX(1,AO56)-(AM58+AN58)))))</f>
+        <f>IF(AND(AO56=0,AO57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MAX(0,AO57-(IF('_JobDays'!AE3,8,10)))*AO56))+((IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO57)*AO56)))-MIN(IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,0,MIN(IF('_JobDays'!AE3,8,10),AO57)*AO56)),MAX(0,40*MAX(1,AO56)-(AM58+AN58)))))</f>
         <v>0</v>
       </c>
       <c r="AP59" s="63">
-        <f>IF(AND(AP56=1,AP57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,AP56*AP57,IF('_JobDays'!AF3,MAX(0,AP57-8)*AP56,0))))+((IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,0,IF('_JobDays'!AF3,MIN(8,AP57)*AP56,AP56*AP57)))))-MIN(IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,IF(WEEKDAY(AP$6,1)=7,0,IF('_JobDays'!AF3,MIN(8,AP57)*AP56,AP56*AP57)))),MAX(0,40*MAX(1,AP56)-(AM58+AN58+AO58)))))</f>
+        <f>IF(AND(AP56=0,AP57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MAX(0,AP57-(IF('_JobDays'!AF3,8,10)))*AP56))+((IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP57)*AP56)))-MIN(IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,0,MIN(IF('_JobDays'!AF3,8,10),AP57)*AP56)),MAX(0,40*MAX(1,AP56)-(AM58+AN58+AO58)))))</f>
         <v>0</v>
       </c>
       <c r="OU59" s="28" t="s">
@@ -14374,15 +14374,15 @@
       </c>
     </row>
     <row r="60" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A60" s="43"/>
+      <c r="A60" s="72"/>
       <c r="B60" s="44"/>
       <c r="C60" s="59">
         <f>H55*N(D60)</f>
-        <v>4833.6</v>
+        <v>3681.3599999999997</v>
       </c>
       <c r="D60" s="59">
         <f>IF(TRIM(B55)="","No rate",IFERROR(INDEX('Rate Tables'!E$7:E$161,MATCH(B55,'Rate Tables'!A$7:A$161,0)),"No rate"))</f>
-        <v>201.4</v>
+        <v>153.39</v>
       </c>
       <c r="E60" s="53" t="s">
         <v>61</v>
@@ -14489,11 +14489,11 @@
         <v>0</v>
       </c>
       <c r="AI60" s="61">
-        <f>IF(AND(AI56=1,AI57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI56*AI57,0)))</f>
+        <f>IF(AND(AI56=0,AI57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AI$6,'Job setup'!$D$11&gt;=AI$6,'Job setup'!$G$11="YES")),0,IF(OR(AI56&lt;=0,NOT('_JobDays'!Y2)),0,IF(WEEKDAY(AI$6,1)=1,AI56*AI57,0)))</f>
         <v>0</v>
       </c>
       <c r="AJ60" s="61">
-        <f>IF(AND(AJ56=1,AJ57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ56*AJ57,0)))</f>
+        <f>IF(AND(AJ56=0,AJ57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AJ$6,'Job setup'!$D$11&gt;=AJ$6,'Job setup'!$G$11="YES")),0,IF(OR(AJ56&lt;=0,NOT('_JobDays'!Z2)),0,IF(WEEKDAY(AJ$6,1)=1,AJ56*AJ57,0)))</f>
         <v>0</v>
       </c>
       <c r="AK60" s="62">
@@ -14505,19 +14505,19 @@
         <v>0</v>
       </c>
       <c r="AM60" s="61">
-        <f>IF(AND(AM56=1,AM57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM56*AM57,0)))</f>
+        <f>IF(AND(AM56=0,AM57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AM$6,'Job setup'!$D$11&gt;=AM$6,'Job setup'!$G$11="YES")),0,IF(OR(AM56&lt;=0,NOT('_JobDays'!AC2)),0,IF(WEEKDAY(AM$6,1)=1,AM56*AM57,0)))</f>
         <v>0</v>
       </c>
       <c r="AN60" s="61">
-        <f>IF(AND(AN56=1,AN57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN56*AN57,0)))</f>
+        <f>IF(AND(AN56=0,AN57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AN$6,'Job setup'!$D$11&gt;=AN$6,'Job setup'!$G$11="YES")),0,IF(OR(AN56&lt;=0,NOT('_JobDays'!AD2)),0,IF(WEEKDAY(AN$6,1)=1,AN56*AN57,0)))</f>
         <v>0</v>
       </c>
       <c r="AO60" s="61">
-        <f>IF(AND(AO56=1,AO57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO56*AO57,0)))</f>
+        <f>IF(AND(AO56=0,AO57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AO$6,'Job setup'!$D$11&gt;=AO$6,'Job setup'!$G$11="YES")),0,IF(OR(AO56&lt;=0,NOT('_JobDays'!AE2)),0,IF(WEEKDAY(AO$6,1)=1,AO56*AO57,0)))</f>
         <v>0</v>
       </c>
       <c r="AP60" s="63">
-        <f>IF(AND(AP56=1,AP57=8,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP56*AP57,0)))</f>
+        <f>IF(AND(AP56=0,AP57=0,AND('Job setup'!$B$11="ON",'Job setup'!$C$11&lt;=AP$6,'Job setup'!$D$11&gt;=AP$6,'Job setup'!$G$11="YES")),0,IF(OR(AP56&lt;=0,NOT('_JobDays'!AF2)),0,IF(WEEKDAY(AP$6,1)=1,AP56*AP57,0)))</f>
         <v>0</v>
       </c>
       <c r="OU60" s="28" t="s">
@@ -14525,7 +14525,7 @@
       </c>
     </row>
     <row r="61" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
-      <c r="A61" s="43"/>
+      <c r="A61" s="72"/>
       <c r="B61" s="44"/>
       <c r="C61" s="65">
         <f>I55*D61</f>
@@ -14688,10 +14688,10 @@
     </row>
     <row r="63" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
       <c r="A63" s="72" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B63" s="44" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C63" s="45">
         <f>J63</f>
@@ -17209,7 +17209,7 @@
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
       <c r="A15" s="72" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B15" s="44" t="s">
         <v>75</v>
@@ -19628,7 +19628,7 @@
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
       <c r="A15" s="72" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B15" s="44" t="s">
         <v>78</v>
@@ -22051,7 +22051,7 @@
     </row>
     <row r="15" ht="16" customHeight="1" spans="1:411" x14ac:dyDescent="0.25">
       <c r="A15" s="72" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B15" s="75" t="s">
         <v>81</v>

</xml_diff>

<commit_message>
Add daily/weekly/monthly Period lists on COE and rental sheets.
Desk period strings live on _Lists. COE, Equipment Rental, Tension, and Crane Period cells stay unlocked with that dropdown so offline edits round-trip.

Co-authored-by: robertmhenderson582-ops <robertmhenderson582-ops@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/look-samples/v151_real_cat2.xlsx
+++ b/look-samples/v151_real_cat2.xlsx
@@ -41,7 +41,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Misc Costs'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'Rate Tables'!$A1:$F168</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'Rate Tables'!$6:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="10">'_Lists'!$A1:$I94</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="10">'_Lists'!$A1:$J94</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'_Lists'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="11">'_JobDays'!$A1:$AF7</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'_JobDays'!$6:$6</definedName>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="904" uniqueCount="288">
   <si>
     <t>HIT SQUAD / PROJECT CONTROLS</t>
   </si>
@@ -891,6 +891,9 @@
   </si>
   <si>
     <t>9</t>
+  </si>
+  <si>
+    <t>weekly</t>
   </si>
   <si>
     <t>4×10 — all 10 ST</t>
@@ -5538,7 +5541,7 @@
     <tabColor rgb="FF0F5F6D"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:J94"/>
   <sheetFormatPr defaultRowHeight="0" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1" zeroHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -5547,7 +5550,7 @@
     <col min="6" max="16384" width="9" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>209</v>
       </c>
@@ -5567,8 +5570,11 @@
       <c r="I1" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>210</v>
       </c>
@@ -5588,8 +5594,11 @@
       <c r="I2" s="2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J2" s="2" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>211</v>
       </c>
@@ -5598,17 +5607,20 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I3" s="85"/>
-    </row>
-    <row r="4" ht="6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J3" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" ht="6" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="86" t="s">
         <v>121</v>
       </c>
@@ -5623,17 +5635,18 @@
         <v>212</v>
       </c>
       <c r="F4" s="86" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G4" s="86" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H4" s="86" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="I4" s="23"/>
-    </row>
-    <row r="5" ht="6" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J4" s="23"/>
+    </row>
+    <row r="5" ht="6" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="86" t="s">
         <v>122</v>
       </c>
@@ -5650,11 +5663,12 @@
       <c r="F5" s="23"/>
       <c r="G5" s="23"/>
       <c r="H5" s="86" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="I5" s="23"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J5" s="23"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
         <v>123</v>
       </c>
@@ -5672,8 +5686,9 @@
       <c r="G6" s="87"/>
       <c r="H6" s="87"/>
       <c r="I6" s="87"/>
-    </row>
-    <row r="7" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J6" s="87"/>
+    </row>
+    <row r="7" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
         <v>124</v>
       </c>
@@ -5691,8 +5706,9 @@
       <c r="G7" s="84"/>
       <c r="H7" s="84"/>
       <c r="I7" s="84"/>
-    </row>
-    <row r="8" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J7" s="84"/>
+    </row>
+    <row r="8" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="29" t="s">
         <v>125</v>
       </c>
@@ -5708,8 +5724,9 @@
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
       <c r="I8" s="20"/>
-    </row>
-    <row r="9" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J8" s="20"/>
+    </row>
+    <row r="9" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
         <v>126</v>
       </c>
@@ -5725,8 +5742,9 @@
       <c r="G9" s="84"/>
       <c r="H9" s="84"/>
       <c r="I9" s="84"/>
-    </row>
-    <row r="10" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J9" s="84"/>
+    </row>
+    <row r="10" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="29" t="s">
         <v>127</v>
       </c>
@@ -5742,8 +5760,9 @@
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
       <c r="I10" s="20"/>
-    </row>
-    <row r="11" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J10" s="20"/>
+    </row>
+    <row r="11" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
         <v>128</v>
       </c>
@@ -5759,8 +5778,9 @@
       <c r="G11" s="84"/>
       <c r="H11" s="84"/>
       <c r="I11" s="84"/>
-    </row>
-    <row r="12" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J11" s="84"/>
+    </row>
+    <row r="12" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="29" t="s">
         <v>129</v>
       </c>
@@ -5776,8 +5796,9 @@
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
       <c r="I12" s="20"/>
-    </row>
-    <row r="13" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J12" s="20"/>
+    </row>
+    <row r="13" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
         <v>130</v>
       </c>
@@ -5793,8 +5814,9 @@
       <c r="G13" s="84"/>
       <c r="H13" s="84"/>
       <c r="I13" s="84"/>
-    </row>
-    <row r="14" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J13" s="84"/>
+    </row>
+    <row r="14" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="29" t="s">
         <v>131</v>
       </c>
@@ -5810,8 +5832,9 @@
       <c r="G14" s="20"/>
       <c r="H14" s="20"/>
       <c r="I14" s="20"/>
-    </row>
-    <row r="15" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J14" s="20"/>
+    </row>
+    <row r="15" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
         <v>132</v>
       </c>
@@ -5827,8 +5850,9 @@
       <c r="G15" s="84"/>
       <c r="H15" s="84"/>
       <c r="I15" s="84"/>
-    </row>
-    <row r="16" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J15" s="84"/>
+    </row>
+    <row r="16" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="29" t="s">
         <v>133</v>
       </c>
@@ -5844,8 +5868,9 @@
       <c r="G16" s="20"/>
       <c r="H16" s="20"/>
       <c r="I16" s="20"/>
-    </row>
-    <row r="17" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J16" s="20"/>
+    </row>
+    <row r="17" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
         <v>134</v>
       </c>
@@ -5861,8 +5886,9 @@
       <c r="G17" s="84"/>
       <c r="H17" s="84"/>
       <c r="I17" s="84"/>
-    </row>
-    <row r="18" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J17" s="84"/>
+    </row>
+    <row r="18" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="29" t="s">
         <v>135</v>
       </c>
@@ -5878,8 +5904,9 @@
       <c r="G18" s="20"/>
       <c r="H18" s="20"/>
       <c r="I18" s="20"/>
-    </row>
-    <row r="19" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J18" s="20"/>
+    </row>
+    <row r="19" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
         <v>63</v>
       </c>
@@ -5895,8 +5922,9 @@
       <c r="G19" s="84"/>
       <c r="H19" s="84"/>
       <c r="I19" s="84"/>
-    </row>
-    <row r="20" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J19" s="84"/>
+    </row>
+    <row r="20" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="29" t="s">
         <v>136</v>
       </c>
@@ -5912,8 +5940,9 @@
       <c r="G20" s="20"/>
       <c r="H20" s="20"/>
       <c r="I20" s="20"/>
-    </row>
-    <row r="21" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J20" s="20"/>
+    </row>
+    <row r="21" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
         <v>137</v>
       </c>
@@ -5929,8 +5958,9 @@
       <c r="G21" s="84"/>
       <c r="H21" s="84"/>
       <c r="I21" s="84"/>
-    </row>
-    <row r="22" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J21" s="84"/>
+    </row>
+    <row r="22" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="29" t="s">
         <v>138</v>
       </c>
@@ -5946,8 +5976,9 @@
       <c r="G22" s="20"/>
       <c r="H22" s="20"/>
       <c r="I22" s="20"/>
-    </row>
-    <row r="23" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J22" s="20"/>
+    </row>
+    <row r="23" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
         <v>139</v>
       </c>
@@ -5963,8 +5994,9 @@
       <c r="G23" s="84"/>
       <c r="H23" s="84"/>
       <c r="I23" s="84"/>
-    </row>
-    <row r="24" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J23" s="84"/>
+    </row>
+    <row r="24" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="29" t="s">
         <v>140</v>
       </c>
@@ -5980,8 +6012,9 @@
       <c r="G24" s="20"/>
       <c r="H24" s="20"/>
       <c r="I24" s="20"/>
-    </row>
-    <row r="25" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J24" s="20"/>
+    </row>
+    <row r="25" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
         <v>141</v>
       </c>
@@ -5997,8 +6030,9 @@
       <c r="G25" s="84"/>
       <c r="H25" s="84"/>
       <c r="I25" s="84"/>
-    </row>
-    <row r="26" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J25" s="84"/>
+    </row>
+    <row r="26" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="29" t="s">
         <v>142</v>
       </c>
@@ -6014,8 +6048,9 @@
       <c r="G26" s="20"/>
       <c r="H26" s="20"/>
       <c r="I26" s="20"/>
-    </row>
-    <row r="27" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J26" s="20"/>
+    </row>
+    <row r="27" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
         <v>143</v>
       </c>
@@ -6031,8 +6066,9 @@
       <c r="G27" s="84"/>
       <c r="H27" s="84"/>
       <c r="I27" s="84"/>
-    </row>
-    <row r="28" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J27" s="84"/>
+    </row>
+    <row r="28" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="29" t="s">
         <v>144</v>
       </c>
@@ -6048,8 +6084,9 @@
       <c r="G28" s="20"/>
       <c r="H28" s="20"/>
       <c r="I28" s="20"/>
-    </row>
-    <row r="29" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J28" s="20"/>
+    </row>
+    <row r="29" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
         <v>145</v>
       </c>
@@ -6065,8 +6102,9 @@
       <c r="G29" s="84"/>
       <c r="H29" s="84"/>
       <c r="I29" s="84"/>
-    </row>
-    <row r="30" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J29" s="84"/>
+    </row>
+    <row r="30" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="29" t="s">
         <v>146</v>
       </c>
@@ -6082,8 +6120,9 @@
       <c r="G30" s="20"/>
       <c r="H30" s="20"/>
       <c r="I30" s="20"/>
-    </row>
-    <row r="31" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J30" s="20"/>
+    </row>
+    <row r="31" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
         <v>147</v>
       </c>
@@ -6099,8 +6138,9 @@
       <c r="G31" s="84"/>
       <c r="H31" s="84"/>
       <c r="I31" s="84"/>
-    </row>
-    <row r="32" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J31" s="84"/>
+    </row>
+    <row r="32" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="29" t="s">
         <v>148</v>
       </c>
@@ -6116,8 +6156,9 @@
       <c r="G32" s="20"/>
       <c r="H32" s="20"/>
       <c r="I32" s="20"/>
-    </row>
-    <row r="33" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J32" s="20"/>
+    </row>
+    <row r="33" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
         <v>149</v>
       </c>
@@ -6133,8 +6174,9 @@
       <c r="G33" s="84"/>
       <c r="H33" s="84"/>
       <c r="I33" s="84"/>
-    </row>
-    <row r="34" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J33" s="84"/>
+    </row>
+    <row r="34" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="29" t="s">
         <v>150</v>
       </c>
@@ -6150,8 +6192,9 @@
       <c r="G34" s="20"/>
       <c r="H34" s="20"/>
       <c r="I34" s="20"/>
-    </row>
-    <row r="35" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J34" s="20"/>
+    </row>
+    <row r="35" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
         <v>151</v>
       </c>
@@ -6167,8 +6210,9 @@
       <c r="G35" s="84"/>
       <c r="H35" s="84"/>
       <c r="I35" s="84"/>
-    </row>
-    <row r="36" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J35" s="84"/>
+    </row>
+    <row r="36" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="29" t="s">
         <v>152</v>
       </c>
@@ -6184,8 +6228,9 @@
       <c r="G36" s="20"/>
       <c r="H36" s="20"/>
       <c r="I36" s="20"/>
-    </row>
-    <row r="37" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J36" s="20"/>
+    </row>
+    <row r="37" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
         <v>153</v>
       </c>
@@ -6201,8 +6246,9 @@
       <c r="G37" s="84"/>
       <c r="H37" s="84"/>
       <c r="I37" s="84"/>
-    </row>
-    <row r="38" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J37" s="84"/>
+    </row>
+    <row r="38" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="29" t="s">
         <v>154</v>
       </c>
@@ -6218,8 +6264,9 @@
       <c r="G38" s="20"/>
       <c r="H38" s="20"/>
       <c r="I38" s="20"/>
-    </row>
-    <row r="39" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J38" s="20"/>
+    </row>
+    <row r="39" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
         <v>155</v>
       </c>
@@ -6235,8 +6282,9 @@
       <c r="G39" s="84"/>
       <c r="H39" s="84"/>
       <c r="I39" s="84"/>
-    </row>
-    <row r="40" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J39" s="84"/>
+    </row>
+    <row r="40" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="29" t="s">
         <v>156</v>
       </c>
@@ -6252,8 +6300,9 @@
       <c r="G40" s="20"/>
       <c r="H40" s="20"/>
       <c r="I40" s="20"/>
-    </row>
-    <row r="41" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J40" s="20"/>
+    </row>
+    <row r="41" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
         <v>157</v>
       </c>
@@ -6269,8 +6318,9 @@
       <c r="G41" s="84"/>
       <c r="H41" s="84"/>
       <c r="I41" s="84"/>
-    </row>
-    <row r="42" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J41" s="84"/>
+    </row>
+    <row r="42" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="29" t="s">
         <v>158</v>
       </c>
@@ -6286,8 +6336,9 @@
       <c r="G42" s="20"/>
       <c r="H42" s="20"/>
       <c r="I42" s="20"/>
-    </row>
-    <row r="43" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J42" s="20"/>
+    </row>
+    <row r="43" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
         <v>159</v>
       </c>
@@ -6303,8 +6354,9 @@
       <c r="G43" s="84"/>
       <c r="H43" s="84"/>
       <c r="I43" s="84"/>
-    </row>
-    <row r="44" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J43" s="84"/>
+    </row>
+    <row r="44" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="29" t="s">
         <v>160</v>
       </c>
@@ -6320,8 +6372,9 @@
       <c r="G44" s="20"/>
       <c r="H44" s="20"/>
       <c r="I44" s="20"/>
-    </row>
-    <row r="45" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J44" s="20"/>
+    </row>
+    <row r="45" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
         <v>161</v>
       </c>
@@ -6337,8 +6390,9 @@
       <c r="G45" s="84"/>
       <c r="H45" s="84"/>
       <c r="I45" s="84"/>
-    </row>
-    <row r="46" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J45" s="84"/>
+    </row>
+    <row r="46" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="29" t="s">
         <v>162</v>
       </c>
@@ -6354,8 +6408,9 @@
       <c r="G46" s="20"/>
       <c r="H46" s="20"/>
       <c r="I46" s="20"/>
-    </row>
-    <row r="47" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J46" s="20"/>
+    </row>
+    <row r="47" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
         <v>163</v>
       </c>
@@ -6371,8 +6426,9 @@
       <c r="G47" s="84"/>
       <c r="H47" s="84"/>
       <c r="I47" s="84"/>
-    </row>
-    <row r="48" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J47" s="84"/>
+    </row>
+    <row r="48" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="29" t="s">
         <v>164</v>
       </c>
@@ -6388,8 +6444,9 @@
       <c r="G48" s="20"/>
       <c r="H48" s="20"/>
       <c r="I48" s="20"/>
-    </row>
-    <row r="49" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J48" s="20"/>
+    </row>
+    <row r="49" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
         <v>165</v>
       </c>
@@ -6405,8 +6462,9 @@
       <c r="G49" s="84"/>
       <c r="H49" s="84"/>
       <c r="I49" s="84"/>
-    </row>
-    <row r="50" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J49" s="84"/>
+    </row>
+    <row r="50" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="29" t="s">
         <v>166</v>
       </c>
@@ -6422,8 +6480,9 @@
       <c r="G50" s="20"/>
       <c r="H50" s="20"/>
       <c r="I50" s="20"/>
-    </row>
-    <row r="51" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J50" s="20"/>
+    </row>
+    <row r="51" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
         <v>167</v>
       </c>
@@ -6439,8 +6498,9 @@
       <c r="G51" s="84"/>
       <c r="H51" s="84"/>
       <c r="I51" s="84"/>
-    </row>
-    <row r="52" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J51" s="84"/>
+    </row>
+    <row r="52" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="29" t="s">
         <v>168</v>
       </c>
@@ -6454,8 +6514,9 @@
       <c r="G52" s="20"/>
       <c r="H52" s="20"/>
       <c r="I52" s="20"/>
-    </row>
-    <row r="53" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J52" s="20"/>
+    </row>
+    <row r="53" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
         <v>169</v>
       </c>
@@ -6469,8 +6530,9 @@
       <c r="G53" s="84"/>
       <c r="H53" s="84"/>
       <c r="I53" s="84"/>
-    </row>
-    <row r="54" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J53" s="84"/>
+    </row>
+    <row r="54" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="29" t="s">
         <v>170</v>
       </c>
@@ -6484,8 +6546,9 @@
       <c r="G54" s="20"/>
       <c r="H54" s="20"/>
       <c r="I54" s="20"/>
-    </row>
-    <row r="55" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J54" s="20"/>
+    </row>
+    <row r="55" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
         <v>171</v>
       </c>
@@ -6499,8 +6562,9 @@
       <c r="G55" s="84"/>
       <c r="H55" s="84"/>
       <c r="I55" s="84"/>
-    </row>
-    <row r="56" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J55" s="84"/>
+    </row>
+    <row r="56" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="29" t="s">
         <v>172</v>
       </c>
@@ -6514,8 +6578,9 @@
       <c r="G56" s="20"/>
       <c r="H56" s="20"/>
       <c r="I56" s="20"/>
-    </row>
-    <row r="57" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J56" s="20"/>
+    </row>
+    <row r="57" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="12" t="s">
         <v>173</v>
       </c>
@@ -6529,8 +6594,9 @@
       <c r="G57" s="84"/>
       <c r="H57" s="84"/>
       <c r="I57" s="84"/>
-    </row>
-    <row r="58" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J57" s="84"/>
+    </row>
+    <row r="58" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="29" t="s">
         <v>174</v>
       </c>
@@ -6544,8 +6610,9 @@
       <c r="G58" s="20"/>
       <c r="H58" s="20"/>
       <c r="I58" s="20"/>
-    </row>
-    <row r="59" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J58" s="20"/>
+    </row>
+    <row r="59" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="12" t="s">
         <v>175</v>
       </c>
@@ -6557,8 +6624,9 @@
       <c r="G59" s="84"/>
       <c r="H59" s="84"/>
       <c r="I59" s="84"/>
-    </row>
-    <row r="60" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J59" s="84"/>
+    </row>
+    <row r="60" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="29" t="s">
         <v>176</v>
       </c>
@@ -6570,8 +6638,9 @@
       <c r="G60" s="20"/>
       <c r="H60" s="20"/>
       <c r="I60" s="20"/>
-    </row>
-    <row r="61" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J60" s="20"/>
+    </row>
+    <row r="61" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="12" t="s">
         <v>177</v>
       </c>
@@ -6583,8 +6652,9 @@
       <c r="G61" s="84"/>
       <c r="H61" s="84"/>
       <c r="I61" s="84"/>
-    </row>
-    <row r="62" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J61" s="84"/>
+    </row>
+    <row r="62" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="29" t="s">
         <v>178</v>
       </c>
@@ -6596,8 +6666,9 @@
       <c r="G62" s="20"/>
       <c r="H62" s="20"/>
       <c r="I62" s="20"/>
-    </row>
-    <row r="63" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J62" s="20"/>
+    </row>
+    <row r="63" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
         <v>179</v>
       </c>
@@ -6609,8 +6680,9 @@
       <c r="G63" s="84"/>
       <c r="H63" s="84"/>
       <c r="I63" s="84"/>
-    </row>
-    <row r="64" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J63" s="84"/>
+    </row>
+    <row r="64" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="29" t="s">
         <v>180</v>
       </c>
@@ -6622,8 +6694,9 @@
       <c r="G64" s="20"/>
       <c r="H64" s="20"/>
       <c r="I64" s="20"/>
-    </row>
-    <row r="65" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J64" s="20"/>
+    </row>
+    <row r="65" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="12" t="s">
         <v>181</v>
       </c>
@@ -6635,8 +6708,9 @@
       <c r="G65" s="84"/>
       <c r="H65" s="84"/>
       <c r="I65" s="84"/>
-    </row>
-    <row r="66" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J65" s="84"/>
+    </row>
+    <row r="66" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="29" t="s">
         <v>182</v>
       </c>
@@ -6648,8 +6722,9 @@
       <c r="G66" s="20"/>
       <c r="H66" s="20"/>
       <c r="I66" s="20"/>
-    </row>
-    <row r="67" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J66" s="20"/>
+    </row>
+    <row r="67" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="12" t="s">
         <v>183</v>
       </c>
@@ -6661,8 +6736,9 @@
       <c r="G67" s="84"/>
       <c r="H67" s="84"/>
       <c r="I67" s="84"/>
-    </row>
-    <row r="68" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J67" s="84"/>
+    </row>
+    <row r="68" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="29" t="s">
         <v>184</v>
       </c>
@@ -6674,8 +6750,9 @@
       <c r="G68" s="20"/>
       <c r="H68" s="20"/>
       <c r="I68" s="20"/>
-    </row>
-    <row r="69" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J68" s="20"/>
+    </row>
+    <row r="69" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="12" t="s">
         <v>185</v>
       </c>
@@ -6687,8 +6764,9 @@
       <c r="G69" s="84"/>
       <c r="H69" s="84"/>
       <c r="I69" s="84"/>
-    </row>
-    <row r="70" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J69" s="84"/>
+    </row>
+    <row r="70" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="29" t="s">
         <v>186</v>
       </c>
@@ -6700,8 +6778,9 @@
       <c r="G70" s="20"/>
       <c r="H70" s="20"/>
       <c r="I70" s="20"/>
-    </row>
-    <row r="71" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J70" s="20"/>
+    </row>
+    <row r="71" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="12" t="s">
         <v>187</v>
       </c>
@@ -6713,8 +6792,9 @@
       <c r="G71" s="84"/>
       <c r="H71" s="84"/>
       <c r="I71" s="84"/>
-    </row>
-    <row r="72" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J71" s="84"/>
+    </row>
+    <row r="72" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="29" t="s">
         <v>188</v>
       </c>
@@ -6726,8 +6806,9 @@
       <c r="G72" s="20"/>
       <c r="H72" s="20"/>
       <c r="I72" s="20"/>
-    </row>
-    <row r="73" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J72" s="20"/>
+    </row>
+    <row r="73" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="12" t="s">
         <v>189</v>
       </c>
@@ -6739,8 +6820,9 @@
       <c r="G73" s="84"/>
       <c r="H73" s="84"/>
       <c r="I73" s="84"/>
-    </row>
-    <row r="74" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J73" s="84"/>
+    </row>
+    <row r="74" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="29" t="s">
         <v>190</v>
       </c>
@@ -6752,8 +6834,9 @@
       <c r="G74" s="20"/>
       <c r="H74" s="20"/>
       <c r="I74" s="20"/>
-    </row>
-    <row r="75" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J74" s="20"/>
+    </row>
+    <row r="75" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
         <v>191</v>
       </c>
@@ -6765,8 +6848,9 @@
       <c r="G75" s="84"/>
       <c r="H75" s="84"/>
       <c r="I75" s="84"/>
-    </row>
-    <row r="76" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J75" s="84"/>
+    </row>
+    <row r="76" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="29" t="s">
         <v>192</v>
       </c>
@@ -6778,8 +6862,9 @@
       <c r="G76" s="20"/>
       <c r="H76" s="20"/>
       <c r="I76" s="20"/>
-    </row>
-    <row r="77" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J76" s="20"/>
+    </row>
+    <row r="77" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="12" t="s">
         <v>193</v>
       </c>
@@ -6791,8 +6876,9 @@
       <c r="G77" s="84"/>
       <c r="H77" s="84"/>
       <c r="I77" s="84"/>
-    </row>
-    <row r="78" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J77" s="84"/>
+    </row>
+    <row r="78" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="29" t="s">
         <v>194</v>
       </c>
@@ -6804,8 +6890,9 @@
       <c r="G78" s="20"/>
       <c r="H78" s="20"/>
       <c r="I78" s="20"/>
-    </row>
-    <row r="79" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J78" s="20"/>
+    </row>
+    <row r="79" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="12" t="s">
         <v>195</v>
       </c>
@@ -6817,8 +6904,9 @@
       <c r="G79" s="84"/>
       <c r="H79" s="84"/>
       <c r="I79" s="84"/>
-    </row>
-    <row r="80" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J79" s="84"/>
+    </row>
+    <row r="80" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="29" t="s">
         <v>196</v>
       </c>
@@ -6830,8 +6918,9 @@
       <c r="G80" s="20"/>
       <c r="H80" s="20"/>
       <c r="I80" s="20"/>
-    </row>
-    <row r="81" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J80" s="20"/>
+    </row>
+    <row r="81" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="12" t="s">
         <v>197</v>
       </c>
@@ -6843,8 +6932,9 @@
       <c r="G81" s="84"/>
       <c r="H81" s="84"/>
       <c r="I81" s="84"/>
-    </row>
-    <row r="82" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J81" s="84"/>
+    </row>
+    <row r="82" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="29" t="s">
         <v>198</v>
       </c>
@@ -6856,8 +6946,9 @@
       <c r="G82" s="20"/>
       <c r="H82" s="20"/>
       <c r="I82" s="20"/>
-    </row>
-    <row r="83" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J82" s="20"/>
+    </row>
+    <row r="83" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
         <v>199</v>
       </c>
@@ -6869,8 +6960,9 @@
       <c r="G83" s="84"/>
       <c r="H83" s="84"/>
       <c r="I83" s="84"/>
-    </row>
-    <row r="84" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J83" s="84"/>
+    </row>
+    <row r="84" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="29" t="s">
         <v>200</v>
       </c>
@@ -6882,8 +6974,9 @@
       <c r="G84" s="20"/>
       <c r="H84" s="20"/>
       <c r="I84" s="20"/>
-    </row>
-    <row r="85" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J84" s="20"/>
+    </row>
+    <row r="85" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
         <v>201</v>
       </c>
@@ -6895,8 +6988,9 @@
       <c r="G85" s="84"/>
       <c r="H85" s="84"/>
       <c r="I85" s="84"/>
-    </row>
-    <row r="86" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J85" s="84"/>
+    </row>
+    <row r="86" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="29" t="s">
         <v>202</v>
       </c>
@@ -6908,8 +7002,9 @@
       <c r="G86" s="20"/>
       <c r="H86" s="20"/>
       <c r="I86" s="20"/>
-    </row>
-    <row r="87" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J86" s="20"/>
+    </row>
+    <row r="87" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" s="12" t="s">
         <v>203</v>
       </c>
@@ -6921,8 +7016,9 @@
       <c r="G87" s="84"/>
       <c r="H87" s="84"/>
       <c r="I87" s="84"/>
-    </row>
-    <row r="88" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J87" s="84"/>
+    </row>
+    <row r="88" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A88" s="29" t="s">
         <v>55</v>
       </c>
@@ -6934,8 +7030,9 @@
       <c r="G88" s="20"/>
       <c r="H88" s="20"/>
       <c r="I88" s="20"/>
-    </row>
-    <row r="89" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J88" s="20"/>
+    </row>
+    <row r="89" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A89" s="12" t="s">
         <v>204</v>
       </c>
@@ -6947,8 +7044,9 @@
       <c r="G89" s="84"/>
       <c r="H89" s="84"/>
       <c r="I89" s="84"/>
-    </row>
-    <row r="90" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J89" s="84"/>
+    </row>
+    <row r="90" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A90" s="29" t="s">
         <v>205</v>
       </c>
@@ -6960,8 +7058,9 @@
       <c r="G90" s="20"/>
       <c r="H90" s="20"/>
       <c r="I90" s="20"/>
-    </row>
-    <row r="91" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J90" s="20"/>
+    </row>
+    <row r="91" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A91" s="12" t="s">
         <v>206</v>
       </c>
@@ -6973,8 +7072,9 @@
       <c r="G91" s="84"/>
       <c r="H91" s="84"/>
       <c r="I91" s="84"/>
-    </row>
-    <row r="92" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J91" s="84"/>
+    </row>
+    <row r="92" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A92" s="29" t="s">
         <v>207</v>
       </c>
@@ -6986,8 +7086,9 @@
       <c r="G92" s="20"/>
       <c r="H92" s="20"/>
       <c r="I92" s="20"/>
-    </row>
-    <row r="93" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J92" s="20"/>
+    </row>
+    <row r="93" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A93" s="12" t="s">
         <v>208</v>
       </c>
@@ -6999,8 +7100,9 @@
       <c r="G93" s="84"/>
       <c r="H93" s="84"/>
       <c r="I93" s="84"/>
-    </row>
-    <row r="94" ht="16" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J93" s="84"/>
+    </row>
+    <row r="94" ht="16" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A94" s="29" t="s">
         <v>67</v>
       </c>
@@ -7012,6 +7114,7 @@
       <c r="G94" s="20"/>
       <c r="H94" s="20"/>
       <c r="I94" s="20"/>
+      <c r="J94" s="20"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1"/>
@@ -23266,6 +23369,14 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="B10">
+      <formula1>=_Lists!$J$1:$J$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="B7:B10">
+      <formula1>=_Lists!$J$1:$J$3</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.65" bottom="0.65" header="0.28" footer="0.28"/>
   <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="20"/>

</xml_diff>